<commit_message>
Atualização automática: 2026-09-03 10:29
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="198">
   <si>
     <t>CodCliente</t>
   </si>
@@ -516,6 +516,9 @@
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/09/2026 
 Tarefa a ser realizada em: 02/09/2026 - Data Comentário: 02/09/2026 16:24</t>
+  </si>
+  <si>
+    <t>Segundo informado pela coordenadora Nayara Oliveira, tarefa será conclupida hoje, 03/09 - Data Comentário: 03/09/2026 10:15</t>
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1879]. - Data Comentário: 01/09/2026 00:58</t>
@@ -1128,10 +1131,10 @@
         <v>112</v>
       </c>
       <c r="AH2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1205,10 +1208,10 @@
         <v>113</v>
       </c>
       <c r="AH3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1279,10 +1282,10 @@
         <v>113</v>
       </c>
       <c r="AH4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1353,10 +1356,10 @@
         <v>112</v>
       </c>
       <c r="AH5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1427,10 +1430,10 @@
         <v>112</v>
       </c>
       <c r="AH6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1501,10 +1504,10 @@
         <v>114</v>
       </c>
       <c r="AH7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1575,10 +1578,10 @@
         <v>113</v>
       </c>
       <c r="AH8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1649,10 +1652,10 @@
         <v>115</v>
       </c>
       <c r="AH9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1723,10 +1726,10 @@
         <v>115</v>
       </c>
       <c r="AH10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1797,10 +1800,10 @@
         <v>116</v>
       </c>
       <c r="AH11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -1868,13 +1871,13 @@
         <v>0</v>
       </c>
       <c r="AC12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AH12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -1942,13 +1945,13 @@
         <v>0</v>
       </c>
       <c r="AC13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AH13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2016,10 +2019,10 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2081,10 +2084,10 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2152,10 +2155,10 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2226,10 +2229,10 @@
         <v>119</v>
       </c>
       <c r="AH17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2300,10 +2303,10 @@
         <v>116</v>
       </c>
       <c r="AH18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2374,10 +2377,10 @@
         <v>116</v>
       </c>
       <c r="AH19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2448,10 +2451,10 @@
         <v>116</v>
       </c>
       <c r="AH20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2522,10 +2525,10 @@
         <v>117</v>
       </c>
       <c r="AH21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI21" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2596,10 +2599,10 @@
         <v>116</v>
       </c>
       <c r="AH22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2670,10 +2673,10 @@
         <v>116</v>
       </c>
       <c r="AH23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI23" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2744,10 +2747,10 @@
         <v>116</v>
       </c>
       <c r="AH24" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI24" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -2824,10 +2827,10 @@
         <v>120</v>
       </c>
       <c r="AH25" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI25" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -2901,10 +2904,10 @@
         <v>121</v>
       </c>
       <c r="AH26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AI26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -2978,10 +2981,10 @@
         <v>136</v>
       </c>
       <c r="AH27" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AI27" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3058,10 +3061,10 @@
         <v>122</v>
       </c>
       <c r="AH28" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AI28" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3138,10 +3141,10 @@
         <v>123</v>
       </c>
       <c r="AH29" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AI29" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3212,10 +3215,10 @@
         <v>122</v>
       </c>
       <c r="AH30" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI30" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3292,10 +3295,10 @@
         <v>120</v>
       </c>
       <c r="AH31" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI31" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3372,10 +3375,10 @@
         <v>124</v>
       </c>
       <c r="AH32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI32" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3452,10 +3455,10 @@
         <v>122</v>
       </c>
       <c r="AH33" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI33" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3532,10 +3535,10 @@
         <v>123</v>
       </c>
       <c r="AH34" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI34" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3606,10 +3609,10 @@
         <v>122</v>
       </c>
       <c r="AH35" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI35" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3680,10 +3683,10 @@
         <v>123</v>
       </c>
       <c r="AH36" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI36" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3754,10 +3757,10 @@
         <v>126</v>
       </c>
       <c r="AH37" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI37" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -3828,10 +3831,10 @@
         <v>126</v>
       </c>
       <c r="AH38" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI38" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -3902,10 +3905,10 @@
         <v>127</v>
       </c>
       <c r="AH39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI39" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -3976,10 +3979,10 @@
         <v>126</v>
       </c>
       <c r="AH40" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI40" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4050,10 +4053,10 @@
         <v>126</v>
       </c>
       <c r="AH41" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI41" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4130,10 +4133,10 @@
         <v>126</v>
       </c>
       <c r="AH42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI42" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4204,10 +4207,10 @@
         <v>127</v>
       </c>
       <c r="AH43" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI43" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4278,10 +4281,10 @@
         <v>126</v>
       </c>
       <c r="AH44" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI44" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4352,10 +4355,10 @@
         <v>126</v>
       </c>
       <c r="AH45" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI45" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4426,10 +4429,10 @@
         <v>126</v>
       </c>
       <c r="AH46" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI46" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4500,10 +4503,10 @@
         <v>126</v>
       </c>
       <c r="AH47" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI47" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4574,10 +4577,10 @@
         <v>127</v>
       </c>
       <c r="AH48" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI48" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4648,10 +4651,10 @@
         <v>126</v>
       </c>
       <c r="AH49" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI49" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4722,10 +4725,10 @@
         <v>126</v>
       </c>
       <c r="AH50" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI50" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -4796,10 +4799,10 @@
         <v>126</v>
       </c>
       <c r="AH51" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI51" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -4870,10 +4873,10 @@
         <v>126</v>
       </c>
       <c r="AH52" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI52" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -4944,10 +4947,10 @@
         <v>127</v>
       </c>
       <c r="AH53" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI53" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5018,10 +5021,10 @@
         <v>126</v>
       </c>
       <c r="AH54" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI54" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5092,10 +5095,10 @@
         <v>126</v>
       </c>
       <c r="AH55" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI55" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5166,10 +5169,10 @@
         <v>127</v>
       </c>
       <c r="AH56" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI56" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5206,6 +5209,9 @@
       <c r="N57" s="1">
         <v>46268</v>
       </c>
+      <c r="O57" t="s">
+        <v>109</v>
+      </c>
       <c r="P57">
         <v>8</v>
       </c>
@@ -5233,6 +5239,9 @@
       <c r="X57" t="s">
         <v>146</v>
       </c>
+      <c r="Y57" t="s">
+        <v>165</v>
+      </c>
       <c r="AB57">
         <v>0</v>
       </c>
@@ -5240,10 +5249,10 @@
         <v>126</v>
       </c>
       <c r="AH57" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI57" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5314,10 +5323,10 @@
         <v>126</v>
       </c>
       <c r="AH58" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI58" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5388,10 +5397,10 @@
         <v>126</v>
       </c>
       <c r="AH59" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI59" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5462,10 +5471,10 @@
         <v>126</v>
       </c>
       <c r="AH60" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI60" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5536,10 +5545,10 @@
         <v>126</v>
       </c>
       <c r="AH61" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI61" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5610,10 +5619,10 @@
         <v>126</v>
       </c>
       <c r="AH62" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI62" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -5684,10 +5693,10 @@
         <v>127</v>
       </c>
       <c r="AH63" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI63" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -5758,10 +5767,10 @@
         <v>126</v>
       </c>
       <c r="AH64" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI64" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -5832,10 +5841,10 @@
         <v>126</v>
       </c>
       <c r="AH65" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI65" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -5906,10 +5915,10 @@
         <v>126</v>
       </c>
       <c r="AH66" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI66" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -5980,10 +5989,10 @@
         <v>127</v>
       </c>
       <c r="AH67" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI67" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6054,10 +6063,10 @@
         <v>128</v>
       </c>
       <c r="AH68" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI68" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6128,10 +6137,10 @@
         <v>127</v>
       </c>
       <c r="AH69" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI69" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6202,10 +6211,10 @@
         <v>125</v>
       </c>
       <c r="AH70" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI70" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6276,10 +6285,10 @@
         <v>128</v>
       </c>
       <c r="AH71" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI71" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6350,10 +6359,10 @@
         <v>127</v>
       </c>
       <c r="AH72" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI72" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6424,10 +6433,10 @@
         <v>126</v>
       </c>
       <c r="AH73" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI73" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6498,10 +6507,10 @@
         <v>126</v>
       </c>
       <c r="AH74" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI74" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6572,10 +6581,10 @@
         <v>126</v>
       </c>
       <c r="AH75" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI75" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6646,10 +6655,10 @@
         <v>126</v>
       </c>
       <c r="AH76" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI76" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -6720,10 +6729,10 @@
         <v>127</v>
       </c>
       <c r="AH77" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI77" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -6794,10 +6803,10 @@
         <v>126</v>
       </c>
       <c r="AH78" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI78" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -6868,10 +6877,10 @@
         <v>126</v>
       </c>
       <c r="AH79" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI79" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -6942,10 +6951,10 @@
         <v>126</v>
       </c>
       <c r="AH80" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI80" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7016,10 +7025,10 @@
         <v>126</v>
       </c>
       <c r="AH81" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI81" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7090,10 +7099,10 @@
         <v>127</v>
       </c>
       <c r="AH82" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI82" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7164,10 +7173,10 @@
         <v>129</v>
       </c>
       <c r="AH83" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI83" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7238,10 +7247,10 @@
         <v>129</v>
       </c>
       <c r="AH84" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI84" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7312,10 +7321,10 @@
         <v>129</v>
       </c>
       <c r="AH85" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI85" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7386,10 +7395,10 @@
         <v>129</v>
       </c>
       <c r="AH86" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI86" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7460,10 +7469,10 @@
         <v>129</v>
       </c>
       <c r="AH87" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI87" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7534,10 +7543,10 @@
         <v>129</v>
       </c>
       <c r="AH88" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI88" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7608,10 +7617,10 @@
         <v>129</v>
       </c>
       <c r="AH89" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI89" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -7682,10 +7691,10 @@
         <v>129</v>
       </c>
       <c r="AH90" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI90" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -7756,10 +7765,10 @@
         <v>129</v>
       </c>
       <c r="AH91" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI91" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -7830,10 +7839,10 @@
         <v>129</v>
       </c>
       <c r="AH92" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI92" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -7904,10 +7913,10 @@
         <v>129</v>
       </c>
       <c r="AH93" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI93" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -7978,10 +7987,10 @@
         <v>129</v>
       </c>
       <c r="AH94" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI94" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8052,10 +8061,10 @@
         <v>129</v>
       </c>
       <c r="AH95" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI95" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8117,7 +8126,7 @@
         <v>142</v>
       </c>
       <c r="Y96" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB96">
         <v>0</v>
@@ -8126,10 +8135,10 @@
         <v>130</v>
       </c>
       <c r="AH96" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI96" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8191,7 +8200,7 @@
         <v>147</v>
       </c>
       <c r="Y97" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB97">
         <v>0</v>
@@ -8200,10 +8209,10 @@
         <v>130</v>
       </c>
       <c r="AH97" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI97" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8265,7 +8274,7 @@
         <v>145</v>
       </c>
       <c r="Y98" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB98">
         <v>0</v>
@@ -8274,10 +8283,10 @@
         <v>130</v>
       </c>
       <c r="AH98" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI98" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8339,7 +8348,7 @@
         <v>148</v>
       </c>
       <c r="Y99" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AB99">
         <v>0</v>
@@ -8348,10 +8357,10 @@
         <v>130</v>
       </c>
       <c r="AH99" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI99" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8413,7 +8422,7 @@
         <v>151</v>
       </c>
       <c r="Y100" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AB100">
         <v>0</v>
@@ -8422,10 +8431,10 @@
         <v>130</v>
       </c>
       <c r="AH100" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI100" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8487,7 +8496,7 @@
         <v>152</v>
       </c>
       <c r="Y101" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AB101">
         <v>0</v>
@@ -8496,10 +8505,10 @@
         <v>130</v>
       </c>
       <c r="AH101" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI101" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8561,7 +8570,7 @@
         <v>152</v>
       </c>
       <c r="Y102" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AB102">
         <v>0</v>
@@ -8570,10 +8579,10 @@
         <v>130</v>
       </c>
       <c r="AH102" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI102" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8635,7 +8644,7 @@
         <v>143</v>
       </c>
       <c r="Y103" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AB103">
         <v>0</v>
@@ -8644,10 +8653,10 @@
         <v>130</v>
       </c>
       <c r="AH103" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI103" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -8709,7 +8718,7 @@
         <v>144</v>
       </c>
       <c r="Y104" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AB104">
         <v>0</v>
@@ -8718,10 +8727,10 @@
         <v>130</v>
       </c>
       <c r="AH104" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI104" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -8783,7 +8792,7 @@
         <v>152</v>
       </c>
       <c r="Y105" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AB105">
         <v>0</v>
@@ -8792,10 +8801,10 @@
         <v>130</v>
       </c>
       <c r="AH105" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI105" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -8857,7 +8866,7 @@
         <v>147</v>
       </c>
       <c r="Y106" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AB106">
         <v>0</v>
@@ -8866,10 +8875,10 @@
         <v>130</v>
       </c>
       <c r="AH106" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI106" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -8931,7 +8940,7 @@
         <v>145</v>
       </c>
       <c r="Y107" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AB107">
         <v>0</v>
@@ -8940,10 +8949,10 @@
         <v>130</v>
       </c>
       <c r="AH107" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI107" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9005,7 +9014,7 @@
         <v>143</v>
       </c>
       <c r="Y108" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AB108">
         <v>0</v>
@@ -9014,10 +9023,10 @@
         <v>130</v>
       </c>
       <c r="AH108" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI108" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9079,7 +9088,7 @@
         <v>148</v>
       </c>
       <c r="Y109" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AB109">
         <v>0</v>
@@ -9088,10 +9097,10 @@
         <v>130</v>
       </c>
       <c r="AH109" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI109" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9153,7 +9162,7 @@
         <v>151</v>
       </c>
       <c r="Y110" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AB110">
         <v>0</v>
@@ -9162,10 +9171,10 @@
         <v>130</v>
       </c>
       <c r="AH110" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI110" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9227,7 +9236,7 @@
         <v>142</v>
       </c>
       <c r="Y111" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AB111">
         <v>0</v>
@@ -9236,10 +9245,10 @@
         <v>130</v>
       </c>
       <c r="AH111" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI111" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9301,7 +9310,7 @@
         <v>152</v>
       </c>
       <c r="Y112" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AB112">
         <v>0</v>
@@ -9310,10 +9319,10 @@
         <v>130</v>
       </c>
       <c r="AH112" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI112" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9375,7 +9384,7 @@
         <v>143</v>
       </c>
       <c r="Y113" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AB113">
         <v>0</v>
@@ -9384,10 +9393,10 @@
         <v>130</v>
       </c>
       <c r="AH113" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI113" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9449,7 +9458,7 @@
         <v>148</v>
       </c>
       <c r="Y114" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB114">
         <v>0</v>
@@ -9458,10 +9467,10 @@
         <v>130</v>
       </c>
       <c r="AH114" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI114" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9523,7 +9532,7 @@
         <v>142</v>
       </c>
       <c r="Y115" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AB115">
         <v>0</v>
@@ -9532,10 +9541,10 @@
         <v>130</v>
       </c>
       <c r="AH115" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI115" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9597,7 +9606,7 @@
         <v>147</v>
       </c>
       <c r="Y116" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AB116">
         <v>0</v>
@@ -9606,10 +9615,10 @@
         <v>130</v>
       </c>
       <c r="AH116" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI116" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -9671,7 +9680,7 @@
         <v>143</v>
       </c>
       <c r="Y117" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AB117">
         <v>0</v>
@@ -9680,10 +9689,10 @@
         <v>130</v>
       </c>
       <c r="AH117" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI117" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -9745,7 +9754,7 @@
         <v>151</v>
       </c>
       <c r="Y118" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AB118">
         <v>0</v>
@@ -9754,10 +9763,10 @@
         <v>55</v>
       </c>
       <c r="AH118" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI118" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -9819,7 +9828,7 @@
         <v>151</v>
       </c>
       <c r="Y119" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AB119">
         <v>0</v>
@@ -9828,10 +9837,10 @@
         <v>55</v>
       </c>
       <c r="AH119" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI119" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -9893,7 +9902,7 @@
         <v>148</v>
       </c>
       <c r="Y120" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AB120">
         <v>0</v>
@@ -9902,10 +9911,10 @@
         <v>55</v>
       </c>
       <c r="AH120" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI120" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -9967,7 +9976,7 @@
         <v>148</v>
       </c>
       <c r="Y121" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AB121">
         <v>0</v>
@@ -9976,10 +9985,10 @@
         <v>55</v>
       </c>
       <c r="AH121" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI121" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10041,7 +10050,7 @@
         <v>149</v>
       </c>
       <c r="Y122" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="AB122">
         <v>0</v>
@@ -10050,10 +10059,10 @@
         <v>55</v>
       </c>
       <c r="AH122" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI122" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10115,7 +10124,7 @@
         <v>149</v>
       </c>
       <c r="Y123" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AB123">
         <v>0</v>
@@ -10124,10 +10133,10 @@
         <v>55</v>
       </c>
       <c r="AH123" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI123" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10195,10 +10204,10 @@
         <v>55</v>
       </c>
       <c r="AH124" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI124" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10266,10 +10275,10 @@
         <v>55</v>
       </c>
       <c r="AH125" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI125" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10337,10 +10346,10 @@
         <v>55</v>
       </c>
       <c r="AH126" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AI126" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-04 11:11
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -4456,7 +4456,7 @@
         <v>129</v>
       </c>
       <c r="AH45" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AI45" t="s">
         <v>219</v>
@@ -4536,7 +4536,7 @@
         <v>128</v>
       </c>
       <c r="AH46" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AI46" t="s">
         <v>219</v>
@@ -4616,7 +4616,7 @@
         <v>132</v>
       </c>
       <c r="AH47" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AI47" t="s">
         <v>219</v>
@@ -4696,7 +4696,7 @@
         <v>133</v>
       </c>
       <c r="AH48" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AI48" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-09 12:19
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3218" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3395" uniqueCount="256">
   <si>
     <t>CodCliente</t>
   </si>
@@ -760,7 +760,17 @@
 Reunião confirmada pelo cliente - Data Comentário: 04/09/2026 11:03</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/09/2026 - Data Comentário: 04/09/2026 16:13</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 10/09/2026 
+Em processamento. - Data Comentário: 04/09/2026 08:41</t>
+  </si>
+  <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 09/09/2026 08:35</t>
+  </si>
+  <si>
+    <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 09/09/2026 10:17:37. - Data Comentário: 09/09/2026 10:12</t>
   </si>
   <si>
     <t>Karen Ribeiro</t>
@@ -1123,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI225"/>
+  <dimension ref="A1:AI238"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1304,10 +1314,10 @@
         <v>132</v>
       </c>
       <c r="AH2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1381,10 +1391,10 @@
         <v>133</v>
       </c>
       <c r="AH3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI3" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1458,10 +1468,10 @@
         <v>132</v>
       </c>
       <c r="AH4" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1532,10 +1542,10 @@
         <v>132</v>
       </c>
       <c r="AH5" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1606,10 +1616,10 @@
         <v>133</v>
       </c>
       <c r="AH6" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI6" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1680,10 +1690,10 @@
         <v>133</v>
       </c>
       <c r="AH7" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI7" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1754,10 +1764,10 @@
         <v>134</v>
       </c>
       <c r="AH8" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI8" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1828,10 +1838,10 @@
         <v>132</v>
       </c>
       <c r="AH9" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1902,10 +1912,10 @@
         <v>135</v>
       </c>
       <c r="AH10" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI10" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1976,10 +1986,10 @@
         <v>135</v>
       </c>
       <c r="AH11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2050,10 +2060,10 @@
         <v>136</v>
       </c>
       <c r="AH12" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI12" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2121,13 +2131,13 @@
         <v>0</v>
       </c>
       <c r="AC13" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="AH13" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI13" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2195,13 +2205,13 @@
         <v>0</v>
       </c>
       <c r="AC14" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="AH14" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI14" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2269,10 +2279,10 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI15" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2334,10 +2344,10 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI16" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2405,10 +2415,10 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI17" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2482,10 +2492,10 @@
         <v>138</v>
       </c>
       <c r="AH18" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI18" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2559,10 +2569,10 @@
         <v>137</v>
       </c>
       <c r="AH19" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI19" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2636,10 +2646,10 @@
         <v>138</v>
       </c>
       <c r="AH20" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI20" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2713,10 +2723,10 @@
         <v>136</v>
       </c>
       <c r="AH21" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI21" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2787,10 +2797,10 @@
         <v>139</v>
       </c>
       <c r="AH22" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2861,10 +2871,10 @@
         <v>136</v>
       </c>
       <c r="AH23" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI23" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2935,10 +2945,10 @@
         <v>136</v>
       </c>
       <c r="AH24" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI24" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3009,10 +3019,10 @@
         <v>136</v>
       </c>
       <c r="AH25" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI25" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3083,10 +3093,10 @@
         <v>137</v>
       </c>
       <c r="AH26" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI26" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3157,10 +3167,10 @@
         <v>136</v>
       </c>
       <c r="AH27" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI27" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3231,10 +3241,10 @@
         <v>136</v>
       </c>
       <c r="AH28" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI28" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3305,10 +3315,10 @@
         <v>136</v>
       </c>
       <c r="AH29" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI29" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3379,10 +3389,10 @@
         <v>140</v>
       </c>
       <c r="AH30" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI30" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3459,10 +3469,10 @@
         <v>141</v>
       </c>
       <c r="AH31" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI31" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3533,10 +3543,10 @@
         <v>142</v>
       </c>
       <c r="AH32" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI32" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3613,10 +3623,10 @@
         <v>143</v>
       </c>
       <c r="AH33" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI33" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3690,10 +3700,10 @@
         <v>144</v>
       </c>
       <c r="AH34" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI34" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3767,13 +3777,13 @@
         <v>0</v>
       </c>
       <c r="AC35" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AH35" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI35" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3850,10 +3860,10 @@
         <v>146</v>
       </c>
       <c r="AH36" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI36" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3930,10 +3940,10 @@
         <v>140</v>
       </c>
       <c r="AH37" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI37" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4007,10 +4017,10 @@
         <v>162</v>
       </c>
       <c r="AH38" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI38" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4087,10 +4097,10 @@
         <v>141</v>
       </c>
       <c r="AH39" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI39" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4167,10 +4177,10 @@
         <v>141</v>
       </c>
       <c r="AH40" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI40" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4247,10 +4257,10 @@
         <v>141</v>
       </c>
       <c r="AH41" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI41" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4327,10 +4337,10 @@
         <v>140</v>
       </c>
       <c r="AH42" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI42" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4407,10 +4417,10 @@
         <v>147</v>
       </c>
       <c r="AH43" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI43" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4487,10 +4497,10 @@
         <v>142</v>
       </c>
       <c r="AH44" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI44" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4567,10 +4577,10 @@
         <v>143</v>
       </c>
       <c r="AH45" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI45" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4638,10 +4648,10 @@
         <v>144</v>
       </c>
       <c r="AH46" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI46" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4712,10 +4722,10 @@
         <v>141</v>
       </c>
       <c r="AH47" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI47" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4786,10 +4796,10 @@
         <v>141</v>
       </c>
       <c r="AH48" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI48" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4860,10 +4870,10 @@
         <v>141</v>
       </c>
       <c r="AH49" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI49" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4934,10 +4944,10 @@
         <v>140</v>
       </c>
       <c r="AH50" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI50" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5008,10 +5018,10 @@
         <v>147</v>
       </c>
       <c r="AH51" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI51" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5088,10 +5098,10 @@
         <v>142</v>
       </c>
       <c r="AH52" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI52" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5162,10 +5172,10 @@
         <v>143</v>
       </c>
       <c r="AH53" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI53" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5242,10 +5252,10 @@
         <v>141</v>
       </c>
       <c r="AH54" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI54" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5322,10 +5332,10 @@
         <v>141</v>
       </c>
       <c r="AH55" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI55" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5402,10 +5412,10 @@
         <v>141</v>
       </c>
       <c r="AH56" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI56" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5482,10 +5492,10 @@
         <v>140</v>
       </c>
       <c r="AH57" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI57" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5559,10 +5569,10 @@
         <v>144</v>
       </c>
       <c r="AH58" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI58" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5636,13 +5646,13 @@
         <v>0</v>
       </c>
       <c r="AC59" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AH59" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI59" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5719,10 +5729,10 @@
         <v>141</v>
       </c>
       <c r="AH60" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI60" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5799,10 +5809,10 @@
         <v>141</v>
       </c>
       <c r="AH61" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI61" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5879,10 +5889,10 @@
         <v>141</v>
       </c>
       <c r="AH62" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI62" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -5959,10 +5969,10 @@
         <v>140</v>
       </c>
       <c r="AH63" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI63" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6039,10 +6049,10 @@
         <v>147</v>
       </c>
       <c r="AH64" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI64" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6119,10 +6129,10 @@
         <v>142</v>
       </c>
       <c r="AH65" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI65" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6199,10 +6209,10 @@
         <v>143</v>
       </c>
       <c r="AH66" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI66" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6279,10 +6289,10 @@
         <v>141</v>
       </c>
       <c r="AH67" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI67" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6350,10 +6360,10 @@
         <v>144</v>
       </c>
       <c r="AH68" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI68" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6421,13 +6431,13 @@
         <v>0</v>
       </c>
       <c r="AC69" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AH69" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI69" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6498,10 +6508,10 @@
         <v>141</v>
       </c>
       <c r="AH70" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI70" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6572,10 +6582,10 @@
         <v>141</v>
       </c>
       <c r="AH71" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI71" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6646,10 +6656,10 @@
         <v>141</v>
       </c>
       <c r="AH72" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI72" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6720,10 +6730,10 @@
         <v>140</v>
       </c>
       <c r="AH73" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI73" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6794,10 +6804,10 @@
         <v>147</v>
       </c>
       <c r="AH74" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI74" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6868,10 +6878,10 @@
         <v>142</v>
       </c>
       <c r="AH75" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI75" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6942,10 +6952,10 @@
         <v>143</v>
       </c>
       <c r="AH76" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI76" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7016,10 +7026,10 @@
         <v>143</v>
       </c>
       <c r="AH77" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI77" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7090,10 +7100,10 @@
         <v>143</v>
       </c>
       <c r="AH78" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI78" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7164,10 +7174,10 @@
         <v>143</v>
       </c>
       <c r="AH79" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI79" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7238,10 +7248,10 @@
         <v>149</v>
       </c>
       <c r="AH80" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI80" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7312,10 +7322,10 @@
         <v>149</v>
       </c>
       <c r="AH81" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI81" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7386,10 +7396,10 @@
         <v>150</v>
       </c>
       <c r="AH82" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI82" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7460,10 +7470,10 @@
         <v>149</v>
       </c>
       <c r="AH83" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI83" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7534,10 +7544,10 @@
         <v>149</v>
       </c>
       <c r="AH84" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI84" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7611,10 +7621,10 @@
         <v>149</v>
       </c>
       <c r="AH85" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI85" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7685,10 +7695,10 @@
         <v>150</v>
       </c>
       <c r="AH86" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI86" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7759,10 +7769,10 @@
         <v>149</v>
       </c>
       <c r="AH87" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI87" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7833,10 +7843,10 @@
         <v>149</v>
       </c>
       <c r="AH88" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI88" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7907,10 +7917,10 @@
         <v>149</v>
       </c>
       <c r="AH89" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI89" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -7978,10 +7988,10 @@
         <v>149</v>
       </c>
       <c r="AH90" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI90" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8052,10 +8062,10 @@
         <v>150</v>
       </c>
       <c r="AH91" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI91" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8126,10 +8136,10 @@
         <v>149</v>
       </c>
       <c r="AH92" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI92" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8200,10 +8210,10 @@
         <v>149</v>
       </c>
       <c r="AH93" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI93" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8274,10 +8284,10 @@
         <v>149</v>
       </c>
       <c r="AH94" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI94" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8345,10 +8355,10 @@
         <v>149</v>
       </c>
       <c r="AH95" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI95" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8419,10 +8429,10 @@
         <v>150</v>
       </c>
       <c r="AH96" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI96" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8493,10 +8503,10 @@
         <v>149</v>
       </c>
       <c r="AH97" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI97" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8567,10 +8577,10 @@
         <v>149</v>
       </c>
       <c r="AH98" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI98" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8641,10 +8651,10 @@
         <v>150</v>
       </c>
       <c r="AH99" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI99" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8721,10 +8731,10 @@
         <v>149</v>
       </c>
       <c r="AH100" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI100" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8792,10 +8802,10 @@
         <v>149</v>
       </c>
       <c r="AH101" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI101" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8866,10 +8876,10 @@
         <v>149</v>
       </c>
       <c r="AH102" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI102" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8940,10 +8950,10 @@
         <v>149</v>
       </c>
       <c r="AH103" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI103" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9014,10 +9024,10 @@
         <v>149</v>
       </c>
       <c r="AH104" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI104" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9085,10 +9095,10 @@
         <v>149</v>
       </c>
       <c r="AH105" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI105" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9159,10 +9169,10 @@
         <v>150</v>
       </c>
       <c r="AH106" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI106" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9233,10 +9243,10 @@
         <v>149</v>
       </c>
       <c r="AH107" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI107" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9307,10 +9317,10 @@
         <v>149</v>
       </c>
       <c r="AH108" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI108" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9378,10 +9388,10 @@
         <v>149</v>
       </c>
       <c r="AH109" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI109" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9452,10 +9462,10 @@
         <v>150</v>
       </c>
       <c r="AH110" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI110" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9523,10 +9533,10 @@
         <v>151</v>
       </c>
       <c r="AH111" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI111" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9597,10 +9607,10 @@
         <v>150</v>
       </c>
       <c r="AH112" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI112" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9671,10 +9681,10 @@
         <v>148</v>
       </c>
       <c r="AH113" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI113" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9742,10 +9752,10 @@
         <v>151</v>
       </c>
       <c r="AH114" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI114" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9816,10 +9826,10 @@
         <v>150</v>
       </c>
       <c r="AH115" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI115" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9890,10 +9900,10 @@
         <v>149</v>
       </c>
       <c r="AH116" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI116" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -9964,10 +9974,10 @@
         <v>149</v>
       </c>
       <c r="AH117" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI117" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10038,10 +10048,10 @@
         <v>149</v>
       </c>
       <c r="AH118" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI118" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10109,10 +10119,10 @@
         <v>149</v>
       </c>
       <c r="AH119" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI119" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10183,10 +10193,10 @@
         <v>150</v>
       </c>
       <c r="AH120" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI120" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10257,10 +10267,10 @@
         <v>149</v>
       </c>
       <c r="AH121" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI121" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10331,10 +10341,10 @@
         <v>149</v>
       </c>
       <c r="AH122" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI122" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10405,10 +10415,10 @@
         <v>149</v>
       </c>
       <c r="AH123" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI123" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10476,10 +10486,10 @@
         <v>149</v>
       </c>
       <c r="AH124" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI124" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10550,10 +10560,10 @@
         <v>150</v>
       </c>
       <c r="AH125" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI125" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10630,10 +10640,10 @@
         <v>150</v>
       </c>
       <c r="AH126" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI126" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10710,10 +10720,10 @@
         <v>150</v>
       </c>
       <c r="AH127" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI127" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10784,10 +10794,10 @@
         <v>153</v>
       </c>
       <c r="AH128" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI128" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10858,10 +10868,10 @@
         <v>153</v>
       </c>
       <c r="AH129" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI129" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -10938,10 +10948,10 @@
         <v>153</v>
       </c>
       <c r="AH130" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI130" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11012,10 +11022,10 @@
         <v>153</v>
       </c>
       <c r="AH131" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI131" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11086,10 +11096,10 @@
         <v>153</v>
       </c>
       <c r="AH132" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI132" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11160,10 +11170,10 @@
         <v>153</v>
       </c>
       <c r="AH133" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI133" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11234,10 +11244,10 @@
         <v>153</v>
       </c>
       <c r="AH134" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI134" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11314,10 +11324,10 @@
         <v>153</v>
       </c>
       <c r="AH135" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI135" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11388,10 +11398,10 @@
         <v>153</v>
       </c>
       <c r="AH136" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI136" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11462,10 +11472,10 @@
         <v>153</v>
       </c>
       <c r="AH137" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI137" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11536,10 +11546,10 @@
         <v>153</v>
       </c>
       <c r="AH138" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI138" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11616,10 +11626,10 @@
         <v>153</v>
       </c>
       <c r="AH139" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI139" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11690,10 +11700,10 @@
         <v>153</v>
       </c>
       <c r="AH140" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI140" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11764,10 +11774,10 @@
         <v>153</v>
       </c>
       <c r="AH141" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI141" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11838,10 +11848,10 @@
         <v>153</v>
       </c>
       <c r="AH142" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI142" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11912,10 +11922,10 @@
         <v>153</v>
       </c>
       <c r="AH143" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI143" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -11986,10 +11996,10 @@
         <v>153</v>
       </c>
       <c r="AH144" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI144" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12060,10 +12070,10 @@
         <v>153</v>
       </c>
       <c r="AH145" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI145" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12134,10 +12144,10 @@
         <v>153</v>
       </c>
       <c r="AH146" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI146" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12208,10 +12218,10 @@
         <v>153</v>
       </c>
       <c r="AH147" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI147" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12282,10 +12292,10 @@
         <v>153</v>
       </c>
       <c r="AH148" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI148" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12356,10 +12366,10 @@
         <v>153</v>
       </c>
       <c r="AH149" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI149" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12436,10 +12446,10 @@
         <v>153</v>
       </c>
       <c r="AH150" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI150" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12510,10 +12520,10 @@
         <v>153</v>
       </c>
       <c r="AH151" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI151" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12584,10 +12594,10 @@
         <v>153</v>
       </c>
       <c r="AH152" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI152" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12658,10 +12668,10 @@
         <v>153</v>
       </c>
       <c r="AH153" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI153" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12732,10 +12742,10 @@
         <v>154</v>
       </c>
       <c r="AH154" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI154" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12806,10 +12816,10 @@
         <v>154</v>
       </c>
       <c r="AH155" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI155" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12880,10 +12890,10 @@
         <v>154</v>
       </c>
       <c r="AH156" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI156" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -12954,10 +12964,10 @@
         <v>154</v>
       </c>
       <c r="AH157" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI157" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13028,10 +13038,10 @@
         <v>154</v>
       </c>
       <c r="AH158" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI158" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13102,10 +13112,10 @@
         <v>154</v>
       </c>
       <c r="AH159" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI159" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13176,10 +13186,10 @@
         <v>154</v>
       </c>
       <c r="AH160" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI160" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13250,10 +13260,10 @@
         <v>154</v>
       </c>
       <c r="AH161" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI161" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13324,10 +13334,10 @@
         <v>154</v>
       </c>
       <c r="AH162" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI162" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13398,10 +13408,10 @@
         <v>154</v>
       </c>
       <c r="AH163" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI163" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13472,10 +13482,10 @@
         <v>154</v>
       </c>
       <c r="AH164" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI164" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13546,10 +13556,10 @@
         <v>154</v>
       </c>
       <c r="AH165" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI165" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13620,10 +13630,10 @@
         <v>154</v>
       </c>
       <c r="AH166" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI166" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13694,10 +13704,10 @@
         <v>154</v>
       </c>
       <c r="AH167" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI167" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13768,10 +13778,10 @@
         <v>154</v>
       </c>
       <c r="AH168" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI168" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13842,10 +13852,10 @@
         <v>154</v>
       </c>
       <c r="AH169" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI169" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13916,10 +13926,10 @@
         <v>154</v>
       </c>
       <c r="AH170" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI170" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -13990,10 +14000,10 @@
         <v>154</v>
       </c>
       <c r="AH171" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI171" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14064,10 +14074,10 @@
         <v>154</v>
       </c>
       <c r="AH172" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI172" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14138,10 +14148,10 @@
         <v>154</v>
       </c>
       <c r="AH173" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AI173" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14215,10 +14225,10 @@
         <v>154</v>
       </c>
       <c r="AH174" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI174" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14292,10 +14302,10 @@
         <v>154</v>
       </c>
       <c r="AH175" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI175" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14369,10 +14379,10 @@
         <v>154</v>
       </c>
       <c r="AH176" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI176" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14446,10 +14456,10 @@
         <v>154</v>
       </c>
       <c r="AH177" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI177" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14523,10 +14533,10 @@
         <v>154</v>
       </c>
       <c r="AH178" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI178" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14600,10 +14610,10 @@
         <v>154</v>
       </c>
       <c r="AH179" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI179" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14677,10 +14687,10 @@
         <v>154</v>
       </c>
       <c r="AH180" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI180" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14754,10 +14764,10 @@
         <v>154</v>
       </c>
       <c r="AH181" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI181" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14831,10 +14841,10 @@
         <v>154</v>
       </c>
       <c r="AH182" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI182" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14908,10 +14918,10 @@
         <v>154</v>
       </c>
       <c r="AH183" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI183" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -14985,10 +14995,10 @@
         <v>154</v>
       </c>
       <c r="AH184" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI184" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15062,10 +15072,10 @@
         <v>154</v>
       </c>
       <c r="AH185" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI185" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15139,10 +15149,10 @@
         <v>154</v>
       </c>
       <c r="AH186" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI186" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15216,10 +15226,10 @@
         <v>154</v>
       </c>
       <c r="AH187" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI187" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15287,10 +15297,10 @@
         <v>154</v>
       </c>
       <c r="AH188" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI188" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15358,10 +15368,10 @@
         <v>154</v>
       </c>
       <c r="AH189" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI189" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15429,10 +15439,10 @@
         <v>154</v>
       </c>
       <c r="AH190" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI190" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15500,10 +15510,10 @@
         <v>154</v>
       </c>
       <c r="AH191" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI191" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15571,10 +15581,10 @@
         <v>154</v>
       </c>
       <c r="AH192" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI192" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15642,10 +15652,10 @@
         <v>154</v>
       </c>
       <c r="AH193" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI193" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15713,10 +15723,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI194" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15784,10 +15794,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI195" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15855,10 +15865,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI196" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15926,10 +15936,10 @@
         <v>54</v>
       </c>
       <c r="AH197" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI197" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -15997,10 +16007,10 @@
         <v>155</v>
       </c>
       <c r="AH198" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI198" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16068,10 +16078,10 @@
         <v>55</v>
       </c>
       <c r="AH199" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI199" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16139,10 +16149,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI200" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16210,10 +16220,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI201" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16281,10 +16291,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI202" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16352,10 +16362,10 @@
         <v>155</v>
       </c>
       <c r="AH203" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI203" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16423,10 +16433,10 @@
         <v>54</v>
       </c>
       <c r="AH204" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI204" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16494,10 +16504,10 @@
         <v>155</v>
       </c>
       <c r="AH205" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI205" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16565,10 +16575,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI206" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16636,10 +16646,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI207" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16707,10 +16717,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI208" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16778,10 +16788,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI209" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16849,10 +16859,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI210" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -16920,10 +16930,10 @@
         <v>54</v>
       </c>
       <c r="AH211" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI211" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -16991,10 +17001,10 @@
         <v>155</v>
       </c>
       <c r="AH212" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI212" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17062,10 +17072,10 @@
         <v>55</v>
       </c>
       <c r="AH213" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AI213" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17136,10 +17146,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI214" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17210,10 +17220,10 @@
         <v>54</v>
       </c>
       <c r="AH215" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI215" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17284,10 +17294,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI216" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17358,10 +17368,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI217" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17429,10 +17439,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI218" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17500,10 +17510,10 @@
         <v>54</v>
       </c>
       <c r="AH219" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI219" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17574,10 +17584,10 @@
         <v>54</v>
       </c>
       <c r="AH220" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI220" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17645,10 +17655,10 @@
         <v>54</v>
       </c>
       <c r="AH221" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI221" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17716,21 +17726,21 @@
         <v>0</v>
       </c>
       <c r="AC222" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="AH222" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI222" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="223" spans="1:35">
       <c r="A223">
-        <v>6949</v>
+        <v>6486</v>
       </c>
       <c r="B223" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C223" t="s">
         <v>50</v>
@@ -17742,7 +17752,7 @@
         <v>54</v>
       </c>
       <c r="F223" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G223">
         <v>9746</v>
@@ -17759,6 +17769,9 @@
       <c r="N223" s="1">
         <v>46275</v>
       </c>
+      <c r="O223" t="s">
+        <v>131</v>
+      </c>
       <c r="P223">
         <v>8</v>
       </c>
@@ -17766,72 +17779,78 @@
         <v>2026</v>
       </c>
       <c r="R223">
-        <v>18190457</v>
+        <v>16976300</v>
       </c>
       <c r="S223" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="T223" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="U223" t="s">
         <v>165</v>
       </c>
       <c r="V223" s="1">
-        <v>46274.34198912037</v>
+        <v>46274.47210818287</v>
       </c>
       <c r="W223">
         <v>-1</v>
       </c>
       <c r="X223" t="s">
-        <v>169</v>
+        <v>174</v>
+      </c>
+      <c r="Y223" t="s">
+        <v>243</v>
       </c>
       <c r="AB223">
         <v>0</v>
       </c>
       <c r="AC223" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="AH223" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI223" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="224" spans="1:35">
       <c r="A224">
-        <v>6627</v>
+        <v>6779</v>
       </c>
       <c r="B224" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C224" t="s">
         <v>50</v>
       </c>
       <c r="D224" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E224" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F224" t="s">
         <v>56</v>
       </c>
       <c r="G224">
-        <v>1866</v>
+        <v>9746</v>
       </c>
       <c r="H224">
         <v>0</v>
       </c>
       <c r="I224" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J224" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="N224" s="1">
-        <v>46274</v>
+        <v>46275</v>
+      </c>
+      <c r="O224" t="s">
+        <v>129</v>
       </c>
       <c r="P224">
         <v>8</v>
@@ -17840,48 +17859,48 @@
         <v>2026</v>
       </c>
       <c r="R224">
-        <v>17968368</v>
+        <v>18090250</v>
       </c>
       <c r="S224" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="T224" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="U224" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="V224" s="1">
-        <v>46274.36843923611</v>
+        <v>46274.48792050926</v>
       </c>
       <c r="W224">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X224" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="Y224" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AB224">
         <v>0</v>
       </c>
       <c r="AC224" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AH224" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AI224" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="225" spans="1:35">
       <c r="A225">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B225" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C225" t="s">
         <v>50</v>
@@ -17890,25 +17909,25 @@
         <v>51</v>
       </c>
       <c r="E225" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F225" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G225">
-        <v>1867</v>
+        <v>9746</v>
       </c>
       <c r="H225">
         <v>0</v>
       </c>
       <c r="I225" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J225" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="N225" s="1">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="P225">
         <v>8</v>
@@ -17917,37 +17936,975 @@
         <v>2026</v>
       </c>
       <c r="R225">
+        <v>18190457</v>
+      </c>
+      <c r="S225" t="s">
+        <v>143</v>
+      </c>
+      <c r="T225" t="s">
+        <v>161</v>
+      </c>
+      <c r="U225" t="s">
+        <v>165</v>
+      </c>
+      <c r="V225" s="1">
+        <v>46274.34198912037</v>
+      </c>
+      <c r="W225">
+        <v>-1</v>
+      </c>
+      <c r="X225" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB225">
+        <v>0</v>
+      </c>
+      <c r="AC225" t="s">
+        <v>143</v>
+      </c>
+      <c r="AH225" t="s">
+        <v>251</v>
+      </c>
+      <c r="AI225" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="226" spans="1:35">
+      <c r="A226">
+        <v>6627</v>
+      </c>
+      <c r="B226" t="s">
+        <v>36</v>
+      </c>
+      <c r="C226" t="s">
+        <v>50</v>
+      </c>
+      <c r="D226" t="s">
+        <v>51</v>
+      </c>
+      <c r="E226" t="s">
+        <v>55</v>
+      </c>
+      <c r="F226" t="s">
+        <v>56</v>
+      </c>
+      <c r="G226">
+        <v>1866</v>
+      </c>
+      <c r="H226">
+        <v>0</v>
+      </c>
+      <c r="I226" t="s">
+        <v>62</v>
+      </c>
+      <c r="J226" t="s">
+        <v>100</v>
+      </c>
+      <c r="N226" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P226">
+        <v>8</v>
+      </c>
+      <c r="Q226">
+        <v>2026</v>
+      </c>
+      <c r="R226">
+        <v>17968368</v>
+      </c>
+      <c r="S226" t="s">
+        <v>149</v>
+      </c>
+      <c r="T226" t="s">
+        <v>149</v>
+      </c>
+      <c r="U226" t="s">
+        <v>166</v>
+      </c>
+      <c r="V226" s="1">
+        <v>46274.36843923611</v>
+      </c>
+      <c r="W226">
+        <v>0</v>
+      </c>
+      <c r="X226" t="s">
+        <v>168</v>
+      </c>
+      <c r="Y226" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB226">
+        <v>0</v>
+      </c>
+      <c r="AC226" t="s">
+        <v>149</v>
+      </c>
+      <c r="AH226" t="s">
+        <v>252</v>
+      </c>
+      <c r="AI226" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="227" spans="1:35">
+      <c r="A227">
+        <v>6627</v>
+      </c>
+      <c r="B227" t="s">
+        <v>36</v>
+      </c>
+      <c r="C227" t="s">
+        <v>50</v>
+      </c>
+      <c r="D227" t="s">
+        <v>51</v>
+      </c>
+      <c r="E227" t="s">
+        <v>55</v>
+      </c>
+      <c r="F227" t="s">
+        <v>56</v>
+      </c>
+      <c r="G227">
+        <v>1867</v>
+      </c>
+      <c r="H227">
+        <v>0</v>
+      </c>
+      <c r="I227" t="s">
+        <v>62</v>
+      </c>
+      <c r="J227" t="s">
+        <v>101</v>
+      </c>
+      <c r="N227" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P227">
+        <v>8</v>
+      </c>
+      <c r="Q227">
+        <v>2026</v>
+      </c>
+      <c r="R227">
         <v>17968379</v>
       </c>
-      <c r="S225" t="s">
+      <c r="S227" t="s">
         <v>149</v>
       </c>
-      <c r="T225" t="s">
+      <c r="T227" t="s">
         <v>149</v>
       </c>
-      <c r="U225" t="s">
+      <c r="U227" t="s">
         <v>166</v>
       </c>
-      <c r="V225" s="1">
+      <c r="V227" s="1">
         <v>46274.36695243056</v>
       </c>
-      <c r="W225">
-        <v>0</v>
-      </c>
-      <c r="X225" t="s">
+      <c r="W227">
+        <v>0</v>
+      </c>
+      <c r="X227" t="s">
         <v>168</v>
       </c>
-      <c r="AB225">
-        <v>0</v>
-      </c>
-      <c r="AC225" t="s">
+      <c r="AB227">
+        <v>0</v>
+      </c>
+      <c r="AC227" t="s">
         <v>149</v>
       </c>
-      <c r="AH225" t="s">
-        <v>249</v>
-      </c>
-      <c r="AI225" t="s">
+      <c r="AH227" t="s">
         <v>252</v>
+      </c>
+      <c r="AI227" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="228" spans="1:35">
+      <c r="A228">
+        <v>5417</v>
+      </c>
+      <c r="B228" t="s">
+        <v>43</v>
+      </c>
+      <c r="C228" t="s">
+        <v>50</v>
+      </c>
+      <c r="D228" t="s">
+        <v>51</v>
+      </c>
+      <c r="E228" t="s">
+        <v>54</v>
+      </c>
+      <c r="F228" t="s">
+        <v>56</v>
+      </c>
+      <c r="G228">
+        <v>11303</v>
+      </c>
+      <c r="H228">
+        <v>0</v>
+      </c>
+      <c r="I228" t="s">
+        <v>63</v>
+      </c>
+      <c r="J228" t="s">
+        <v>111</v>
+      </c>
+      <c r="N228" s="1">
+        <v>46279</v>
+      </c>
+      <c r="P228">
+        <v>8</v>
+      </c>
+      <c r="Q228">
+        <v>2026</v>
+      </c>
+      <c r="R228">
+        <v>17399454</v>
+      </c>
+      <c r="S228" t="s">
+        <v>153</v>
+      </c>
+      <c r="T228" t="s">
+        <v>163</v>
+      </c>
+      <c r="U228" t="s">
+        <v>165</v>
+      </c>
+      <c r="V228" s="1">
+        <v>46274.42878043981</v>
+      </c>
+      <c r="W228">
+        <v>-5</v>
+      </c>
+      <c r="X228" t="s">
+        <v>173</v>
+      </c>
+      <c r="Y228" t="s">
+        <v>246</v>
+      </c>
+      <c r="AB228">
+        <v>0</v>
+      </c>
+      <c r="AC228" t="s">
+        <v>153</v>
+      </c>
+      <c r="AH228" t="s">
+        <v>251</v>
+      </c>
+      <c r="AI228" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="229" spans="1:35">
+      <c r="A229">
+        <v>6703</v>
+      </c>
+      <c r="B229" t="s">
+        <v>46</v>
+      </c>
+      <c r="C229" t="s">
+        <v>50</v>
+      </c>
+      <c r="D229" t="s">
+        <v>53</v>
+      </c>
+      <c r="E229" t="s">
+        <v>54</v>
+      </c>
+      <c r="F229" t="s">
+        <v>56</v>
+      </c>
+      <c r="G229">
+        <v>5989</v>
+      </c>
+      <c r="H229">
+        <v>0</v>
+      </c>
+      <c r="I229" t="s">
+        <v>64</v>
+      </c>
+      <c r="J229" t="s">
+        <v>119</v>
+      </c>
+      <c r="N229" s="1">
+        <v>46273</v>
+      </c>
+      <c r="P229">
+        <v>9</v>
+      </c>
+      <c r="Q229">
+        <v>2026</v>
+      </c>
+      <c r="R229">
+        <v>17941177</v>
+      </c>
+      <c r="S229" t="s">
+        <v>154</v>
+      </c>
+      <c r="U229" t="s">
+        <v>164</v>
+      </c>
+      <c r="V229" s="1">
+        <v>46274.41771849537</v>
+      </c>
+      <c r="W229">
+        <v>1</v>
+      </c>
+      <c r="X229" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB229">
+        <v>0</v>
+      </c>
+      <c r="AC229" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH229" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI229" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="230" spans="1:35">
+      <c r="A230">
+        <v>6704</v>
+      </c>
+      <c r="B230" t="s">
+        <v>42</v>
+      </c>
+      <c r="C230" t="s">
+        <v>50</v>
+      </c>
+      <c r="D230" t="s">
+        <v>51</v>
+      </c>
+      <c r="E230" t="s">
+        <v>54</v>
+      </c>
+      <c r="F230" t="s">
+        <v>56</v>
+      </c>
+      <c r="G230">
+        <v>5989</v>
+      </c>
+      <c r="H230">
+        <v>0</v>
+      </c>
+      <c r="I230" t="s">
+        <v>64</v>
+      </c>
+      <c r="J230" t="s">
+        <v>119</v>
+      </c>
+      <c r="N230" s="1">
+        <v>46273</v>
+      </c>
+      <c r="P230">
+        <v>9</v>
+      </c>
+      <c r="Q230">
+        <v>2026</v>
+      </c>
+      <c r="R230">
+        <v>17952385</v>
+      </c>
+      <c r="S230" t="s">
+        <v>154</v>
+      </c>
+      <c r="U230" t="s">
+        <v>164</v>
+      </c>
+      <c r="V230" s="1">
+        <v>46274.41775447917</v>
+      </c>
+      <c r="W230">
+        <v>1</v>
+      </c>
+      <c r="X230" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB230">
+        <v>0</v>
+      </c>
+      <c r="AC230" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH230" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI230" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="231" spans="1:35">
+      <c r="A231">
+        <v>6705</v>
+      </c>
+      <c r="B231" t="s">
+        <v>48</v>
+      </c>
+      <c r="C231" t="s">
+        <v>50</v>
+      </c>
+      <c r="D231" t="s">
+        <v>52</v>
+      </c>
+      <c r="E231" t="s">
+        <v>54</v>
+      </c>
+      <c r="F231" t="s">
+        <v>56</v>
+      </c>
+      <c r="G231">
+        <v>5989</v>
+      </c>
+      <c r="H231">
+        <v>0</v>
+      </c>
+      <c r="I231" t="s">
+        <v>64</v>
+      </c>
+      <c r="J231" t="s">
+        <v>119</v>
+      </c>
+      <c r="N231" s="1">
+        <v>46273</v>
+      </c>
+      <c r="P231">
+        <v>9</v>
+      </c>
+      <c r="Q231">
+        <v>2026</v>
+      </c>
+      <c r="R231">
+        <v>17952569</v>
+      </c>
+      <c r="S231" t="s">
+        <v>154</v>
+      </c>
+      <c r="U231" t="s">
+        <v>164</v>
+      </c>
+      <c r="V231" s="1">
+        <v>46274.41777533565</v>
+      </c>
+      <c r="W231">
+        <v>1</v>
+      </c>
+      <c r="X231" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB231">
+        <v>0</v>
+      </c>
+      <c r="AC231" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH231" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI231" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="232" spans="1:35">
+      <c r="A232">
+        <v>6945</v>
+      </c>
+      <c r="B232" t="s">
+        <v>39</v>
+      </c>
+      <c r="C232" t="s">
+        <v>50</v>
+      </c>
+      <c r="D232" t="s">
+        <v>52</v>
+      </c>
+      <c r="E232" t="s">
+        <v>54</v>
+      </c>
+      <c r="F232" t="s">
+        <v>57</v>
+      </c>
+      <c r="G232">
+        <v>5989</v>
+      </c>
+      <c r="H232">
+        <v>0</v>
+      </c>
+      <c r="I232" t="s">
+        <v>64</v>
+      </c>
+      <c r="J232" t="s">
+        <v>119</v>
+      </c>
+      <c r="N232" s="1">
+        <v>46273</v>
+      </c>
+      <c r="P232">
+        <v>9</v>
+      </c>
+      <c r="Q232">
+        <v>2026</v>
+      </c>
+      <c r="R232">
+        <v>18164516</v>
+      </c>
+      <c r="S232" t="s">
+        <v>154</v>
+      </c>
+      <c r="U232" t="s">
+        <v>164</v>
+      </c>
+      <c r="V232" s="1">
+        <v>46274.41799166667</v>
+      </c>
+      <c r="W232">
+        <v>1</v>
+      </c>
+      <c r="X232" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB232">
+        <v>0</v>
+      </c>
+      <c r="AC232" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH232" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI232" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="233" spans="1:35">
+      <c r="A233">
+        <v>6949</v>
+      </c>
+      <c r="B233" t="s">
+        <v>37</v>
+      </c>
+      <c r="C233" t="s">
+        <v>50</v>
+      </c>
+      <c r="D233" t="s">
+        <v>51</v>
+      </c>
+      <c r="E233" t="s">
+        <v>54</v>
+      </c>
+      <c r="F233" t="s">
+        <v>57</v>
+      </c>
+      <c r="G233">
+        <v>5989</v>
+      </c>
+      <c r="H233">
+        <v>0</v>
+      </c>
+      <c r="I233" t="s">
+        <v>64</v>
+      </c>
+      <c r="J233" t="s">
+        <v>119</v>
+      </c>
+      <c r="N233" s="1">
+        <v>46273</v>
+      </c>
+      <c r="P233">
+        <v>9</v>
+      </c>
+      <c r="Q233">
+        <v>2026</v>
+      </c>
+      <c r="R233">
+        <v>18178157</v>
+      </c>
+      <c r="S233" t="s">
+        <v>154</v>
+      </c>
+      <c r="U233" t="s">
+        <v>164</v>
+      </c>
+      <c r="V233" s="1">
+        <v>46274.41800114583</v>
+      </c>
+      <c r="W233">
+        <v>1</v>
+      </c>
+      <c r="X233" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB233">
+        <v>0</v>
+      </c>
+      <c r="AC233" t="s">
+        <v>154</v>
+      </c>
+      <c r="AH233" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI233" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="234" spans="1:35">
+      <c r="A234">
+        <v>6703</v>
+      </c>
+      <c r="B234" t="s">
+        <v>46</v>
+      </c>
+      <c r="C234" t="s">
+        <v>50</v>
+      </c>
+      <c r="D234" t="s">
+        <v>53</v>
+      </c>
+      <c r="E234" t="s">
+        <v>54</v>
+      </c>
+      <c r="F234" t="s">
+        <v>56</v>
+      </c>
+      <c r="G234">
+        <v>6215</v>
+      </c>
+      <c r="H234">
+        <v>0</v>
+      </c>
+      <c r="I234" t="s">
+        <v>65</v>
+      </c>
+      <c r="J234" t="s">
+        <v>121</v>
+      </c>
+      <c r="N234" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P234">
+        <v>9</v>
+      </c>
+      <c r="Q234">
+        <v>2026</v>
+      </c>
+      <c r="R234">
+        <v>17941187</v>
+      </c>
+      <c r="S234" t="s">
+        <v>54</v>
+      </c>
+      <c r="U234" t="s">
+        <v>166</v>
+      </c>
+      <c r="V234" s="1">
+        <v>46274.41772148148</v>
+      </c>
+      <c r="W234">
+        <v>0</v>
+      </c>
+      <c r="X234" t="s">
+        <v>176</v>
+      </c>
+      <c r="AB234">
+        <v>0</v>
+      </c>
+      <c r="AC234" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH234" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI234" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="235" spans="1:35">
+      <c r="A235">
+        <v>6704</v>
+      </c>
+      <c r="B235" t="s">
+        <v>42</v>
+      </c>
+      <c r="C235" t="s">
+        <v>50</v>
+      </c>
+      <c r="D235" t="s">
+        <v>51</v>
+      </c>
+      <c r="E235" t="s">
+        <v>54</v>
+      </c>
+      <c r="F235" t="s">
+        <v>56</v>
+      </c>
+      <c r="G235">
+        <v>6215</v>
+      </c>
+      <c r="H235">
+        <v>0</v>
+      </c>
+      <c r="I235" t="s">
+        <v>65</v>
+      </c>
+      <c r="J235" t="s">
+        <v>121</v>
+      </c>
+      <c r="N235" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P235">
+        <v>9</v>
+      </c>
+      <c r="Q235">
+        <v>2026</v>
+      </c>
+      <c r="R235">
+        <v>17952400</v>
+      </c>
+      <c r="S235" t="s">
+        <v>54</v>
+      </c>
+      <c r="U235" t="s">
+        <v>166</v>
+      </c>
+      <c r="V235" s="1">
+        <v>46274.41773631945</v>
+      </c>
+      <c r="W235">
+        <v>0</v>
+      </c>
+      <c r="X235" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB235">
+        <v>0</v>
+      </c>
+      <c r="AC235" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH235" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI235" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="236" spans="1:35">
+      <c r="A236">
+        <v>6705</v>
+      </c>
+      <c r="B236" t="s">
+        <v>48</v>
+      </c>
+      <c r="C236" t="s">
+        <v>50</v>
+      </c>
+      <c r="D236" t="s">
+        <v>52</v>
+      </c>
+      <c r="E236" t="s">
+        <v>54</v>
+      </c>
+      <c r="F236" t="s">
+        <v>56</v>
+      </c>
+      <c r="G236">
+        <v>6215</v>
+      </c>
+      <c r="H236">
+        <v>0</v>
+      </c>
+      <c r="I236" t="s">
+        <v>65</v>
+      </c>
+      <c r="J236" t="s">
+        <v>121</v>
+      </c>
+      <c r="N236" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P236">
+        <v>9</v>
+      </c>
+      <c r="Q236">
+        <v>2026</v>
+      </c>
+      <c r="R236">
+        <v>17952580</v>
+      </c>
+      <c r="S236" t="s">
+        <v>54</v>
+      </c>
+      <c r="U236" t="s">
+        <v>166</v>
+      </c>
+      <c r="V236" s="1">
+        <v>46274.41777481481</v>
+      </c>
+      <c r="W236">
+        <v>0</v>
+      </c>
+      <c r="X236" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB236">
+        <v>0</v>
+      </c>
+      <c r="AC236" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH236" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI236" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="237" spans="1:35">
+      <c r="A237">
+        <v>6945</v>
+      </c>
+      <c r="B237" t="s">
+        <v>39</v>
+      </c>
+      <c r="C237" t="s">
+        <v>50</v>
+      </c>
+      <c r="D237" t="s">
+        <v>52</v>
+      </c>
+      <c r="E237" t="s">
+        <v>54</v>
+      </c>
+      <c r="F237" t="s">
+        <v>57</v>
+      </c>
+      <c r="G237">
+        <v>6215</v>
+      </c>
+      <c r="H237">
+        <v>0</v>
+      </c>
+      <c r="I237" t="s">
+        <v>65</v>
+      </c>
+      <c r="J237" t="s">
+        <v>121</v>
+      </c>
+      <c r="N237" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P237">
+        <v>9</v>
+      </c>
+      <c r="Q237">
+        <v>2026</v>
+      </c>
+      <c r="R237">
+        <v>18164523</v>
+      </c>
+      <c r="S237" t="s">
+        <v>54</v>
+      </c>
+      <c r="U237" t="s">
+        <v>166</v>
+      </c>
+      <c r="V237" s="1">
+        <v>46274.41799332176</v>
+      </c>
+      <c r="W237">
+        <v>0</v>
+      </c>
+      <c r="X237" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB237">
+        <v>0</v>
+      </c>
+      <c r="AC237" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH237" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI237" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="238" spans="1:35">
+      <c r="A238">
+        <v>6949</v>
+      </c>
+      <c r="B238" t="s">
+        <v>37</v>
+      </c>
+      <c r="C238" t="s">
+        <v>50</v>
+      </c>
+      <c r="D238" t="s">
+        <v>51</v>
+      </c>
+      <c r="E238" t="s">
+        <v>54</v>
+      </c>
+      <c r="F238" t="s">
+        <v>57</v>
+      </c>
+      <c r="G238">
+        <v>6215</v>
+      </c>
+      <c r="H238">
+        <v>0</v>
+      </c>
+      <c r="I238" t="s">
+        <v>65</v>
+      </c>
+      <c r="J238" t="s">
+        <v>121</v>
+      </c>
+      <c r="N238" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P238">
+        <v>9</v>
+      </c>
+      <c r="Q238">
+        <v>2026</v>
+      </c>
+      <c r="R238">
+        <v>18178163</v>
+      </c>
+      <c r="S238" t="s">
+        <v>155</v>
+      </c>
+      <c r="U238" t="s">
+        <v>166</v>
+      </c>
+      <c r="V238" s="1">
+        <v>46274.41800085648</v>
+      </c>
+      <c r="W238">
+        <v>0</v>
+      </c>
+      <c r="X238" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB238">
+        <v>0</v>
+      </c>
+      <c r="AC238" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH238" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI238" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-09 14:42
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3395" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3426" uniqueCount="258">
   <si>
     <t>CodCliente</t>
   </si>
@@ -760,11 +760,18 @@
 Reunião confirmada pelo cliente - Data Comentário: 04/09/2026 11:03</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 10/09/2026 
+em processamento - Data Comentário: 08/09/2026 16:10</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/09/2026 - Data Comentário: 04/09/2026 16:13</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 10/09/2026 
 Em processamento. - Data Comentário: 04/09/2026 08:41</t>
+  </si>
+  <si>
+    <t>1. Folha em Processamento  Previsão para conclusão dia 10/09/2026 - Data Comentário: 08/09/2026 15:22</t>
   </si>
   <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 09/09/2026 08:35</t>
@@ -1133,7 +1140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI238"/>
+  <dimension ref="A1:AI240"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1314,10 +1321,10 @@
         <v>132</v>
       </c>
       <c r="AH2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1391,10 +1398,10 @@
         <v>133</v>
       </c>
       <c r="AH3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1468,10 +1475,10 @@
         <v>132</v>
       </c>
       <c r="AH4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI4" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1542,10 +1549,10 @@
         <v>132</v>
       </c>
       <c r="AH5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1616,10 +1623,10 @@
         <v>133</v>
       </c>
       <c r="AH6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1690,10 +1697,10 @@
         <v>133</v>
       </c>
       <c r="AH7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI7" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1764,10 +1771,10 @@
         <v>134</v>
       </c>
       <c r="AH8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI8" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1838,10 +1845,10 @@
         <v>132</v>
       </c>
       <c r="AH9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI9" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1912,10 +1919,10 @@
         <v>135</v>
       </c>
       <c r="AH10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1986,10 +1993,10 @@
         <v>135</v>
       </c>
       <c r="AH11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI11" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2060,10 +2067,10 @@
         <v>136</v>
       </c>
       <c r="AH12" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI12" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2131,13 +2138,13 @@
         <v>0</v>
       </c>
       <c r="AC13" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="AH13" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI13" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2205,13 +2212,13 @@
         <v>0</v>
       </c>
       <c r="AC14" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AH14" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2279,10 +2286,10 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI15" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2344,10 +2351,10 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2415,10 +2422,10 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI17" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2492,10 +2499,10 @@
         <v>138</v>
       </c>
       <c r="AH18" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI18" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2569,10 +2576,10 @@
         <v>137</v>
       </c>
       <c r="AH19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2646,10 +2653,10 @@
         <v>138</v>
       </c>
       <c r="AH20" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2723,10 +2730,10 @@
         <v>136</v>
       </c>
       <c r="AH21" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2797,10 +2804,10 @@
         <v>139</v>
       </c>
       <c r="AH22" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI22" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2871,10 +2878,10 @@
         <v>136</v>
       </c>
       <c r="AH23" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI23" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2945,10 +2952,10 @@
         <v>136</v>
       </c>
       <c r="AH24" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI24" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3019,10 +3026,10 @@
         <v>136</v>
       </c>
       <c r="AH25" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI25" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3093,10 +3100,10 @@
         <v>137</v>
       </c>
       <c r="AH26" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI26" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3167,10 +3174,10 @@
         <v>136</v>
       </c>
       <c r="AH27" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI27" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3241,10 +3248,10 @@
         <v>136</v>
       </c>
       <c r="AH28" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI28" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3315,10 +3322,10 @@
         <v>136</v>
       </c>
       <c r="AH29" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI29" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3389,10 +3396,10 @@
         <v>140</v>
       </c>
       <c r="AH30" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI30" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3469,10 +3476,10 @@
         <v>141</v>
       </c>
       <c r="AH31" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI31" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3543,10 +3550,10 @@
         <v>142</v>
       </c>
       <c r="AH32" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI32" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3623,10 +3630,10 @@
         <v>143</v>
       </c>
       <c r="AH33" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI33" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3700,10 +3707,10 @@
         <v>144</v>
       </c>
       <c r="AH34" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI34" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3777,13 +3784,13 @@
         <v>0</v>
       </c>
       <c r="AC35" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AH35" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI35" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3860,10 +3867,10 @@
         <v>146</v>
       </c>
       <c r="AH36" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI36" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3940,10 +3947,10 @@
         <v>140</v>
       </c>
       <c r="AH37" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI37" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4017,10 +4024,10 @@
         <v>162</v>
       </c>
       <c r="AH38" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI38" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4097,10 +4104,10 @@
         <v>141</v>
       </c>
       <c r="AH39" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI39" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4177,10 +4184,10 @@
         <v>141</v>
       </c>
       <c r="AH40" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI40" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4257,10 +4264,10 @@
         <v>141</v>
       </c>
       <c r="AH41" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI41" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4337,10 +4344,10 @@
         <v>140</v>
       </c>
       <c r="AH42" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI42" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4417,10 +4424,10 @@
         <v>147</v>
       </c>
       <c r="AH43" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI43" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4497,10 +4504,10 @@
         <v>142</v>
       </c>
       <c r="AH44" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI44" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4577,10 +4584,10 @@
         <v>143</v>
       </c>
       <c r="AH45" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI45" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4648,10 +4655,10 @@
         <v>144</v>
       </c>
       <c r="AH46" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI46" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4722,10 +4729,10 @@
         <v>141</v>
       </c>
       <c r="AH47" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI47" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4796,10 +4803,10 @@
         <v>141</v>
       </c>
       <c r="AH48" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI48" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4870,10 +4877,10 @@
         <v>141</v>
       </c>
       <c r="AH49" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI49" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4944,10 +4951,10 @@
         <v>140</v>
       </c>
       <c r="AH50" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI50" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5018,10 +5025,10 @@
         <v>147</v>
       </c>
       <c r="AH51" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI51" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5098,10 +5105,10 @@
         <v>142</v>
       </c>
       <c r="AH52" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI52" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5172,10 +5179,10 @@
         <v>143</v>
       </c>
       <c r="AH53" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI53" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5252,10 +5259,10 @@
         <v>141</v>
       </c>
       <c r="AH54" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI54" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5332,10 +5339,10 @@
         <v>141</v>
       </c>
       <c r="AH55" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI55" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5412,10 +5419,10 @@
         <v>141</v>
       </c>
       <c r="AH56" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI56" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5492,10 +5499,10 @@
         <v>140</v>
       </c>
       <c r="AH57" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI57" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5569,10 +5576,10 @@
         <v>144</v>
       </c>
       <c r="AH58" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI58" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5646,13 +5653,13 @@
         <v>0</v>
       </c>
       <c r="AC59" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AH59" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI59" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5729,10 +5736,10 @@
         <v>141</v>
       </c>
       <c r="AH60" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI60" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5809,10 +5816,10 @@
         <v>141</v>
       </c>
       <c r="AH61" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI61" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5889,10 +5896,10 @@
         <v>141</v>
       </c>
       <c r="AH62" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI62" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -5969,10 +5976,10 @@
         <v>140</v>
       </c>
       <c r="AH63" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI63" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6049,10 +6056,10 @@
         <v>147</v>
       </c>
       <c r="AH64" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI64" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6129,10 +6136,10 @@
         <v>142</v>
       </c>
       <c r="AH65" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI65" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6209,10 +6216,10 @@
         <v>143</v>
       </c>
       <c r="AH66" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI66" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6289,10 +6296,10 @@
         <v>141</v>
       </c>
       <c r="AH67" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI67" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6360,10 +6367,10 @@
         <v>144</v>
       </c>
       <c r="AH68" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI68" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6431,13 +6438,13 @@
         <v>0</v>
       </c>
       <c r="AC69" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AH69" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI69" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6508,10 +6515,10 @@
         <v>141</v>
       </c>
       <c r="AH70" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI70" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6582,10 +6589,10 @@
         <v>141</v>
       </c>
       <c r="AH71" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI71" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6656,10 +6663,10 @@
         <v>141</v>
       </c>
       <c r="AH72" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI72" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6730,10 +6737,10 @@
         <v>140</v>
       </c>
       <c r="AH73" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI73" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6804,10 +6811,10 @@
         <v>147</v>
       </c>
       <c r="AH74" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI74" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6878,10 +6885,10 @@
         <v>142</v>
       </c>
       <c r="AH75" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI75" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6952,10 +6959,10 @@
         <v>143</v>
       </c>
       <c r="AH76" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI76" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7026,10 +7033,10 @@
         <v>143</v>
       </c>
       <c r="AH77" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI77" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7100,10 +7107,10 @@
         <v>143</v>
       </c>
       <c r="AH78" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI78" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7174,10 +7181,10 @@
         <v>143</v>
       </c>
       <c r="AH79" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI79" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7248,10 +7255,10 @@
         <v>149</v>
       </c>
       <c r="AH80" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI80" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7322,10 +7329,10 @@
         <v>149</v>
       </c>
       <c r="AH81" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI81" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7396,10 +7403,10 @@
         <v>150</v>
       </c>
       <c r="AH82" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI82" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7470,10 +7477,10 @@
         <v>149</v>
       </c>
       <c r="AH83" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI83" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7544,10 +7551,10 @@
         <v>149</v>
       </c>
       <c r="AH84" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI84" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7621,10 +7628,10 @@
         <v>149</v>
       </c>
       <c r="AH85" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI85" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7695,10 +7702,10 @@
         <v>150</v>
       </c>
       <c r="AH86" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI86" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7769,10 +7776,10 @@
         <v>149</v>
       </c>
       <c r="AH87" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI87" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7843,10 +7850,10 @@
         <v>149</v>
       </c>
       <c r="AH88" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI88" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7917,10 +7924,10 @@
         <v>149</v>
       </c>
       <c r="AH89" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI89" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -7988,10 +7995,10 @@
         <v>149</v>
       </c>
       <c r="AH90" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI90" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8062,10 +8069,10 @@
         <v>150</v>
       </c>
       <c r="AH91" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI91" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8136,10 +8143,10 @@
         <v>149</v>
       </c>
       <c r="AH92" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI92" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8210,10 +8217,10 @@
         <v>149</v>
       </c>
       <c r="AH93" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI93" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8284,10 +8291,10 @@
         <v>149</v>
       </c>
       <c r="AH94" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI94" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8355,10 +8362,10 @@
         <v>149</v>
       </c>
       <c r="AH95" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI95" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8429,10 +8436,10 @@
         <v>150</v>
       </c>
       <c r="AH96" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI96" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8503,10 +8510,10 @@
         <v>149</v>
       </c>
       <c r="AH97" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI97" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8577,10 +8584,10 @@
         <v>149</v>
       </c>
       <c r="AH98" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI98" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8651,10 +8658,10 @@
         <v>150</v>
       </c>
       <c r="AH99" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI99" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8731,10 +8738,10 @@
         <v>149</v>
       </c>
       <c r="AH100" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI100" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8802,10 +8809,10 @@
         <v>149</v>
       </c>
       <c r="AH101" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI101" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8876,10 +8883,10 @@
         <v>149</v>
       </c>
       <c r="AH102" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI102" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8950,10 +8957,10 @@
         <v>149</v>
       </c>
       <c r="AH103" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI103" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9024,10 +9031,10 @@
         <v>149</v>
       </c>
       <c r="AH104" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI104" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9095,10 +9102,10 @@
         <v>149</v>
       </c>
       <c r="AH105" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI105" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9169,10 +9176,10 @@
         <v>150</v>
       </c>
       <c r="AH106" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI106" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9243,10 +9250,10 @@
         <v>149</v>
       </c>
       <c r="AH107" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI107" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9317,10 +9324,10 @@
         <v>149</v>
       </c>
       <c r="AH108" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI108" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9388,10 +9395,10 @@
         <v>149</v>
       </c>
       <c r="AH109" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI109" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9462,10 +9469,10 @@
         <v>150</v>
       </c>
       <c r="AH110" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI110" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9533,10 +9540,10 @@
         <v>151</v>
       </c>
       <c r="AH111" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI111" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9607,10 +9614,10 @@
         <v>150</v>
       </c>
       <c r="AH112" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI112" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9681,10 +9688,10 @@
         <v>148</v>
       </c>
       <c r="AH113" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI113" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9752,10 +9759,10 @@
         <v>151</v>
       </c>
       <c r="AH114" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI114" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9826,10 +9833,10 @@
         <v>150</v>
       </c>
       <c r="AH115" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI115" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9900,10 +9907,10 @@
         <v>149</v>
       </c>
       <c r="AH116" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI116" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -9974,10 +9981,10 @@
         <v>149</v>
       </c>
       <c r="AH117" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI117" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10048,10 +10055,10 @@
         <v>149</v>
       </c>
       <c r="AH118" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI118" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10119,10 +10126,10 @@
         <v>149</v>
       </c>
       <c r="AH119" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI119" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10193,10 +10200,10 @@
         <v>150</v>
       </c>
       <c r="AH120" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI120" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10267,10 +10274,10 @@
         <v>149</v>
       </c>
       <c r="AH121" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI121" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10341,10 +10348,10 @@
         <v>149</v>
       </c>
       <c r="AH122" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI122" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10415,10 +10422,10 @@
         <v>149</v>
       </c>
       <c r="AH123" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI123" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10486,10 +10493,10 @@
         <v>149</v>
       </c>
       <c r="AH124" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI124" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10560,10 +10567,10 @@
         <v>150</v>
       </c>
       <c r="AH125" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI125" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10640,10 +10647,10 @@
         <v>150</v>
       </c>
       <c r="AH126" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI126" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10720,10 +10727,10 @@
         <v>150</v>
       </c>
       <c r="AH127" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI127" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10794,10 +10801,10 @@
         <v>153</v>
       </c>
       <c r="AH128" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI128" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10868,10 +10875,10 @@
         <v>153</v>
       </c>
       <c r="AH129" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI129" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -10948,10 +10955,10 @@
         <v>153</v>
       </c>
       <c r="AH130" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI130" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11022,10 +11029,10 @@
         <v>153</v>
       </c>
       <c r="AH131" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI131" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11096,10 +11103,10 @@
         <v>153</v>
       </c>
       <c r="AH132" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI132" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11170,10 +11177,10 @@
         <v>153</v>
       </c>
       <c r="AH133" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11244,10 +11251,10 @@
         <v>153</v>
       </c>
       <c r="AH134" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI134" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11324,10 +11331,10 @@
         <v>153</v>
       </c>
       <c r="AH135" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI135" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11398,10 +11405,10 @@
         <v>153</v>
       </c>
       <c r="AH136" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI136" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11472,10 +11479,10 @@
         <v>153</v>
       </c>
       <c r="AH137" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI137" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11546,10 +11553,10 @@
         <v>153</v>
       </c>
       <c r="AH138" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI138" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11626,10 +11633,10 @@
         <v>153</v>
       </c>
       <c r="AH139" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI139" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11700,10 +11707,10 @@
         <v>153</v>
       </c>
       <c r="AH140" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI140" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11774,10 +11781,10 @@
         <v>153</v>
       </c>
       <c r="AH141" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI141" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11848,10 +11855,10 @@
         <v>153</v>
       </c>
       <c r="AH142" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI142" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11922,10 +11929,10 @@
         <v>153</v>
       </c>
       <c r="AH143" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI143" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -11996,10 +12003,10 @@
         <v>153</v>
       </c>
       <c r="AH144" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI144" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12070,10 +12077,10 @@
         <v>153</v>
       </c>
       <c r="AH145" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI145" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12144,10 +12151,10 @@
         <v>153</v>
       </c>
       <c r="AH146" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI146" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12218,10 +12225,10 @@
         <v>153</v>
       </c>
       <c r="AH147" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI147" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12292,10 +12299,10 @@
         <v>153</v>
       </c>
       <c r="AH148" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI148" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12366,10 +12373,10 @@
         <v>153</v>
       </c>
       <c r="AH149" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI149" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12446,10 +12453,10 @@
         <v>153</v>
       </c>
       <c r="AH150" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI150" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12520,10 +12527,10 @@
         <v>153</v>
       </c>
       <c r="AH151" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI151" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12594,10 +12601,10 @@
         <v>153</v>
       </c>
       <c r="AH152" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI152" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12668,10 +12675,10 @@
         <v>153</v>
       </c>
       <c r="AH153" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI153" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12742,10 +12749,10 @@
         <v>154</v>
       </c>
       <c r="AH154" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI154" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12816,10 +12823,10 @@
         <v>154</v>
       </c>
       <c r="AH155" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI155" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12890,10 +12897,10 @@
         <v>154</v>
       </c>
       <c r="AH156" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI156" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -12964,10 +12971,10 @@
         <v>154</v>
       </c>
       <c r="AH157" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI157" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13038,10 +13045,10 @@
         <v>154</v>
       </c>
       <c r="AH158" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI158" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13112,10 +13119,10 @@
         <v>154</v>
       </c>
       <c r="AH159" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI159" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13186,10 +13193,10 @@
         <v>154</v>
       </c>
       <c r="AH160" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI160" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13260,10 +13267,10 @@
         <v>154</v>
       </c>
       <c r="AH161" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI161" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13334,10 +13341,10 @@
         <v>154</v>
       </c>
       <c r="AH162" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI162" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13408,10 +13415,10 @@
         <v>154</v>
       </c>
       <c r="AH163" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI163" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13482,10 +13489,10 @@
         <v>154</v>
       </c>
       <c r="AH164" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI164" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13556,10 +13563,10 @@
         <v>154</v>
       </c>
       <c r="AH165" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI165" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13630,10 +13637,10 @@
         <v>154</v>
       </c>
       <c r="AH166" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI166" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13704,10 +13711,10 @@
         <v>154</v>
       </c>
       <c r="AH167" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI167" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13778,10 +13785,10 @@
         <v>154</v>
       </c>
       <c r="AH168" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI168" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13852,10 +13859,10 @@
         <v>154</v>
       </c>
       <c r="AH169" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI169" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13926,10 +13933,10 @@
         <v>154</v>
       </c>
       <c r="AH170" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI170" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14000,10 +14007,10 @@
         <v>154</v>
       </c>
       <c r="AH171" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI171" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14074,10 +14081,10 @@
         <v>154</v>
       </c>
       <c r="AH172" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI172" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14148,10 +14155,10 @@
         <v>154</v>
       </c>
       <c r="AH173" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AI173" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14225,10 +14232,10 @@
         <v>154</v>
       </c>
       <c r="AH174" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI174" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14302,10 +14309,10 @@
         <v>154</v>
       </c>
       <c r="AH175" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI175" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14379,10 +14386,10 @@
         <v>154</v>
       </c>
       <c r="AH176" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI176" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14456,10 +14463,10 @@
         <v>154</v>
       </c>
       <c r="AH177" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI177" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14533,10 +14540,10 @@
         <v>154</v>
       </c>
       <c r="AH178" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI178" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14610,10 +14617,10 @@
         <v>154</v>
       </c>
       <c r="AH179" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI179" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14687,10 +14694,10 @@
         <v>154</v>
       </c>
       <c r="AH180" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI180" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14764,10 +14771,10 @@
         <v>154</v>
       </c>
       <c r="AH181" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI181" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14841,10 +14848,10 @@
         <v>154</v>
       </c>
       <c r="AH182" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI182" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14918,10 +14925,10 @@
         <v>154</v>
       </c>
       <c r="AH183" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI183" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -14995,10 +15002,10 @@
         <v>154</v>
       </c>
       <c r="AH184" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI184" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15072,10 +15079,10 @@
         <v>154</v>
       </c>
       <c r="AH185" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI185" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15149,10 +15156,10 @@
         <v>154</v>
       </c>
       <c r="AH186" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI186" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15226,10 +15233,10 @@
         <v>154</v>
       </c>
       <c r="AH187" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI187" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15297,10 +15304,10 @@
         <v>154</v>
       </c>
       <c r="AH188" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI188" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15368,10 +15375,10 @@
         <v>154</v>
       </c>
       <c r="AH189" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI189" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15439,10 +15446,10 @@
         <v>154</v>
       </c>
       <c r="AH190" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI190" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15510,10 +15517,10 @@
         <v>154</v>
       </c>
       <c r="AH191" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI191" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15581,10 +15588,10 @@
         <v>154</v>
       </c>
       <c r="AH192" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI192" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15652,10 +15659,10 @@
         <v>154</v>
       </c>
       <c r="AH193" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI193" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15723,10 +15730,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI194" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15794,10 +15801,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI195" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15865,10 +15872,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI196" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15936,10 +15943,10 @@
         <v>54</v>
       </c>
       <c r="AH197" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI197" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -16007,10 +16014,10 @@
         <v>155</v>
       </c>
       <c r="AH198" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI198" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16078,10 +16085,10 @@
         <v>55</v>
       </c>
       <c r="AH199" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI199" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16149,10 +16156,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI200" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16220,10 +16227,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI201" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16291,10 +16298,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI202" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16362,10 +16369,10 @@
         <v>155</v>
       </c>
       <c r="AH203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI203" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16433,10 +16440,10 @@
         <v>54</v>
       </c>
       <c r="AH204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16504,10 +16511,10 @@
         <v>155</v>
       </c>
       <c r="AH205" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16575,10 +16582,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI206" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16646,10 +16653,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI207" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16717,10 +16724,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI208" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16788,10 +16795,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI209" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16859,10 +16866,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI210" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -16930,10 +16937,10 @@
         <v>54</v>
       </c>
       <c r="AH211" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI211" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -17001,10 +17008,10 @@
         <v>155</v>
       </c>
       <c r="AH212" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI212" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17072,10 +17079,10 @@
         <v>55</v>
       </c>
       <c r="AH213" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI213" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17146,10 +17153,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI214" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17220,10 +17227,10 @@
         <v>54</v>
       </c>
       <c r="AH215" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI215" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17294,10 +17301,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI216" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17368,10 +17375,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI217" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17439,10 +17446,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI218" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17510,10 +17517,10 @@
         <v>54</v>
       </c>
       <c r="AH219" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI219" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17584,10 +17591,10 @@
         <v>54</v>
       </c>
       <c r="AH220" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI220" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17655,10 +17662,10 @@
         <v>54</v>
       </c>
       <c r="AH221" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI221" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17726,21 +17733,21 @@
         <v>0</v>
       </c>
       <c r="AC222" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="AH222" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI222" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="223" spans="1:35">
       <c r="A223">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B223" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C223" t="s">
         <v>50</v>
@@ -17770,7 +17777,7 @@
         <v>46275</v>
       </c>
       <c r="O223" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="P223">
         <v>8</v>
@@ -17779,25 +17786,22 @@
         <v>2026</v>
       </c>
       <c r="R223">
-        <v>16976300</v>
+        <v>17399403</v>
       </c>
       <c r="S223" t="s">
-        <v>141</v>
-      </c>
-      <c r="T223" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="U223" t="s">
         <v>165</v>
       </c>
       <c r="V223" s="1">
-        <v>46274.47210818287</v>
+        <v>46274.60593387731</v>
       </c>
       <c r="W223">
         <v>-1</v>
       </c>
       <c r="X223" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Y223" t="s">
         <v>243</v>
@@ -17806,27 +17810,27 @@
         <v>0</v>
       </c>
       <c r="AC223" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AH223" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI223" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="224" spans="1:35">
       <c r="A224">
-        <v>6779</v>
+        <v>6486</v>
       </c>
       <c r="B224" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C224" t="s">
         <v>50</v>
       </c>
       <c r="D224" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E224" t="s">
         <v>54</v>
@@ -17850,7 +17854,7 @@
         <v>46275</v>
       </c>
       <c r="O224" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P224">
         <v>8</v>
@@ -17859,25 +17863,25 @@
         <v>2026</v>
       </c>
       <c r="R224">
-        <v>18090250</v>
+        <v>16976300</v>
       </c>
       <c r="S224" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="T224" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="U224" t="s">
         <v>165</v>
       </c>
       <c r="V224" s="1">
-        <v>46274.48792050926</v>
+        <v>46274.47210818287</v>
       </c>
       <c r="W224">
         <v>-1</v>
       </c>
       <c r="X224" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="Y224" t="s">
         <v>244</v>
@@ -17886,33 +17890,33 @@
         <v>0</v>
       </c>
       <c r="AC224" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="AH224" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI224" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="225" spans="1:35">
       <c r="A225">
-        <v>6949</v>
+        <v>6779</v>
       </c>
       <c r="B225" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C225" t="s">
         <v>50</v>
       </c>
       <c r="D225" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E225" t="s">
         <v>54</v>
       </c>
       <c r="F225" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G225">
         <v>9746</v>
@@ -17929,6 +17933,9 @@
       <c r="N225" s="1">
         <v>46275</v>
       </c>
+      <c r="O225" t="s">
+        <v>129</v>
+      </c>
       <c r="P225">
         <v>8</v>
       </c>
@@ -17936,72 +17943,78 @@
         <v>2026</v>
       </c>
       <c r="R225">
-        <v>18190457</v>
+        <v>18090250</v>
       </c>
       <c r="S225" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="T225" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="U225" t="s">
         <v>165</v>
       </c>
       <c r="V225" s="1">
-        <v>46274.34198912037</v>
+        <v>46274.48792050926</v>
       </c>
       <c r="W225">
         <v>-1</v>
       </c>
       <c r="X225" t="s">
-        <v>169</v>
+        <v>172</v>
+      </c>
+      <c r="Y225" t="s">
+        <v>245</v>
       </c>
       <c r="AB225">
         <v>0</v>
       </c>
       <c r="AC225" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="AH225" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AI225" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="226" spans="1:35">
       <c r="A226">
-        <v>6627</v>
+        <v>6945</v>
       </c>
       <c r="B226" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C226" t="s">
         <v>50</v>
       </c>
       <c r="D226" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E226" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F226" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G226">
-        <v>1866</v>
+        <v>9746</v>
       </c>
       <c r="H226">
         <v>0</v>
       </c>
       <c r="I226" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J226" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="N226" s="1">
-        <v>46274</v>
+        <v>46275</v>
+      </c>
+      <c r="O226" t="s">
+        <v>129</v>
       </c>
       <c r="P226">
         <v>8</v>
@@ -18010,48 +18023,48 @@
         <v>2026</v>
       </c>
       <c r="R226">
-        <v>17968368</v>
+        <v>18179154</v>
       </c>
       <c r="S226" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="T226" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="U226" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="V226" s="1">
-        <v>46274.36843923611</v>
+        <v>46274.588374375</v>
       </c>
       <c r="W226">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X226" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="Y226" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AB226">
         <v>0</v>
       </c>
       <c r="AC226" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="AH226" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AI226" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="227" spans="1:35">
       <c r="A227">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B227" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C227" t="s">
         <v>50</v>
@@ -18060,25 +18073,25 @@
         <v>51</v>
       </c>
       <c r="E227" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F227" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G227">
-        <v>1867</v>
+        <v>9746</v>
       </c>
       <c r="H227">
         <v>0</v>
       </c>
       <c r="I227" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J227" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="N227" s="1">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="P227">
         <v>8</v>
@@ -18087,45 +18100,45 @@
         <v>2026</v>
       </c>
       <c r="R227">
-        <v>17968379</v>
+        <v>18190457</v>
       </c>
       <c r="S227" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="T227" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="U227" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="V227" s="1">
-        <v>46274.36695243056</v>
+        <v>46274.34198912037</v>
       </c>
       <c r="W227">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X227" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AB227">
         <v>0</v>
       </c>
       <c r="AC227" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="AH227" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AI227" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="228" spans="1:35">
       <c r="A228">
-        <v>5417</v>
+        <v>6627</v>
       </c>
       <c r="B228" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C228" t="s">
         <v>50</v>
@@ -18134,25 +18147,25 @@
         <v>51</v>
       </c>
       <c r="E228" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F228" t="s">
         <v>56</v>
       </c>
       <c r="G228">
-        <v>11303</v>
+        <v>1866</v>
       </c>
       <c r="H228">
         <v>0</v>
       </c>
       <c r="I228" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J228" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="N228" s="1">
-        <v>46279</v>
+        <v>46274</v>
       </c>
       <c r="P228">
         <v>8</v>
@@ -18161,119 +18174,122 @@
         <v>2026</v>
       </c>
       <c r="R228">
-        <v>17399454</v>
+        <v>17968368</v>
       </c>
       <c r="S228" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="T228" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="U228" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V228" s="1">
-        <v>46274.42878043981</v>
+        <v>46274.36843923611</v>
       </c>
       <c r="W228">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="X228" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="Y228" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AB228">
         <v>0</v>
       </c>
       <c r="AC228" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="AH228" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="AI228" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="229" spans="1:35">
       <c r="A229">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B229" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C229" t="s">
         <v>50</v>
       </c>
       <c r="D229" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E229" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F229" t="s">
         <v>56</v>
       </c>
       <c r="G229">
-        <v>5989</v>
+        <v>1867</v>
       </c>
       <c r="H229">
         <v>0</v>
       </c>
       <c r="I229" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J229" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="N229" s="1">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="P229">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q229">
         <v>2026</v>
       </c>
       <c r="R229">
-        <v>17941177</v>
+        <v>17968379</v>
       </c>
       <c r="S229" t="s">
-        <v>154</v>
+        <v>149</v>
+      </c>
+      <c r="T229" t="s">
+        <v>149</v>
       </c>
       <c r="U229" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="V229" s="1">
-        <v>46274.41771849537</v>
+        <v>46274.36695243056</v>
       </c>
       <c r="W229">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X229" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="AB229">
         <v>0</v>
       </c>
       <c r="AC229" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="AH229" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI229" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="230" spans="1:35">
       <c r="A230">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B230" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C230" t="s">
         <v>50</v>
@@ -18288,69 +18304,75 @@
         <v>56</v>
       </c>
       <c r="G230">
-        <v>5989</v>
+        <v>11303</v>
       </c>
       <c r="H230">
         <v>0</v>
       </c>
       <c r="I230" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J230" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="N230" s="1">
-        <v>46273</v>
+        <v>46279</v>
       </c>
       <c r="P230">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q230">
         <v>2026</v>
       </c>
       <c r="R230">
-        <v>17952385</v>
+        <v>17399454</v>
       </c>
       <c r="S230" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+      <c r="T230" t="s">
+        <v>163</v>
       </c>
       <c r="U230" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="V230" s="1">
-        <v>46274.41775447917</v>
+        <v>46274.42878043981</v>
       </c>
       <c r="W230">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="X230" t="s">
-        <v>172</v>
+        <v>173</v>
+      </c>
+      <c r="Y230" t="s">
+        <v>248</v>
       </c>
       <c r="AB230">
         <v>0</v>
       </c>
       <c r="AC230" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AH230" t="s">
         <v>253</v>
       </c>
       <c r="AI230" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="231" spans="1:35">
       <c r="A231">
-        <v>6705</v>
+        <v>6703</v>
       </c>
       <c r="B231" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C231" t="s">
         <v>50</v>
       </c>
       <c r="D231" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E231" t="s">
         <v>54</v>
@@ -18380,7 +18402,7 @@
         <v>2026</v>
       </c>
       <c r="R231">
-        <v>17952569</v>
+        <v>17941177</v>
       </c>
       <c r="S231" t="s">
         <v>154</v>
@@ -18389,13 +18411,13 @@
         <v>164</v>
       </c>
       <c r="V231" s="1">
-        <v>46274.41777533565</v>
+        <v>46274.41771849537</v>
       </c>
       <c r="W231">
         <v>1</v>
       </c>
       <c r="X231" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="AB231">
         <v>0</v>
@@ -18404,30 +18426,30 @@
         <v>154</v>
       </c>
       <c r="AH231" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI231" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="232" spans="1:35">
       <c r="A232">
-        <v>6945</v>
+        <v>6704</v>
       </c>
       <c r="B232" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C232" t="s">
         <v>50</v>
       </c>
       <c r="D232" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E232" t="s">
         <v>54</v>
       </c>
       <c r="F232" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G232">
         <v>5989</v>
@@ -18451,7 +18473,7 @@
         <v>2026</v>
       </c>
       <c r="R232">
-        <v>18164516</v>
+        <v>17952385</v>
       </c>
       <c r="S232" t="s">
         <v>154</v>
@@ -18460,13 +18482,13 @@
         <v>164</v>
       </c>
       <c r="V232" s="1">
-        <v>46274.41799166667</v>
+        <v>46274.41775447917</v>
       </c>
       <c r="W232">
         <v>1</v>
       </c>
       <c r="X232" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AB232">
         <v>0</v>
@@ -18475,30 +18497,30 @@
         <v>154</v>
       </c>
       <c r="AH232" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI232" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="233" spans="1:35">
       <c r="A233">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B233" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C233" t="s">
         <v>50</v>
       </c>
       <c r="D233" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E233" t="s">
         <v>54</v>
       </c>
       <c r="F233" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G233">
         <v>5989</v>
@@ -18522,7 +18544,7 @@
         <v>2026</v>
       </c>
       <c r="R233">
-        <v>18178157</v>
+        <v>17952569</v>
       </c>
       <c r="S233" t="s">
         <v>154</v>
@@ -18531,13 +18553,13 @@
         <v>164</v>
       </c>
       <c r="V233" s="1">
-        <v>46274.41800114583</v>
+        <v>46274.41777533565</v>
       </c>
       <c r="W233">
         <v>1</v>
       </c>
       <c r="X233" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB233">
         <v>0</v>
@@ -18546,45 +18568,45 @@
         <v>154</v>
       </c>
       <c r="AH233" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI233" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="234" spans="1:35">
       <c r="A234">
-        <v>6703</v>
+        <v>6945</v>
       </c>
       <c r="B234" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C234" t="s">
         <v>50</v>
       </c>
       <c r="D234" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E234" t="s">
         <v>54</v>
       </c>
       <c r="F234" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G234">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H234">
         <v>0</v>
       </c>
       <c r="I234" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J234" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N234" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P234">
         <v>9</v>
@@ -18593,42 +18615,42 @@
         <v>2026</v>
       </c>
       <c r="R234">
-        <v>17941187</v>
+        <v>18164516</v>
       </c>
       <c r="S234" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="U234" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="V234" s="1">
-        <v>46274.41772148148</v>
+        <v>46274.41799166667</v>
       </c>
       <c r="W234">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X234" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="AB234">
         <v>0</v>
       </c>
       <c r="AC234" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="AH234" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI234" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="235" spans="1:35">
       <c r="A235">
-        <v>6704</v>
+        <v>6949</v>
       </c>
       <c r="B235" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C235" t="s">
         <v>50</v>
@@ -18640,22 +18662,22 @@
         <v>54</v>
       </c>
       <c r="F235" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G235">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H235">
         <v>0</v>
       </c>
       <c r="I235" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J235" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N235" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P235">
         <v>9</v>
@@ -18664,48 +18686,48 @@
         <v>2026</v>
       </c>
       <c r="R235">
-        <v>17952400</v>
+        <v>18178157</v>
       </c>
       <c r="S235" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="U235" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="V235" s="1">
-        <v>46274.41773631945</v>
+        <v>46274.41800114583</v>
       </c>
       <c r="W235">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X235" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="AB235">
         <v>0</v>
       </c>
       <c r="AC235" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="AH235" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI235" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="236" spans="1:35">
       <c r="A236">
-        <v>6705</v>
+        <v>6703</v>
       </c>
       <c r="B236" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C236" t="s">
         <v>50</v>
       </c>
       <c r="D236" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E236" t="s">
         <v>54</v>
@@ -18735,7 +18757,7 @@
         <v>2026</v>
       </c>
       <c r="R236">
-        <v>17952580</v>
+        <v>17941187</v>
       </c>
       <c r="S236" t="s">
         <v>54</v>
@@ -18744,13 +18766,13 @@
         <v>166</v>
       </c>
       <c r="V236" s="1">
-        <v>46274.41777481481</v>
+        <v>46274.41772148148</v>
       </c>
       <c r="W236">
         <v>0</v>
       </c>
       <c r="X236" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="AB236">
         <v>0</v>
@@ -18759,30 +18781,30 @@
         <v>54</v>
       </c>
       <c r="AH236" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI236" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="237" spans="1:35">
       <c r="A237">
-        <v>6945</v>
+        <v>6704</v>
       </c>
       <c r="B237" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C237" t="s">
         <v>50</v>
       </c>
       <c r="D237" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E237" t="s">
         <v>54</v>
       </c>
       <c r="F237" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G237">
         <v>6215</v>
@@ -18806,7 +18828,7 @@
         <v>2026</v>
       </c>
       <c r="R237">
-        <v>18164523</v>
+        <v>17952400</v>
       </c>
       <c r="S237" t="s">
         <v>54</v>
@@ -18815,13 +18837,13 @@
         <v>166</v>
       </c>
       <c r="V237" s="1">
-        <v>46274.41799332176</v>
+        <v>46274.41773631945</v>
       </c>
       <c r="W237">
         <v>0</v>
       </c>
       <c r="X237" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AB237">
         <v>0</v>
@@ -18830,30 +18852,30 @@
         <v>54</v>
       </c>
       <c r="AH237" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI237" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="238" spans="1:35">
       <c r="A238">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B238" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C238" t="s">
         <v>50</v>
       </c>
       <c r="D238" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E238" t="s">
         <v>54</v>
       </c>
       <c r="F238" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G238">
         <v>6215</v>
@@ -18877,34 +18899,176 @@
         <v>2026</v>
       </c>
       <c r="R238">
-        <v>18178163</v>
+        <v>17952580</v>
       </c>
       <c r="S238" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="U238" t="s">
         <v>166</v>
       </c>
       <c r="V238" s="1">
+        <v>46274.41777481481</v>
+      </c>
+      <c r="W238">
+        <v>0</v>
+      </c>
+      <c r="X238" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB238">
+        <v>0</v>
+      </c>
+      <c r="AC238" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH238" t="s">
+        <v>255</v>
+      </c>
+      <c r="AI238" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="239" spans="1:35">
+      <c r="A239">
+        <v>6945</v>
+      </c>
+      <c r="B239" t="s">
+        <v>39</v>
+      </c>
+      <c r="C239" t="s">
+        <v>50</v>
+      </c>
+      <c r="D239" t="s">
+        <v>52</v>
+      </c>
+      <c r="E239" t="s">
+        <v>54</v>
+      </c>
+      <c r="F239" t="s">
+        <v>57</v>
+      </c>
+      <c r="G239">
+        <v>6215</v>
+      </c>
+      <c r="H239">
+        <v>0</v>
+      </c>
+      <c r="I239" t="s">
+        <v>65</v>
+      </c>
+      <c r="J239" t="s">
+        <v>121</v>
+      </c>
+      <c r="N239" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P239">
+        <v>9</v>
+      </c>
+      <c r="Q239">
+        <v>2026</v>
+      </c>
+      <c r="R239">
+        <v>18164523</v>
+      </c>
+      <c r="S239" t="s">
+        <v>54</v>
+      </c>
+      <c r="U239" t="s">
+        <v>166</v>
+      </c>
+      <c r="V239" s="1">
+        <v>46274.41799332176</v>
+      </c>
+      <c r="W239">
+        <v>0</v>
+      </c>
+      <c r="X239" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB239">
+        <v>0</v>
+      </c>
+      <c r="AC239" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH239" t="s">
+        <v>255</v>
+      </c>
+      <c r="AI239" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="240" spans="1:35">
+      <c r="A240">
+        <v>6949</v>
+      </c>
+      <c r="B240" t="s">
+        <v>37</v>
+      </c>
+      <c r="C240" t="s">
+        <v>50</v>
+      </c>
+      <c r="D240" t="s">
+        <v>51</v>
+      </c>
+      <c r="E240" t="s">
+        <v>54</v>
+      </c>
+      <c r="F240" t="s">
+        <v>57</v>
+      </c>
+      <c r="G240">
+        <v>6215</v>
+      </c>
+      <c r="H240">
+        <v>0</v>
+      </c>
+      <c r="I240" t="s">
+        <v>65</v>
+      </c>
+      <c r="J240" t="s">
+        <v>121</v>
+      </c>
+      <c r="N240" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P240">
+        <v>9</v>
+      </c>
+      <c r="Q240">
+        <v>2026</v>
+      </c>
+      <c r="R240">
+        <v>18178163</v>
+      </c>
+      <c r="S240" t="s">
+        <v>155</v>
+      </c>
+      <c r="U240" t="s">
+        <v>166</v>
+      </c>
+      <c r="V240" s="1">
         <v>46274.41800085648</v>
       </c>
-      <c r="W238">
-        <v>0</v>
-      </c>
-      <c r="X238" t="s">
+      <c r="W240">
+        <v>0</v>
+      </c>
+      <c r="X240" t="s">
         <v>169</v>
       </c>
-      <c r="AB238">
-        <v>0</v>
-      </c>
-      <c r="AC238" t="s">
+      <c r="AB240">
+        <v>0</v>
+      </c>
+      <c r="AC240" t="s">
         <v>155</v>
       </c>
-      <c r="AH238" t="s">
-        <v>253</v>
-      </c>
-      <c r="AI238" t="s">
+      <c r="AH240" t="s">
         <v>255</v>
+      </c>
+      <c r="AI240" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-09 15:48
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3426" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3428" uniqueCount="258">
   <si>
     <t>CodCliente</t>
   </si>
@@ -699,9 +699,6 @@
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1792]. - Data Comentário: 01/09/2026 06:02</t>
   </si>
   <si>
-    <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1867]. - Data Comentário: 01/09/2026 06:01</t>
-  </si>
-  <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1793]. - Data Comentário: 01/09/2026 06:02</t>
   </si>
   <si>
@@ -775,6 +772,10 @@
   </si>
   <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 09/09/2026 08:35</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/09/2026 
+EM PROCESSO - Data Comentário: 08/09/2026 19:19</t>
   </si>
   <si>
     <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 09/09/2026 10:17:37. - Data Comentário: 09/09/2026 10:12</t>
@@ -13201,16 +13202,16 @@
     </row>
     <row r="161" spans="1:35">
       <c r="A161">
-        <v>6548</v>
+        <v>6703</v>
       </c>
       <c r="B161" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C161" t="s">
         <v>50</v>
       </c>
       <c r="D161" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E161" t="s">
         <v>54</v>
@@ -13240,7 +13241,7 @@
         <v>2026</v>
       </c>
       <c r="R161">
-        <v>17222405</v>
+        <v>17941156</v>
       </c>
       <c r="S161" t="s">
         <v>154</v>
@@ -13249,13 +13250,13 @@
         <v>165</v>
       </c>
       <c r="V161" s="1">
-        <v>46266.25161940972</v>
+        <v>46266.25232392361</v>
       </c>
       <c r="W161">
         <v>-1</v>
       </c>
       <c r="X161" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="Y161" t="s">
         <v>223</v>
@@ -13275,16 +13276,16 @@
     </row>
     <row r="162" spans="1:35">
       <c r="A162">
-        <v>6703</v>
+        <v>6779</v>
       </c>
       <c r="B162" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C162" t="s">
         <v>50</v>
       </c>
       <c r="D162" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E162" t="s">
         <v>54</v>
@@ -13314,7 +13315,7 @@
         <v>2026</v>
       </c>
       <c r="R162">
-        <v>17941156</v>
+        <v>18056705</v>
       </c>
       <c r="S162" t="s">
         <v>154</v>
@@ -13323,16 +13324,16 @@
         <v>165</v>
       </c>
       <c r="V162" s="1">
-        <v>46266.25232392361</v>
+        <v>46266.25239591435</v>
       </c>
       <c r="W162">
         <v>-1</v>
       </c>
       <c r="X162" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="Y162" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AB162">
         <v>0</v>
@@ -13349,10 +13350,10 @@
     </row>
     <row r="163" spans="1:35">
       <c r="A163">
-        <v>6779</v>
+        <v>6945</v>
       </c>
       <c r="B163" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C163" t="s">
         <v>50</v>
@@ -13364,7 +13365,7 @@
         <v>54</v>
       </c>
       <c r="F163" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G163">
         <v>951</v>
@@ -13388,7 +13389,7 @@
         <v>2026</v>
       </c>
       <c r="R163">
-        <v>18056705</v>
+        <v>18164501</v>
       </c>
       <c r="S163" t="s">
         <v>154</v>
@@ -13397,13 +13398,13 @@
         <v>165</v>
       </c>
       <c r="V163" s="1">
-        <v>46266.25239591435</v>
+        <v>46266.25258329861</v>
       </c>
       <c r="W163">
         <v>-1</v>
       </c>
       <c r="X163" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="Y163" t="s">
         <v>224</v>
@@ -13423,25 +13424,25 @@
     </row>
     <row r="164" spans="1:35">
       <c r="A164">
-        <v>6945</v>
+        <v>5417</v>
       </c>
       <c r="B164" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C164" t="s">
         <v>50</v>
       </c>
       <c r="D164" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E164" t="s">
         <v>54</v>
       </c>
       <c r="F164" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G164">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="H164">
         <v>0</v>
@@ -13450,10 +13451,10 @@
         <v>64</v>
       </c>
       <c r="J164" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N164" s="1">
-        <v>46275</v>
+        <v>46290</v>
       </c>
       <c r="P164">
         <v>8</v>
@@ -13462,7 +13463,7 @@
         <v>2026</v>
       </c>
       <c r="R164">
-        <v>18164501</v>
+        <v>17398883</v>
       </c>
       <c r="S164" t="s">
         <v>154</v>
@@ -13471,13 +13472,13 @@
         <v>165</v>
       </c>
       <c r="V164" s="1">
-        <v>46266.25258329861</v>
+        <v>46266.25305</v>
       </c>
       <c r="W164">
-        <v>-1</v>
+        <v>-16</v>
       </c>
       <c r="X164" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="Y164" t="s">
         <v>225</v>
@@ -13497,16 +13498,16 @@
     </row>
     <row r="165" spans="1:35">
       <c r="A165">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B165" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C165" t="s">
         <v>50</v>
       </c>
       <c r="D165" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E165" t="s">
         <v>54</v>
@@ -13536,7 +13537,7 @@
         <v>2026</v>
       </c>
       <c r="R165">
-        <v>17398883</v>
+        <v>16962107</v>
       </c>
       <c r="S165" t="s">
         <v>154</v>
@@ -13545,13 +13546,13 @@
         <v>165</v>
       </c>
       <c r="V165" s="1">
-        <v>46266.25305</v>
+        <v>46266.25270034722</v>
       </c>
       <c r="W165">
         <v>-16</v>
       </c>
       <c r="X165" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="Y165" t="s">
         <v>226</v>
@@ -13571,19 +13572,19 @@
     </row>
     <row r="166" spans="1:35">
       <c r="A166">
-        <v>6404</v>
+        <v>6627</v>
       </c>
       <c r="B166" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C166" t="s">
         <v>50</v>
       </c>
       <c r="D166" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E166" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F166" t="s">
         <v>56</v>
@@ -13610,7 +13611,7 @@
         <v>2026</v>
       </c>
       <c r="R166">
-        <v>16962107</v>
+        <v>17042317</v>
       </c>
       <c r="S166" t="s">
         <v>154</v>
@@ -13619,13 +13620,13 @@
         <v>165</v>
       </c>
       <c r="V166" s="1">
-        <v>46266.25270034722</v>
+        <v>46266.25274991898</v>
       </c>
       <c r="W166">
         <v>-16</v>
       </c>
       <c r="X166" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Y166" t="s">
         <v>227</v>
@@ -13645,19 +13646,19 @@
     </row>
     <row r="167" spans="1:35">
       <c r="A167">
-        <v>6627</v>
+        <v>6703</v>
       </c>
       <c r="B167" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C167" t="s">
         <v>50</v>
       </c>
       <c r="D167" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E167" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F167" t="s">
         <v>56</v>
@@ -13684,7 +13685,7 @@
         <v>2026</v>
       </c>
       <c r="R167">
-        <v>17042317</v>
+        <v>17941166</v>
       </c>
       <c r="S167" t="s">
         <v>154</v>
@@ -13693,13 +13694,13 @@
         <v>165</v>
       </c>
       <c r="V167" s="1">
-        <v>46266.25274991898</v>
+        <v>46266.25364633102</v>
       </c>
       <c r="W167">
         <v>-16</v>
       </c>
       <c r="X167" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="Y167" t="s">
         <v>228</v>
@@ -13719,22 +13720,22 @@
     </row>
     <row r="168" spans="1:35">
       <c r="A168">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B168" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C168" t="s">
         <v>50</v>
       </c>
       <c r="D168" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E168" t="s">
         <v>54</v>
       </c>
       <c r="F168" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G168">
         <v>953</v>
@@ -13758,7 +13759,7 @@
         <v>2026</v>
       </c>
       <c r="R168">
-        <v>17941166</v>
+        <v>18178144</v>
       </c>
       <c r="S168" t="s">
         <v>154</v>
@@ -13767,13 +13768,13 @@
         <v>165</v>
       </c>
       <c r="V168" s="1">
-        <v>46266.25364633102</v>
+        <v>46266.25369826389</v>
       </c>
       <c r="W168">
         <v>-16</v>
       </c>
       <c r="X168" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="Y168" t="s">
         <v>229</v>
@@ -13793,10 +13794,10 @@
     </row>
     <row r="169" spans="1:35">
       <c r="A169">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B169" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C169" t="s">
         <v>50</v>
@@ -13808,10 +13809,10 @@
         <v>54</v>
       </c>
       <c r="F169" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G169">
-        <v>953</v>
+        <v>7022</v>
       </c>
       <c r="H169">
         <v>0</v>
@@ -13820,10 +13821,10 @@
         <v>64</v>
       </c>
       <c r="J169" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N169" s="1">
-        <v>46290</v>
+        <v>46283</v>
       </c>
       <c r="P169">
         <v>8</v>
@@ -13832,7 +13833,7 @@
         <v>2026</v>
       </c>
       <c r="R169">
-        <v>18178144</v>
+        <v>17399270</v>
       </c>
       <c r="S169" t="s">
         <v>154</v>
@@ -13841,13 +13842,13 @@
         <v>165</v>
       </c>
       <c r="V169" s="1">
-        <v>46266.25369826389</v>
+        <v>46266.25305112269</v>
       </c>
       <c r="W169">
-        <v>-16</v>
+        <v>-9</v>
       </c>
       <c r="X169" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="Y169" t="s">
         <v>230</v>
@@ -13867,10 +13868,10 @@
     </row>
     <row r="170" spans="1:35">
       <c r="A170">
-        <v>5417</v>
+        <v>6627</v>
       </c>
       <c r="B170" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C170" t="s">
         <v>50</v>
@@ -13879,7 +13880,7 @@
         <v>51</v>
       </c>
       <c r="E170" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F170" t="s">
         <v>56</v>
@@ -13906,7 +13907,7 @@
         <v>2026</v>
       </c>
       <c r="R170">
-        <v>17399270</v>
+        <v>17042505</v>
       </c>
       <c r="S170" t="s">
         <v>154</v>
@@ -13915,13 +13916,13 @@
         <v>165</v>
       </c>
       <c r="V170" s="1">
-        <v>46266.25305112269</v>
+        <v>46266.25275173611</v>
       </c>
       <c r="W170">
         <v>-9</v>
       </c>
       <c r="X170" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="Y170" t="s">
         <v>231</v>
@@ -13941,10 +13942,10 @@
     </row>
     <row r="171" spans="1:35">
       <c r="A171">
-        <v>6627</v>
+        <v>6704</v>
       </c>
       <c r="B171" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C171" t="s">
         <v>50</v>
@@ -13953,7 +13954,7 @@
         <v>51</v>
       </c>
       <c r="E171" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F171" t="s">
         <v>56</v>
@@ -13980,7 +13981,7 @@
         <v>2026</v>
       </c>
       <c r="R171">
-        <v>17042505</v>
+        <v>17952421</v>
       </c>
       <c r="S171" t="s">
         <v>154</v>
@@ -13989,13 +13990,13 @@
         <v>165</v>
       </c>
       <c r="V171" s="1">
-        <v>46266.25275173611</v>
+        <v>46266.25364869213</v>
       </c>
       <c r="W171">
         <v>-9</v>
       </c>
       <c r="X171" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="Y171" t="s">
         <v>232</v>
@@ -14015,10 +14016,10 @@
     </row>
     <row r="172" spans="1:35">
       <c r="A172">
-        <v>6704</v>
+        <v>6949</v>
       </c>
       <c r="B172" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C172" t="s">
         <v>50</v>
@@ -14030,7 +14031,7 @@
         <v>54</v>
       </c>
       <c r="F172" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G172">
         <v>7022</v>
@@ -14054,7 +14055,7 @@
         <v>2026</v>
       </c>
       <c r="R172">
-        <v>17952421</v>
+        <v>18178174</v>
       </c>
       <c r="S172" t="s">
         <v>154</v>
@@ -14063,13 +14064,13 @@
         <v>165</v>
       </c>
       <c r="V172" s="1">
-        <v>46266.25364869213</v>
+        <v>46266.25369988426</v>
       </c>
       <c r="W172">
         <v>-9</v>
       </c>
       <c r="X172" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="Y172" t="s">
         <v>233</v>
@@ -14089,10 +14090,10 @@
     </row>
     <row r="173" spans="1:35">
       <c r="A173">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B173" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C173" t="s">
         <v>50</v>
@@ -14104,10 +14105,10 @@
         <v>54</v>
       </c>
       <c r="F173" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G173">
-        <v>7022</v>
+        <v>9085</v>
       </c>
       <c r="H173">
         <v>0</v>
@@ -14116,34 +14117,37 @@
         <v>64</v>
       </c>
       <c r="J173" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="N173" s="1">
-        <v>46283</v>
+        <v>46268</v>
+      </c>
+      <c r="O173" t="s">
+        <v>126</v>
       </c>
       <c r="P173">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q173">
         <v>2026</v>
       </c>
       <c r="R173">
-        <v>18178174</v>
+        <v>17399353</v>
       </c>
       <c r="S173" t="s">
         <v>154</v>
       </c>
       <c r="U173" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V173" s="1">
-        <v>46266.25369988426</v>
+        <v>46268.62318445602</v>
       </c>
       <c r="W173">
-        <v>-9</v>
+        <v>6</v>
       </c>
       <c r="X173" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="Y173" t="s">
         <v>234</v>
@@ -14155,7 +14159,7 @@
         <v>154</v>
       </c>
       <c r="AH173" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI173" t="s">
         <v>256</v>
@@ -14163,16 +14167,16 @@
     </row>
     <row r="174" spans="1:35">
       <c r="A174">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B174" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C174" t="s">
         <v>50</v>
       </c>
       <c r="D174" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E174" t="s">
         <v>54</v>
@@ -14205,7 +14209,7 @@
         <v>2026</v>
       </c>
       <c r="R174">
-        <v>17399353</v>
+        <v>16962370</v>
       </c>
       <c r="S174" t="s">
         <v>154</v>
@@ -14214,13 +14218,13 @@
         <v>166</v>
       </c>
       <c r="V174" s="1">
-        <v>46268.62318445602</v>
+        <v>46268.62319864584</v>
       </c>
       <c r="W174">
         <v>6</v>
       </c>
       <c r="X174" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="Y174" t="s">
         <v>235</v>
@@ -14240,16 +14244,16 @@
     </row>
     <row r="175" spans="1:35">
       <c r="A175">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B175" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C175" t="s">
         <v>50</v>
       </c>
       <c r="D175" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E175" t="s">
         <v>54</v>
@@ -14282,7 +14286,7 @@
         <v>2026</v>
       </c>
       <c r="R175">
-        <v>16962370</v>
+        <v>16976260</v>
       </c>
       <c r="S175" t="s">
         <v>154</v>
@@ -14291,16 +14295,16 @@
         <v>166</v>
       </c>
       <c r="V175" s="1">
-        <v>46268.62319864584</v>
+        <v>46268.62320026621</v>
       </c>
       <c r="W175">
         <v>6</v>
       </c>
       <c r="X175" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="Y175" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB175">
         <v>0</v>
@@ -14317,10 +14321,10 @@
     </row>
     <row r="176" spans="1:35">
       <c r="A176">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B176" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C176" t="s">
         <v>50</v>
@@ -14359,7 +14363,7 @@
         <v>2026</v>
       </c>
       <c r="R176">
-        <v>16976260</v>
+        <v>17222852</v>
       </c>
       <c r="S176" t="s">
         <v>154</v>
@@ -14368,16 +14372,16 @@
         <v>166</v>
       </c>
       <c r="V176" s="1">
-        <v>46268.62320026621</v>
+        <v>46268.62320177083</v>
       </c>
       <c r="W176">
         <v>6</v>
       </c>
       <c r="X176" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="Y176" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB176">
         <v>0</v>
@@ -14394,10 +14398,10 @@
     </row>
     <row r="177" spans="1:35">
       <c r="A177">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B177" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C177" t="s">
         <v>50</v>
@@ -14406,7 +14410,7 @@
         <v>51</v>
       </c>
       <c r="E177" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F177" t="s">
         <v>56</v>
@@ -14436,7 +14440,7 @@
         <v>2026</v>
       </c>
       <c r="R177">
-        <v>17222852</v>
+        <v>17042569</v>
       </c>
       <c r="S177" t="s">
         <v>154</v>
@@ -14445,16 +14449,16 @@
         <v>166</v>
       </c>
       <c r="V177" s="1">
-        <v>46268.62320177083</v>
+        <v>46268.62320378472</v>
       </c>
       <c r="W177">
         <v>6</v>
       </c>
       <c r="X177" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Y177" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB177">
         <v>0</v>
@@ -14471,16 +14475,16 @@
     </row>
     <row r="178" spans="1:35">
       <c r="A178">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B178" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C178" t="s">
         <v>50</v>
       </c>
       <c r="D178" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E178" t="s">
         <v>55</v>
@@ -14513,7 +14517,7 @@
         <v>2026</v>
       </c>
       <c r="R178">
-        <v>17042569</v>
+        <v>16960062</v>
       </c>
       <c r="S178" t="s">
         <v>154</v>
@@ -14522,7 +14526,7 @@
         <v>166</v>
       </c>
       <c r="V178" s="1">
-        <v>46268.62320378472</v>
+        <v>46268.62320393518</v>
       </c>
       <c r="W178">
         <v>6</v>
@@ -14531,7 +14535,7 @@
         <v>168</v>
       </c>
       <c r="Y178" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB178">
         <v>0</v>
@@ -14548,19 +14552,19 @@
     </row>
     <row r="179" spans="1:35">
       <c r="A179">
-        <v>6628</v>
+        <v>6703</v>
       </c>
       <c r="B179" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C179" t="s">
         <v>50</v>
       </c>
       <c r="D179" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E179" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F179" t="s">
         <v>56</v>
@@ -14590,7 +14594,7 @@
         <v>2026</v>
       </c>
       <c r="R179">
-        <v>16960062</v>
+        <v>17941207</v>
       </c>
       <c r="S179" t="s">
         <v>154</v>
@@ -14599,16 +14603,16 @@
         <v>166</v>
       </c>
       <c r="V179" s="1">
-        <v>46268.62320393518</v>
+        <v>46268.62320697917</v>
       </c>
       <c r="W179">
         <v>6</v>
       </c>
       <c r="X179" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="Y179" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB179">
         <v>0</v>
@@ -14625,16 +14629,16 @@
     </row>
     <row r="180" spans="1:35">
       <c r="A180">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B180" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C180" t="s">
         <v>50</v>
       </c>
       <c r="D180" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E180" t="s">
         <v>54</v>
@@ -14667,7 +14671,7 @@
         <v>2026</v>
       </c>
       <c r="R180">
-        <v>17941207</v>
+        <v>17952433</v>
       </c>
       <c r="S180" t="s">
         <v>154</v>
@@ -14676,16 +14680,16 @@
         <v>166</v>
       </c>
       <c r="V180" s="1">
-        <v>46268.62320697917</v>
+        <v>46268.62320717592</v>
       </c>
       <c r="W180">
         <v>6</v>
       </c>
       <c r="X180" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="Y180" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB180">
         <v>0</v>
@@ -14702,16 +14706,16 @@
     </row>
     <row r="181" spans="1:35">
       <c r="A181">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B181" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C181" t="s">
         <v>50</v>
       </c>
       <c r="D181" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E181" t="s">
         <v>54</v>
@@ -14744,7 +14748,7 @@
         <v>2026</v>
       </c>
       <c r="R181">
-        <v>17952433</v>
+        <v>17952613</v>
       </c>
       <c r="S181" t="s">
         <v>154</v>
@@ -14753,7 +14757,7 @@
         <v>166</v>
       </c>
       <c r="V181" s="1">
-        <v>46268.62320717592</v>
+        <v>46268.62320732639</v>
       </c>
       <c r="W181">
         <v>6</v>
@@ -14762,7 +14766,7 @@
         <v>172</v>
       </c>
       <c r="Y181" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB181">
         <v>0</v>
@@ -14779,10 +14783,10 @@
     </row>
     <row r="182" spans="1:35">
       <c r="A182">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B182" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C182" t="s">
         <v>50</v>
@@ -14821,7 +14825,7 @@
         <v>2026</v>
       </c>
       <c r="R182">
-        <v>17952613</v>
+        <v>18056791</v>
       </c>
       <c r="S182" t="s">
         <v>154</v>
@@ -14830,7 +14834,7 @@
         <v>166</v>
       </c>
       <c r="V182" s="1">
-        <v>46268.62320732639</v>
+        <v>46268.62320810185</v>
       </c>
       <c r="W182">
         <v>6</v>
@@ -14839,7 +14843,7 @@
         <v>172</v>
       </c>
       <c r="Y182" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB182">
         <v>0</v>
@@ -14856,10 +14860,10 @@
     </row>
     <row r="183" spans="1:35">
       <c r="A183">
-        <v>6779</v>
+        <v>6945</v>
       </c>
       <c r="B183" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C183" t="s">
         <v>50</v>
@@ -14871,7 +14875,7 @@
         <v>54</v>
       </c>
       <c r="F183" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G183">
         <v>9085</v>
@@ -14898,7 +14902,7 @@
         <v>2026</v>
       </c>
       <c r="R183">
-        <v>18056791</v>
+        <v>18164544</v>
       </c>
       <c r="S183" t="s">
         <v>154</v>
@@ -14907,16 +14911,16 @@
         <v>166</v>
       </c>
       <c r="V183" s="1">
-        <v>46268.62320810185</v>
+        <v>46268.6232125</v>
       </c>
       <c r="W183">
         <v>6</v>
       </c>
       <c r="X183" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="Y183" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB183">
         <v>0</v>
@@ -14933,16 +14937,16 @@
     </row>
     <row r="184" spans="1:35">
       <c r="A184">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B184" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C184" t="s">
         <v>50</v>
       </c>
       <c r="D184" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E184" t="s">
         <v>54</v>
@@ -14975,7 +14979,7 @@
         <v>2026</v>
       </c>
       <c r="R184">
-        <v>18164544</v>
+        <v>18178181</v>
       </c>
       <c r="S184" t="s">
         <v>154</v>
@@ -14984,16 +14988,16 @@
         <v>166</v>
       </c>
       <c r="V184" s="1">
-        <v>46268.6232125</v>
+        <v>46268.62321412037</v>
       </c>
       <c r="W184">
         <v>6</v>
       </c>
       <c r="X184" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Y184" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB184">
         <v>0</v>
@@ -15010,16 +15014,16 @@
     </row>
     <row r="185" spans="1:35">
       <c r="A185">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B185" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C185" t="s">
         <v>50</v>
       </c>
       <c r="D185" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E185" t="s">
         <v>54</v>
@@ -15052,7 +15056,7 @@
         <v>2026</v>
       </c>
       <c r="R185">
-        <v>18178181</v>
+        <v>18188767</v>
       </c>
       <c r="S185" t="s">
         <v>154</v>
@@ -15061,16 +15065,16 @@
         <v>166</v>
       </c>
       <c r="V185" s="1">
-        <v>46268.62321412037</v>
+        <v>46268.6232128125</v>
       </c>
       <c r="W185">
         <v>6</v>
       </c>
       <c r="X185" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="Y185" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB185">
         <v>0</v>
@@ -15087,10 +15091,10 @@
     </row>
     <row r="186" spans="1:35">
       <c r="A186">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B186" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C186" t="s">
         <v>50</v>
@@ -15129,7 +15133,7 @@
         <v>2026</v>
       </c>
       <c r="R186">
-        <v>18188767</v>
+        <v>18188673</v>
       </c>
       <c r="S186" t="s">
         <v>154</v>
@@ -15138,7 +15142,7 @@
         <v>166</v>
       </c>
       <c r="V186" s="1">
-        <v>46268.6232128125</v>
+        <v>46268.62321296296</v>
       </c>
       <c r="W186">
         <v>6</v>
@@ -15147,7 +15151,7 @@
         <v>171</v>
       </c>
       <c r="Y186" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AB186">
         <v>0</v>
@@ -15164,25 +15168,25 @@
     </row>
     <row r="187" spans="1:35">
       <c r="A187">
-        <v>6963</v>
+        <v>5417</v>
       </c>
       <c r="B187" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C187" t="s">
         <v>50</v>
       </c>
       <c r="D187" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E187" t="s">
         <v>54</v>
       </c>
       <c r="F187" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G187">
-        <v>9085</v>
+        <v>5989</v>
       </c>
       <c r="H187">
         <v>0</v>
@@ -15191,13 +15195,10 @@
         <v>64</v>
       </c>
       <c r="J187" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N187" s="1">
-        <v>46268</v>
-      </c>
-      <c r="O187" t="s">
-        <v>126</v>
+        <v>46273</v>
       </c>
       <c r="P187">
         <v>9</v>
@@ -15206,25 +15207,22 @@
         <v>2026</v>
       </c>
       <c r="R187">
-        <v>18188673</v>
+        <v>17399127</v>
       </c>
       <c r="S187" t="s">
         <v>154</v>
       </c>
       <c r="U187" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="V187" s="1">
-        <v>46268.62321296296</v>
+        <v>46269.41908927084</v>
       </c>
       <c r="W187">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="X187" t="s">
-        <v>171</v>
-      </c>
-      <c r="Y187" t="s">
-        <v>236</v>
+        <v>173</v>
       </c>
       <c r="AB187">
         <v>0</v>
@@ -15241,16 +15239,16 @@
     </row>
     <row r="188" spans="1:35">
       <c r="A188">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B188" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C188" t="s">
         <v>50</v>
       </c>
       <c r="D188" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E188" t="s">
         <v>54</v>
@@ -15280,7 +15278,7 @@
         <v>2026</v>
       </c>
       <c r="R188">
-        <v>17399127</v>
+        <v>16962251</v>
       </c>
       <c r="S188" t="s">
         <v>154</v>
@@ -15289,13 +15287,13 @@
         <v>165</v>
       </c>
       <c r="V188" s="1">
-        <v>46269.41908927084</v>
+        <v>46269.41910457176</v>
       </c>
       <c r="W188">
         <v>1</v>
       </c>
       <c r="X188" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="AB188">
         <v>0</v>
@@ -15312,16 +15310,16 @@
     </row>
     <row r="189" spans="1:35">
       <c r="A189">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B189" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C189" t="s">
         <v>50</v>
       </c>
       <c r="D189" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E189" t="s">
         <v>54</v>
@@ -15351,7 +15349,7 @@
         <v>2026</v>
       </c>
       <c r="R189">
-        <v>16962251</v>
+        <v>16976117</v>
       </c>
       <c r="S189" t="s">
         <v>154</v>
@@ -15360,13 +15358,13 @@
         <v>165</v>
       </c>
       <c r="V189" s="1">
-        <v>46269.41910457176</v>
+        <v>46269.37885223379</v>
       </c>
       <c r="W189">
         <v>1</v>
       </c>
       <c r="X189" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="AB189">
         <v>0</v>
@@ -15383,10 +15381,10 @@
     </row>
     <row r="190" spans="1:35">
       <c r="A190">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B190" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C190" t="s">
         <v>50</v>
@@ -15422,7 +15420,7 @@
         <v>2026</v>
       </c>
       <c r="R190">
-        <v>16976117</v>
+        <v>17222714</v>
       </c>
       <c r="S190" t="s">
         <v>154</v>
@@ -15431,13 +15429,13 @@
         <v>165</v>
       </c>
       <c r="V190" s="1">
-        <v>46269.37885223379</v>
+        <v>46269.3782503125</v>
       </c>
       <c r="W190">
         <v>1</v>
       </c>
       <c r="X190" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="AB190">
         <v>0</v>
@@ -15454,10 +15452,10 @@
     </row>
     <row r="191" spans="1:35">
       <c r="A191">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B191" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C191" t="s">
         <v>50</v>
@@ -15466,7 +15464,7 @@
         <v>51</v>
       </c>
       <c r="E191" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F191" t="s">
         <v>56</v>
@@ -15493,7 +15491,7 @@
         <v>2026</v>
       </c>
       <c r="R191">
-        <v>17222714</v>
+        <v>17042423</v>
       </c>
       <c r="S191" t="s">
         <v>154</v>
@@ -15502,13 +15500,13 @@
         <v>165</v>
       </c>
       <c r="V191" s="1">
-        <v>46269.3782503125</v>
+        <v>46269.41913152778</v>
       </c>
       <c r="W191">
         <v>1</v>
       </c>
       <c r="X191" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB191">
         <v>0</v>
@@ -15525,16 +15523,16 @@
     </row>
     <row r="192" spans="1:35">
       <c r="A192">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B192" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C192" t="s">
         <v>50</v>
       </c>
       <c r="D192" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E192" t="s">
         <v>55</v>
@@ -15564,7 +15562,7 @@
         <v>2026</v>
       </c>
       <c r="R192">
-        <v>17042423</v>
+        <v>16959989</v>
       </c>
       <c r="S192" t="s">
         <v>154</v>
@@ -15573,7 +15571,7 @@
         <v>165</v>
       </c>
       <c r="V192" s="1">
-        <v>46269.41913152778</v>
+        <v>46269.41913775463</v>
       </c>
       <c r="W192">
         <v>1</v>
@@ -15596,37 +15594,37 @@
     </row>
     <row r="193" spans="1:35">
       <c r="A193">
-        <v>6628</v>
+        <v>5417</v>
       </c>
       <c r="B193" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C193" t="s">
         <v>50</v>
       </c>
       <c r="D193" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E193" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F193" t="s">
         <v>56</v>
       </c>
       <c r="G193">
-        <v>5989</v>
+        <v>9087</v>
       </c>
       <c r="H193">
         <v>0</v>
       </c>
       <c r="I193" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J193" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N193" s="1">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="P193">
         <v>9</v>
@@ -15635,28 +15633,28 @@
         <v>2026</v>
       </c>
       <c r="R193">
-        <v>16959989</v>
+        <v>17399373</v>
       </c>
       <c r="S193" t="s">
-        <v>154</v>
+        <v>54</v>
       </c>
       <c r="U193" t="s">
         <v>165</v>
       </c>
       <c r="V193" s="1">
-        <v>46269.41913775463</v>
+        <v>46268.7596207176</v>
       </c>
       <c r="W193">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X193" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="AB193">
         <v>0</v>
       </c>
       <c r="AC193" t="s">
-        <v>154</v>
+        <v>54</v>
       </c>
       <c r="AH193" t="s">
         <v>255</v>
@@ -15667,16 +15665,16 @@
     </row>
     <row r="194" spans="1:35">
       <c r="A194">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B194" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C194" t="s">
         <v>50</v>
       </c>
       <c r="D194" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E194" t="s">
         <v>54</v>
@@ -15706,7 +15704,7 @@
         <v>2026</v>
       </c>
       <c r="R194">
-        <v>17399373</v>
+        <v>16962390</v>
       </c>
       <c r="S194" t="s">
         <v>54</v>
@@ -15715,13 +15713,13 @@
         <v>165</v>
       </c>
       <c r="V194" s="1">
-        <v>46268.7596207176</v>
+        <v>46268.75963109954</v>
       </c>
       <c r="W194">
         <v>5</v>
       </c>
       <c r="X194" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="AB194">
         <v>0</v>
@@ -15738,16 +15736,16 @@
     </row>
     <row r="195" spans="1:35">
       <c r="A195">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B195" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C195" t="s">
         <v>50</v>
       </c>
       <c r="D195" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E195" t="s">
         <v>54</v>
@@ -15777,7 +15775,7 @@
         <v>2026</v>
       </c>
       <c r="R195">
-        <v>16962390</v>
+        <v>16976280</v>
       </c>
       <c r="S195" t="s">
         <v>54</v>
@@ -15786,13 +15784,13 @@
         <v>165</v>
       </c>
       <c r="V195" s="1">
-        <v>46268.75963109954</v>
+        <v>46268.75963225694</v>
       </c>
       <c r="W195">
         <v>5</v>
       </c>
       <c r="X195" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="AB195">
         <v>0</v>
@@ -15809,10 +15807,10 @@
     </row>
     <row r="196" spans="1:35">
       <c r="A196">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B196" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C196" t="s">
         <v>50</v>
@@ -15848,7 +15846,7 @@
         <v>2026</v>
       </c>
       <c r="R196">
-        <v>16976280</v>
+        <v>17222885</v>
       </c>
       <c r="S196" t="s">
         <v>54</v>
@@ -15857,13 +15855,13 @@
         <v>165</v>
       </c>
       <c r="V196" s="1">
-        <v>46268.75963225694</v>
+        <v>46268.75963348379</v>
       </c>
       <c r="W196">
         <v>5</v>
       </c>
       <c r="X196" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="AB196">
         <v>0</v>
@@ -15880,10 +15878,10 @@
     </row>
     <row r="197" spans="1:35">
       <c r="A197">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B197" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C197" t="s">
         <v>50</v>
@@ -15892,7 +15890,7 @@
         <v>51</v>
       </c>
       <c r="E197" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F197" t="s">
         <v>56</v>
@@ -15919,28 +15917,28 @@
         <v>2026</v>
       </c>
       <c r="R197">
-        <v>17222885</v>
+        <v>17042605</v>
       </c>
       <c r="S197" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="U197" t="s">
         <v>165</v>
       </c>
       <c r="V197" s="1">
-        <v>46268.75963348379</v>
+        <v>46268.75963414352</v>
       </c>
       <c r="W197">
         <v>5</v>
       </c>
       <c r="X197" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB197">
         <v>0</v>
       </c>
       <c r="AC197" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="AH197" t="s">
         <v>255</v>
@@ -15951,16 +15949,16 @@
     </row>
     <row r="198" spans="1:35">
       <c r="A198">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B198" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C198" t="s">
         <v>50</v>
       </c>
       <c r="D198" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E198" t="s">
         <v>55</v>
@@ -15990,16 +15988,16 @@
         <v>2026</v>
       </c>
       <c r="R198">
-        <v>17042605</v>
+        <v>16960086</v>
       </c>
       <c r="S198" t="s">
-        <v>155</v>
+        <v>55</v>
       </c>
       <c r="U198" t="s">
         <v>165</v>
       </c>
       <c r="V198" s="1">
-        <v>46268.75963414352</v>
+        <v>46268.62326365741</v>
       </c>
       <c r="W198">
         <v>5</v>
@@ -16011,7 +16009,7 @@
         <v>0</v>
       </c>
       <c r="AC198" t="s">
-        <v>155</v>
+        <v>55</v>
       </c>
       <c r="AH198" t="s">
         <v>255</v>
@@ -16022,19 +16020,19 @@
     </row>
     <row r="199" spans="1:35">
       <c r="A199">
-        <v>6628</v>
+        <v>6703</v>
       </c>
       <c r="B199" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C199" t="s">
         <v>50</v>
       </c>
       <c r="D199" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E199" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F199" t="s">
         <v>56</v>
@@ -16061,28 +16059,28 @@
         <v>2026</v>
       </c>
       <c r="R199">
-        <v>16960086</v>
+        <v>17941227</v>
       </c>
       <c r="S199" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U199" t="s">
         <v>165</v>
       </c>
       <c r="V199" s="1">
-        <v>46268.62326365741</v>
+        <v>46268.75963472222</v>
       </c>
       <c r="W199">
         <v>5</v>
       </c>
       <c r="X199" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="AB199">
         <v>0</v>
       </c>
       <c r="AC199" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AH199" t="s">
         <v>255</v>
@@ -16093,16 +16091,16 @@
     </row>
     <row r="200" spans="1:35">
       <c r="A200">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B200" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C200" t="s">
         <v>50</v>
       </c>
       <c r="D200" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E200" t="s">
         <v>54</v>
@@ -16132,7 +16130,7 @@
         <v>2026</v>
       </c>
       <c r="R200">
-        <v>17941227</v>
+        <v>17952455</v>
       </c>
       <c r="S200" t="s">
         <v>54</v>
@@ -16141,13 +16139,13 @@
         <v>165</v>
       </c>
       <c r="V200" s="1">
-        <v>46268.75963472222</v>
+        <v>46268.75963475694</v>
       </c>
       <c r="W200">
         <v>5</v>
       </c>
       <c r="X200" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AB200">
         <v>0</v>
@@ -16164,16 +16162,16 @@
     </row>
     <row r="201" spans="1:35">
       <c r="A201">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B201" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C201" t="s">
         <v>50</v>
       </c>
       <c r="D201" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E201" t="s">
         <v>54</v>
@@ -16203,7 +16201,7 @@
         <v>2026</v>
       </c>
       <c r="R201">
-        <v>17952455</v>
+        <v>17952635</v>
       </c>
       <c r="S201" t="s">
         <v>54</v>
@@ -16212,7 +16210,7 @@
         <v>165</v>
       </c>
       <c r="V201" s="1">
-        <v>46268.75963475694</v>
+        <v>46268.75963506944</v>
       </c>
       <c r="W201">
         <v>5</v>
@@ -16235,10 +16233,10 @@
     </row>
     <row r="202" spans="1:35">
       <c r="A202">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B202" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C202" t="s">
         <v>50</v>
@@ -16274,16 +16272,16 @@
         <v>2026</v>
       </c>
       <c r="R202">
-        <v>17952635</v>
+        <v>18056811</v>
       </c>
       <c r="S202" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="U202" t="s">
         <v>165</v>
       </c>
       <c r="V202" s="1">
-        <v>46268.75963506944</v>
+        <v>46268.7596360301</v>
       </c>
       <c r="W202">
         <v>5</v>
@@ -16295,7 +16293,7 @@
         <v>0</v>
       </c>
       <c r="AC202" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="AH202" t="s">
         <v>255</v>
@@ -16306,10 +16304,10 @@
     </row>
     <row r="203" spans="1:35">
       <c r="A203">
-        <v>6779</v>
+        <v>6945</v>
       </c>
       <c r="B203" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C203" t="s">
         <v>50</v>
@@ -16321,7 +16319,7 @@
         <v>54</v>
       </c>
       <c r="F203" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G203">
         <v>9087</v>
@@ -16345,28 +16343,28 @@
         <v>2026</v>
       </c>
       <c r="R203">
-        <v>18056811</v>
+        <v>18164558</v>
       </c>
       <c r="S203" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="U203" t="s">
         <v>165</v>
       </c>
       <c r="V203" s="1">
-        <v>46268.7596360301</v>
+        <v>46268.62327121528</v>
       </c>
       <c r="W203">
         <v>5</v>
       </c>
       <c r="X203" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="AB203">
         <v>0</v>
       </c>
       <c r="AC203" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="AH203" t="s">
         <v>255</v>
@@ -16377,16 +16375,16 @@
     </row>
     <row r="204" spans="1:35">
       <c r="A204">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B204" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C204" t="s">
         <v>50</v>
       </c>
       <c r="D204" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E204" t="s">
         <v>54</v>
@@ -16416,28 +16414,28 @@
         <v>2026</v>
       </c>
       <c r="R204">
-        <v>18164558</v>
+        <v>18178193</v>
       </c>
       <c r="S204" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="U204" t="s">
         <v>165</v>
       </c>
       <c r="V204" s="1">
-        <v>46268.62327121528</v>
+        <v>46268.75963931713</v>
       </c>
       <c r="W204">
         <v>5</v>
       </c>
       <c r="X204" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AB204">
         <v>0</v>
       </c>
       <c r="AC204" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="AH204" t="s">
         <v>255</v>
@@ -16448,16 +16446,16 @@
     </row>
     <row r="205" spans="1:35">
       <c r="A205">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B205" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C205" t="s">
         <v>50</v>
       </c>
       <c r="D205" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E205" t="s">
         <v>54</v>
@@ -16487,28 +16485,28 @@
         <v>2026</v>
       </c>
       <c r="R205">
-        <v>18178193</v>
+        <v>18188781</v>
       </c>
       <c r="S205" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="U205" t="s">
         <v>165</v>
       </c>
       <c r="V205" s="1">
-        <v>46268.75963931713</v>
+        <v>46268.75963822917</v>
       </c>
       <c r="W205">
         <v>5</v>
       </c>
       <c r="X205" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="AB205">
         <v>0</v>
       </c>
       <c r="AC205" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="AH205" t="s">
         <v>255</v>
@@ -16519,10 +16517,10 @@
     </row>
     <row r="206" spans="1:35">
       <c r="A206">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B206" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C206" t="s">
         <v>50</v>
@@ -16558,7 +16556,7 @@
         <v>2026</v>
       </c>
       <c r="R206">
-        <v>18188781</v>
+        <v>18188687</v>
       </c>
       <c r="S206" t="s">
         <v>54</v>
@@ -16567,7 +16565,7 @@
         <v>165</v>
       </c>
       <c r="V206" s="1">
-        <v>46268.75963822917</v>
+        <v>46268.75963857639</v>
       </c>
       <c r="W206">
         <v>5</v>
@@ -16590,25 +16588,25 @@
     </row>
     <row r="207" spans="1:35">
       <c r="A207">
-        <v>6963</v>
+        <v>5417</v>
       </c>
       <c r="B207" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C207" t="s">
         <v>50</v>
       </c>
       <c r="D207" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E207" t="s">
         <v>54</v>
       </c>
       <c r="F207" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G207">
-        <v>9087</v>
+        <v>6215</v>
       </c>
       <c r="H207">
         <v>0</v>
@@ -16617,10 +16615,10 @@
         <v>65</v>
       </c>
       <c r="J207" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N207" s="1">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="P207">
         <v>9</v>
@@ -16629,7 +16627,7 @@
         <v>2026</v>
       </c>
       <c r="R207">
-        <v>18188687</v>
+        <v>17399147</v>
       </c>
       <c r="S207" t="s">
         <v>54</v>
@@ -16638,13 +16636,13 @@
         <v>165</v>
       </c>
       <c r="V207" s="1">
-        <v>46268.75963857639</v>
+        <v>46269.41908901621</v>
       </c>
       <c r="W207">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X207" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="AB207">
         <v>0</v>
@@ -16661,16 +16659,16 @@
     </row>
     <row r="208" spans="1:35">
       <c r="A208">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B208" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C208" t="s">
         <v>50</v>
       </c>
       <c r="D208" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E208" t="s">
         <v>54</v>
@@ -16700,7 +16698,7 @@
         <v>2026</v>
       </c>
       <c r="R208">
-        <v>17399147</v>
+        <v>16962265</v>
       </c>
       <c r="S208" t="s">
         <v>54</v>
@@ -16709,13 +16707,13 @@
         <v>165</v>
       </c>
       <c r="V208" s="1">
-        <v>46269.41908901621</v>
+        <v>46269.41910425926</v>
       </c>
       <c r="W208">
         <v>0</v>
       </c>
       <c r="X208" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="AB208">
         <v>0</v>
@@ -16732,16 +16730,16 @@
     </row>
     <row r="209" spans="1:35">
       <c r="A209">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B209" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C209" t="s">
         <v>50</v>
       </c>
       <c r="D209" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E209" t="s">
         <v>54</v>
@@ -16771,7 +16769,7 @@
         <v>2026</v>
       </c>
       <c r="R209">
-        <v>16962265</v>
+        <v>16976127</v>
       </c>
       <c r="S209" t="s">
         <v>54</v>
@@ -16780,13 +16778,13 @@
         <v>165</v>
       </c>
       <c r="V209" s="1">
-        <v>46269.41910425926</v>
+        <v>46269.37890997685</v>
       </c>
       <c r="W209">
         <v>0</v>
       </c>
       <c r="X209" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="AB209">
         <v>0</v>
@@ -16803,10 +16801,10 @@
     </row>
     <row r="210" spans="1:35">
       <c r="A210">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B210" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C210" t="s">
         <v>50</v>
@@ -16842,7 +16840,7 @@
         <v>2026</v>
       </c>
       <c r="R210">
-        <v>16976127</v>
+        <v>17222729</v>
       </c>
       <c r="S210" t="s">
         <v>54</v>
@@ -16851,13 +16849,13 @@
         <v>165</v>
       </c>
       <c r="V210" s="1">
-        <v>46269.37890997685</v>
+        <v>46269.37833320602</v>
       </c>
       <c r="W210">
         <v>0</v>
       </c>
       <c r="X210" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="AB210">
         <v>0</v>
@@ -16874,10 +16872,10 @@
     </row>
     <row r="211" spans="1:35">
       <c r="A211">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B211" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C211" t="s">
         <v>50</v>
@@ -16886,7 +16884,7 @@
         <v>51</v>
       </c>
       <c r="E211" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F211" t="s">
         <v>56</v>
@@ -16913,28 +16911,28 @@
         <v>2026</v>
       </c>
       <c r="R211">
-        <v>17222729</v>
+        <v>17042445</v>
       </c>
       <c r="S211" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="U211" t="s">
         <v>165</v>
       </c>
       <c r="V211" s="1">
-        <v>46269.37833320602</v>
+        <v>46269.41913112268</v>
       </c>
       <c r="W211">
         <v>0</v>
       </c>
       <c r="X211" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB211">
         <v>0</v>
       </c>
       <c r="AC211" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
       <c r="AH211" t="s">
         <v>255</v>
@@ -16945,16 +16943,16 @@
     </row>
     <row r="212" spans="1:35">
       <c r="A212">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B212" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C212" t="s">
         <v>50</v>
       </c>
       <c r="D212" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E212" t="s">
         <v>55</v>
@@ -16984,16 +16982,16 @@
         <v>2026</v>
       </c>
       <c r="R212">
-        <v>17042445</v>
+        <v>16960001</v>
       </c>
       <c r="S212" t="s">
-        <v>155</v>
+        <v>55</v>
       </c>
       <c r="U212" t="s">
         <v>165</v>
       </c>
       <c r="V212" s="1">
-        <v>46269.41913112268</v>
+        <v>46269.41913740741</v>
       </c>
       <c r="W212">
         <v>0</v>
@@ -17005,7 +17003,7 @@
         <v>0</v>
       </c>
       <c r="AC212" t="s">
-        <v>155</v>
+        <v>55</v>
       </c>
       <c r="AH212" t="s">
         <v>255</v>
@@ -17016,25 +17014,25 @@
     </row>
     <row r="213" spans="1:35">
       <c r="A213">
-        <v>6628</v>
+        <v>6404</v>
       </c>
       <c r="B213" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C213" t="s">
         <v>50</v>
       </c>
       <c r="D213" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E213" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F213" t="s">
         <v>56</v>
       </c>
       <c r="G213">
-        <v>6215</v>
+        <v>11001</v>
       </c>
       <c r="H213">
         <v>0</v>
@@ -17043,43 +17041,46 @@
         <v>65</v>
       </c>
       <c r="J213" t="s">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="N213" s="1">
-        <v>46274</v>
+        <v>46259</v>
       </c>
       <c r="P213">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q213">
         <v>2026</v>
       </c>
       <c r="R213">
-        <v>16960001</v>
+        <v>16962453</v>
       </c>
       <c r="S213" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U213" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="V213" s="1">
-        <v>46269.41913740741</v>
+        <v>46267.66131466435</v>
       </c>
       <c r="W213">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="X213" t="s">
-        <v>168</v>
+        <v>177</v>
+      </c>
+      <c r="Y213" t="s">
+        <v>236</v>
       </c>
       <c r="AB213">
         <v>0</v>
       </c>
       <c r="AC213" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AH213" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="AI213" t="s">
         <v>256</v>
@@ -17117,28 +17118,28 @@
         <v>74</v>
       </c>
       <c r="N214" s="1">
-        <v>46259</v>
+        <v>46321</v>
       </c>
       <c r="P214">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q214">
         <v>2026</v>
       </c>
       <c r="R214">
-        <v>16962453</v>
+        <v>16962455</v>
       </c>
       <c r="S214" t="s">
         <v>54</v>
       </c>
       <c r="U214" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="V214" s="1">
-        <v>46267.66131466435</v>
+        <v>46266.21595836805</v>
       </c>
       <c r="W214">
-        <v>15</v>
+        <v>-47</v>
       </c>
       <c r="X214" t="s">
         <v>177</v>
@@ -17161,16 +17162,16 @@
     </row>
     <row r="215" spans="1:35">
       <c r="A215">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B215" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C215" t="s">
         <v>50</v>
       </c>
       <c r="D215" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E215" t="s">
         <v>54</v>
@@ -17179,7 +17180,7 @@
         <v>56</v>
       </c>
       <c r="G215">
-        <v>11001</v>
+        <v>7877</v>
       </c>
       <c r="H215">
         <v>0</v>
@@ -17188,7 +17189,7 @@
         <v>65</v>
       </c>
       <c r="J215" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="N215" s="1">
         <v>46321</v>
@@ -17200,7 +17201,7 @@
         <v>2026</v>
       </c>
       <c r="R215">
-        <v>16962455</v>
+        <v>17399331</v>
       </c>
       <c r="S215" t="s">
         <v>54</v>
@@ -17209,13 +17210,13 @@
         <v>165</v>
       </c>
       <c r="V215" s="1">
-        <v>46266.21595836805</v>
+        <v>46266.21572962963</v>
       </c>
       <c r="W215">
         <v>-47</v>
       </c>
       <c r="X215" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="Y215" t="s">
         <v>238</v>
@@ -17235,10 +17236,10 @@
     </row>
     <row r="216" spans="1:35">
       <c r="A216">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B216" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C216" t="s">
         <v>50</v>
@@ -17253,7 +17254,7 @@
         <v>56</v>
       </c>
       <c r="G216">
-        <v>7877</v>
+        <v>9774</v>
       </c>
       <c r="H216">
         <v>0</v>
@@ -17262,7 +17263,7 @@
         <v>65</v>
       </c>
       <c r="J216" t="s">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="N216" s="1">
         <v>46321</v>
@@ -17274,7 +17275,7 @@
         <v>2026</v>
       </c>
       <c r="R216">
-        <v>17399331</v>
+        <v>16976322</v>
       </c>
       <c r="S216" t="s">
         <v>54</v>
@@ -17283,13 +17284,13 @@
         <v>165</v>
       </c>
       <c r="V216" s="1">
-        <v>46266.21572962963</v>
+        <v>46266.21550011574</v>
       </c>
       <c r="W216">
         <v>-47</v>
       </c>
       <c r="X216" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Y216" t="s">
         <v>239</v>
@@ -17309,10 +17310,10 @@
     </row>
     <row r="217" spans="1:35">
       <c r="A217">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B217" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C217" t="s">
         <v>50</v>
@@ -17327,7 +17328,7 @@
         <v>56</v>
       </c>
       <c r="G217">
-        <v>9774</v>
+        <v>7027</v>
       </c>
       <c r="H217">
         <v>0</v>
@@ -17336,7 +17337,7 @@
         <v>65</v>
       </c>
       <c r="J217" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N217" s="1">
         <v>46321</v>
@@ -17348,7 +17349,7 @@
         <v>2026</v>
       </c>
       <c r="R217">
-        <v>16976322</v>
+        <v>17399291</v>
       </c>
       <c r="S217" t="s">
         <v>54</v>
@@ -17357,16 +17358,13 @@
         <v>165</v>
       </c>
       <c r="V217" s="1">
-        <v>46266.21550011574</v>
+        <v>46266.00006921296</v>
       </c>
       <c r="W217">
         <v>-47</v>
       </c>
       <c r="X217" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y217" t="s">
-        <v>240</v>
+        <v>173</v>
       </c>
       <c r="AB217">
         <v>0</v>
@@ -17383,16 +17381,16 @@
     </row>
     <row r="218" spans="1:35">
       <c r="A218">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B218" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C218" t="s">
         <v>50</v>
       </c>
       <c r="D218" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E218" t="s">
         <v>54</v>
@@ -17422,7 +17420,7 @@
         <v>2026</v>
       </c>
       <c r="R218">
-        <v>17399291</v>
+        <v>16962349</v>
       </c>
       <c r="S218" t="s">
         <v>54</v>
@@ -17437,7 +17435,7 @@
         <v>-47</v>
       </c>
       <c r="X218" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="AB218">
         <v>0</v>
@@ -17454,16 +17452,16 @@
     </row>
     <row r="219" spans="1:35">
       <c r="A219">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B219" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C219" t="s">
         <v>50</v>
       </c>
       <c r="D219" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E219" t="s">
         <v>54</v>
@@ -17484,31 +17482,34 @@
         <v>123</v>
       </c>
       <c r="N219" s="1">
-        <v>46321</v>
+        <v>46260</v>
       </c>
       <c r="P219">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q219">
         <v>2026</v>
       </c>
       <c r="R219">
-        <v>16962349</v>
+        <v>16976236</v>
       </c>
       <c r="S219" t="s">
         <v>54</v>
       </c>
       <c r="U219" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="V219" s="1">
-        <v>46266.00006921296</v>
+        <v>46269.57097615741</v>
       </c>
       <c r="W219">
-        <v>-47</v>
+        <v>14</v>
       </c>
       <c r="X219" t="s">
-        <v>177</v>
+        <v>174</v>
+      </c>
+      <c r="Y219" t="s">
+        <v>240</v>
       </c>
       <c r="AB219">
         <v>0</v>
@@ -17555,35 +17556,32 @@
         <v>123</v>
       </c>
       <c r="N220" s="1">
-        <v>46260</v>
+        <v>46321</v>
       </c>
       <c r="P220">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q220">
         <v>2026</v>
       </c>
       <c r="R220">
-        <v>16976236</v>
+        <v>16976238</v>
       </c>
       <c r="S220" t="s">
         <v>54</v>
       </c>
       <c r="U220" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="V220" s="1">
-        <v>46269.57097615741</v>
+        <v>46266.00006921296</v>
       </c>
       <c r="W220">
-        <v>14</v>
+        <v>-47</v>
       </c>
       <c r="X220" t="s">
         <v>174</v>
       </c>
-      <c r="Y220" t="s">
-        <v>241</v>
-      </c>
       <c r="AB220">
         <v>0</v>
       </c>
@@ -17599,67 +17597,70 @@
     </row>
     <row r="221" spans="1:35">
       <c r="A221">
-        <v>6486</v>
+        <v>6945</v>
       </c>
       <c r="B221" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C221" t="s">
         <v>50</v>
       </c>
       <c r="D221" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E221" t="s">
         <v>54</v>
       </c>
       <c r="F221" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G221">
-        <v>7027</v>
+        <v>11056</v>
       </c>
       <c r="H221">
         <v>0</v>
       </c>
       <c r="I221" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J221" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N221" s="1">
-        <v>46321</v>
+        <v>46269</v>
+      </c>
+      <c r="O221" t="s">
+        <v>127</v>
       </c>
       <c r="P221">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q221">
         <v>2026</v>
       </c>
       <c r="R221">
-        <v>16976238</v>
-      </c>
-      <c r="S221" t="s">
-        <v>54</v>
+        <v>18261776</v>
       </c>
       <c r="U221" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V221" s="1">
-        <v>46266.00006921296</v>
+        <v>46269.46753030093</v>
       </c>
       <c r="W221">
-        <v>-47</v>
+        <v>5</v>
       </c>
       <c r="X221" t="s">
-        <v>174</v>
+        <v>170</v>
+      </c>
+      <c r="Y221" t="s">
+        <v>241</v>
       </c>
       <c r="AB221">
         <v>0</v>
       </c>
       <c r="AC221" t="s">
-        <v>54</v>
+        <v>252</v>
       </c>
       <c r="AH221" t="s">
         <v>253</v>
@@ -17670,40 +17671,40 @@
     </row>
     <row r="222" spans="1:35">
       <c r="A222">
-        <v>6945</v>
+        <v>5417</v>
       </c>
       <c r="B222" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C222" t="s">
         <v>50</v>
       </c>
       <c r="D222" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E222" t="s">
         <v>54</v>
       </c>
       <c r="F222" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G222">
-        <v>11056</v>
+        <v>9746</v>
       </c>
       <c r="H222">
         <v>0</v>
       </c>
       <c r="I222" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="J222" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="N222" s="1">
-        <v>46269</v>
+        <v>46275</v>
       </c>
       <c r="O222" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P222">
         <v>8</v>
@@ -17712,19 +17713,22 @@
         <v>2026</v>
       </c>
       <c r="R222">
-        <v>18261776</v>
+        <v>17399403</v>
+      </c>
+      <c r="S222" t="s">
+        <v>144</v>
       </c>
       <c r="U222" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="V222" s="1">
-        <v>46269.46753030093</v>
+        <v>46274.60593387731</v>
       </c>
       <c r="W222">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="X222" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="Y222" t="s">
         <v>242</v>
@@ -17733,21 +17737,21 @@
         <v>0</v>
       </c>
       <c r="AC222" t="s">
-        <v>252</v>
+        <v>144</v>
       </c>
       <c r="AH222" t="s">
         <v>253</v>
       </c>
       <c r="AI222" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="223" spans="1:35">
       <c r="A223">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B223" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C223" t="s">
         <v>50</v>
@@ -17777,7 +17781,7 @@
         <v>46275</v>
       </c>
       <c r="O223" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="P223">
         <v>8</v>
@@ -17786,22 +17790,25 @@
         <v>2026</v>
       </c>
       <c r="R223">
-        <v>17399403</v>
+        <v>16976300</v>
       </c>
       <c r="S223" t="s">
-        <v>144</v>
+        <v>141</v>
+      </c>
+      <c r="T223" t="s">
+        <v>160</v>
       </c>
       <c r="U223" t="s">
         <v>165</v>
       </c>
       <c r="V223" s="1">
-        <v>46274.60593387731</v>
+        <v>46274.47210818287</v>
       </c>
       <c r="W223">
         <v>-1</v>
       </c>
       <c r="X223" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Y223" t="s">
         <v>243</v>
@@ -17810,7 +17817,7 @@
         <v>0</v>
       </c>
       <c r="AC223" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="AH223" t="s">
         <v>253</v>
@@ -17821,16 +17828,16 @@
     </row>
     <row r="224" spans="1:35">
       <c r="A224">
-        <v>6486</v>
+        <v>6779</v>
       </c>
       <c r="B224" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C224" t="s">
         <v>50</v>
       </c>
       <c r="D224" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E224" t="s">
         <v>54</v>
@@ -17854,7 +17861,7 @@
         <v>46275</v>
       </c>
       <c r="O224" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="P224">
         <v>8</v>
@@ -17863,25 +17870,25 @@
         <v>2026</v>
       </c>
       <c r="R224">
-        <v>16976300</v>
+        <v>18090250</v>
       </c>
       <c r="S224" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="T224" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="U224" t="s">
         <v>165</v>
       </c>
       <c r="V224" s="1">
-        <v>46274.47210818287</v>
+        <v>46274.48792050926</v>
       </c>
       <c r="W224">
         <v>-1</v>
       </c>
       <c r="X224" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="Y224" t="s">
         <v>244</v>
@@ -17890,7 +17897,7 @@
         <v>0</v>
       </c>
       <c r="AC224" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="AH224" t="s">
         <v>253</v>
@@ -17901,10 +17908,10 @@
     </row>
     <row r="225" spans="1:35">
       <c r="A225">
-        <v>6779</v>
+        <v>6945</v>
       </c>
       <c r="B225" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C225" t="s">
         <v>50</v>
@@ -17916,7 +17923,7 @@
         <v>54</v>
       </c>
       <c r="F225" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G225">
         <v>9746</v>
@@ -17943,25 +17950,25 @@
         <v>2026</v>
       </c>
       <c r="R225">
-        <v>18090250</v>
+        <v>18179154</v>
       </c>
       <c r="S225" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="T225" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="U225" t="s">
         <v>165</v>
       </c>
       <c r="V225" s="1">
-        <v>46274.48792050926</v>
+        <v>46274.588374375</v>
       </c>
       <c r="W225">
         <v>-1</v>
       </c>
       <c r="X225" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="Y225" t="s">
         <v>245</v>
@@ -17970,7 +17977,7 @@
         <v>0</v>
       </c>
       <c r="AC225" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="AH225" t="s">
         <v>253</v>
@@ -17981,16 +17988,16 @@
     </row>
     <row r="226" spans="1:35">
       <c r="A226">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B226" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C226" t="s">
         <v>50</v>
       </c>
       <c r="D226" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E226" t="s">
         <v>54</v>
@@ -18013,9 +18020,6 @@
       <c r="N226" s="1">
         <v>46275</v>
       </c>
-      <c r="O226" t="s">
-        <v>129</v>
-      </c>
       <c r="P226">
         <v>8</v>
       </c>
@@ -18023,10 +18027,10 @@
         <v>2026</v>
       </c>
       <c r="R226">
-        <v>18179154</v>
+        <v>18190457</v>
       </c>
       <c r="S226" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T226" t="s">
         <v>161</v>
@@ -18035,22 +18039,19 @@
         <v>165</v>
       </c>
       <c r="V226" s="1">
-        <v>46274.588374375</v>
+        <v>46274.34198912037</v>
       </c>
       <c r="W226">
         <v>-1</v>
       </c>
       <c r="X226" t="s">
-        <v>170</v>
-      </c>
-      <c r="Y226" t="s">
-        <v>246</v>
+        <v>169</v>
       </c>
       <c r="AB226">
         <v>0</v>
       </c>
       <c r="AC226" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AH226" t="s">
         <v>253</v>
@@ -18061,10 +18062,10 @@
     </row>
     <row r="227" spans="1:35">
       <c r="A227">
-        <v>6949</v>
+        <v>6627</v>
       </c>
       <c r="B227" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C227" t="s">
         <v>50</v>
@@ -18073,25 +18074,25 @@
         <v>51</v>
       </c>
       <c r="E227" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F227" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G227">
-        <v>9746</v>
+        <v>1866</v>
       </c>
       <c r="H227">
         <v>0</v>
       </c>
       <c r="I227" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J227" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="N227" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P227">
         <v>8</v>
@@ -18100,34 +18101,37 @@
         <v>2026</v>
       </c>
       <c r="R227">
-        <v>18190457</v>
+        <v>17968368</v>
       </c>
       <c r="S227" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="T227" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="U227" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V227" s="1">
-        <v>46274.34198912037</v>
+        <v>46274.36843923611</v>
       </c>
       <c r="W227">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X227" t="s">
-        <v>169</v>
+        <v>168</v>
+      </c>
+      <c r="Y227" t="s">
+        <v>246</v>
       </c>
       <c r="AB227">
         <v>0</v>
       </c>
       <c r="AC227" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="AH227" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI227" t="s">
         <v>257</v>
@@ -18135,10 +18139,10 @@
     </row>
     <row r="228" spans="1:35">
       <c r="A228">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B228" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C228" t="s">
         <v>50</v>
@@ -18147,13 +18151,13 @@
         <v>51</v>
       </c>
       <c r="E228" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F228" t="s">
         <v>56</v>
       </c>
       <c r="G228">
-        <v>1866</v>
+        <v>1867</v>
       </c>
       <c r="H228">
         <v>0</v>
@@ -18162,11 +18166,14 @@
         <v>62</v>
       </c>
       <c r="J228" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N228" s="1">
         <v>46274</v>
       </c>
+      <c r="O228" t="s">
+        <v>131</v>
+      </c>
       <c r="P228">
         <v>8</v>
       </c>
@@ -18174,10 +18181,10 @@
         <v>2026</v>
       </c>
       <c r="R228">
-        <v>17968368</v>
+        <v>17988543</v>
       </c>
       <c r="S228" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="T228" t="s">
         <v>149</v>
@@ -18186,13 +18193,13 @@
         <v>166</v>
       </c>
       <c r="V228" s="1">
-        <v>46274.36843923611</v>
+        <v>46274.64801501157</v>
       </c>
       <c r="W228">
         <v>0</v>
       </c>
       <c r="X228" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y228" t="s">
         <v>247</v>
@@ -18201,7 +18208,7 @@
         <v>0</v>
       </c>
       <c r="AC228" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AH228" t="s">
         <v>254</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-09 16:50
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3428" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3443" uniqueCount="259">
   <si>
     <t>CodCliente</t>
   </si>
@@ -772,6 +772,9 @@
   </si>
   <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 09/09/2026 08:35</t>
+  </si>
+  <si>
+    <t>Imposto enviado via SCI Report - Data Comentário: 09/09/2026 15:41</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/09/2026 
@@ -1141,7 +1144,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI240"/>
+  <dimension ref="A1:AI241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1322,10 +1325,10 @@
         <v>132</v>
       </c>
       <c r="AH2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1399,10 +1402,10 @@
         <v>133</v>
       </c>
       <c r="AH3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1476,10 +1479,10 @@
         <v>132</v>
       </c>
       <c r="AH4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1550,10 +1553,10 @@
         <v>132</v>
       </c>
       <c r="AH5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1624,10 +1627,10 @@
         <v>133</v>
       </c>
       <c r="AH6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1698,10 +1701,10 @@
         <v>133</v>
       </c>
       <c r="AH7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI7" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1772,10 +1775,10 @@
         <v>134</v>
       </c>
       <c r="AH8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1846,10 +1849,10 @@
         <v>132</v>
       </c>
       <c r="AH9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1920,10 +1923,10 @@
         <v>135</v>
       </c>
       <c r="AH10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1994,10 +1997,10 @@
         <v>135</v>
       </c>
       <c r="AH11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2068,10 +2071,10 @@
         <v>136</v>
       </c>
       <c r="AH12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2139,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="AC13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AH13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2213,13 +2216,13 @@
         <v>0</v>
       </c>
       <c r="AC14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AH14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2287,10 +2290,10 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2352,10 +2355,10 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI16" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2423,10 +2426,10 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI17" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2500,10 +2503,10 @@
         <v>138</v>
       </c>
       <c r="AH18" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2577,10 +2580,10 @@
         <v>137</v>
       </c>
       <c r="AH19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2654,10 +2657,10 @@
         <v>138</v>
       </c>
       <c r="AH20" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI20" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2731,10 +2734,10 @@
         <v>136</v>
       </c>
       <c r="AH21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI21" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2805,10 +2808,10 @@
         <v>139</v>
       </c>
       <c r="AH22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2879,10 +2882,10 @@
         <v>136</v>
       </c>
       <c r="AH23" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI23" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2953,10 +2956,10 @@
         <v>136</v>
       </c>
       <c r="AH24" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI24" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3027,10 +3030,10 @@
         <v>136</v>
       </c>
       <c r="AH25" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI25" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3101,10 +3104,10 @@
         <v>137</v>
       </c>
       <c r="AH26" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI26" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3175,10 +3178,10 @@
         <v>136</v>
       </c>
       <c r="AH27" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI27" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3249,10 +3252,10 @@
         <v>136</v>
       </c>
       <c r="AH28" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI28" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3323,10 +3326,10 @@
         <v>136</v>
       </c>
       <c r="AH29" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI29" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3397,10 +3400,10 @@
         <v>140</v>
       </c>
       <c r="AH30" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI30" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3477,10 +3480,10 @@
         <v>141</v>
       </c>
       <c r="AH31" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI31" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3551,10 +3554,10 @@
         <v>142</v>
       </c>
       <c r="AH32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3631,10 +3634,10 @@
         <v>143</v>
       </c>
       <c r="AH33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3708,10 +3711,10 @@
         <v>144</v>
       </c>
       <c r="AH34" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI34" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3785,13 +3788,13 @@
         <v>0</v>
       </c>
       <c r="AC35" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AH35" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI35" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3868,10 +3871,10 @@
         <v>146</v>
       </c>
       <c r="AH36" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI36" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3948,10 +3951,10 @@
         <v>140</v>
       </c>
       <c r="AH37" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI37" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4025,10 +4028,10 @@
         <v>162</v>
       </c>
       <c r="AH38" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI38" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4105,10 +4108,10 @@
         <v>141</v>
       </c>
       <c r="AH39" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI39" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4185,10 +4188,10 @@
         <v>141</v>
       </c>
       <c r="AH40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4265,10 +4268,10 @@
         <v>141</v>
       </c>
       <c r="AH41" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4345,10 +4348,10 @@
         <v>140</v>
       </c>
       <c r="AH42" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI42" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4425,10 +4428,10 @@
         <v>147</v>
       </c>
       <c r="AH43" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI43" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4505,10 +4508,10 @@
         <v>142</v>
       </c>
       <c r="AH44" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4585,10 +4588,10 @@
         <v>143</v>
       </c>
       <c r="AH45" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI45" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4656,10 +4659,10 @@
         <v>144</v>
       </c>
       <c r="AH46" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI46" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4730,10 +4733,10 @@
         <v>141</v>
       </c>
       <c r="AH47" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI47" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4804,10 +4807,10 @@
         <v>141</v>
       </c>
       <c r="AH48" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI48" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4878,10 +4881,10 @@
         <v>141</v>
       </c>
       <c r="AH49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI49" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4952,10 +4955,10 @@
         <v>140</v>
       </c>
       <c r="AH50" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI50" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5026,10 +5029,10 @@
         <v>147</v>
       </c>
       <c r="AH51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI51" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5106,10 +5109,10 @@
         <v>142</v>
       </c>
       <c r="AH52" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI52" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5180,10 +5183,10 @@
         <v>143</v>
       </c>
       <c r="AH53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI53" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5260,10 +5263,10 @@
         <v>141</v>
       </c>
       <c r="AH54" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI54" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5340,10 +5343,10 @@
         <v>141</v>
       </c>
       <c r="AH55" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI55" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5420,10 +5423,10 @@
         <v>141</v>
       </c>
       <c r="AH56" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI56" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5500,10 +5503,10 @@
         <v>140</v>
       </c>
       <c r="AH57" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI57" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5577,10 +5580,10 @@
         <v>144</v>
       </c>
       <c r="AH58" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI58" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5654,13 +5657,13 @@
         <v>0</v>
       </c>
       <c r="AC59" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AH59" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI59" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5737,10 +5740,10 @@
         <v>141</v>
       </c>
       <c r="AH60" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI60" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5817,10 +5820,10 @@
         <v>141</v>
       </c>
       <c r="AH61" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI61" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5897,10 +5900,10 @@
         <v>141</v>
       </c>
       <c r="AH62" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI62" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -5977,10 +5980,10 @@
         <v>140</v>
       </c>
       <c r="AH63" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI63" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6057,10 +6060,10 @@
         <v>147</v>
       </c>
       <c r="AH64" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI64" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6137,10 +6140,10 @@
         <v>142</v>
       </c>
       <c r="AH65" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI65" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6217,10 +6220,10 @@
         <v>143</v>
       </c>
       <c r="AH66" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI66" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6297,10 +6300,10 @@
         <v>141</v>
       </c>
       <c r="AH67" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI67" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6368,10 +6371,10 @@
         <v>144</v>
       </c>
       <c r="AH68" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI68" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6439,13 +6442,13 @@
         <v>0</v>
       </c>
       <c r="AC69" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AH69" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI69" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6516,10 +6519,10 @@
         <v>141</v>
       </c>
       <c r="AH70" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI70" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6590,10 +6593,10 @@
         <v>141</v>
       </c>
       <c r="AH71" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI71" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6664,10 +6667,10 @@
         <v>141</v>
       </c>
       <c r="AH72" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI72" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6738,10 +6741,10 @@
         <v>140</v>
       </c>
       <c r="AH73" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI73" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6812,10 +6815,10 @@
         <v>147</v>
       </c>
       <c r="AH74" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI74" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6886,10 +6889,10 @@
         <v>142</v>
       </c>
       <c r="AH75" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI75" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6960,10 +6963,10 @@
         <v>143</v>
       </c>
       <c r="AH76" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI76" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7034,10 +7037,10 @@
         <v>143</v>
       </c>
       <c r="AH77" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI77" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7108,10 +7111,10 @@
         <v>143</v>
       </c>
       <c r="AH78" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI78" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7182,10 +7185,10 @@
         <v>143</v>
       </c>
       <c r="AH79" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI79" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7256,10 +7259,10 @@
         <v>149</v>
       </c>
       <c r="AH80" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI80" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7330,10 +7333,10 @@
         <v>149</v>
       </c>
       <c r="AH81" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI81" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7404,10 +7407,10 @@
         <v>150</v>
       </c>
       <c r="AH82" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI82" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7478,10 +7481,10 @@
         <v>149</v>
       </c>
       <c r="AH83" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI83" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7552,10 +7555,10 @@
         <v>149</v>
       </c>
       <c r="AH84" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI84" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7629,10 +7632,10 @@
         <v>149</v>
       </c>
       <c r="AH85" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI85" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7703,10 +7706,10 @@
         <v>150</v>
       </c>
       <c r="AH86" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI86" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7777,10 +7780,10 @@
         <v>149</v>
       </c>
       <c r="AH87" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI87" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7851,10 +7854,10 @@
         <v>149</v>
       </c>
       <c r="AH88" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI88" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7925,10 +7928,10 @@
         <v>149</v>
       </c>
       <c r="AH89" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI89" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -7996,10 +7999,10 @@
         <v>149</v>
       </c>
       <c r="AH90" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI90" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8070,10 +8073,10 @@
         <v>150</v>
       </c>
       <c r="AH91" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI91" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8144,10 +8147,10 @@
         <v>149</v>
       </c>
       <c r="AH92" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI92" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8218,10 +8221,10 @@
         <v>149</v>
       </c>
       <c r="AH93" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI93" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8292,10 +8295,10 @@
         <v>149</v>
       </c>
       <c r="AH94" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI94" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8363,10 +8366,10 @@
         <v>149</v>
       </c>
       <c r="AH95" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI95" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8437,10 +8440,10 @@
         <v>150</v>
       </c>
       <c r="AH96" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI96" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8511,10 +8514,10 @@
         <v>149</v>
       </c>
       <c r="AH97" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI97" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8585,10 +8588,10 @@
         <v>149</v>
       </c>
       <c r="AH98" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI98" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8659,10 +8662,10 @@
         <v>150</v>
       </c>
       <c r="AH99" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI99" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8739,10 +8742,10 @@
         <v>149</v>
       </c>
       <c r="AH100" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI100" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8810,10 +8813,10 @@
         <v>149</v>
       </c>
       <c r="AH101" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI101" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8884,10 +8887,10 @@
         <v>149</v>
       </c>
       <c r="AH102" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI102" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8958,10 +8961,10 @@
         <v>149</v>
       </c>
       <c r="AH103" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI103" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9032,10 +9035,10 @@
         <v>149</v>
       </c>
       <c r="AH104" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI104" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9103,10 +9106,10 @@
         <v>149</v>
       </c>
       <c r="AH105" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI105" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9177,10 +9180,10 @@
         <v>150</v>
       </c>
       <c r="AH106" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI106" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9251,10 +9254,10 @@
         <v>149</v>
       </c>
       <c r="AH107" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI107" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9325,10 +9328,10 @@
         <v>149</v>
       </c>
       <c r="AH108" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI108" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9396,10 +9399,10 @@
         <v>149</v>
       </c>
       <c r="AH109" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI109" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9470,10 +9473,10 @@
         <v>150</v>
       </c>
       <c r="AH110" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI110" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9541,10 +9544,10 @@
         <v>151</v>
       </c>
       <c r="AH111" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI111" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9615,10 +9618,10 @@
         <v>150</v>
       </c>
       <c r="AH112" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI112" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9689,10 +9692,10 @@
         <v>148</v>
       </c>
       <c r="AH113" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI113" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9760,10 +9763,10 @@
         <v>151</v>
       </c>
       <c r="AH114" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI114" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9834,10 +9837,10 @@
         <v>150</v>
       </c>
       <c r="AH115" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI115" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9908,10 +9911,10 @@
         <v>149</v>
       </c>
       <c r="AH116" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI116" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -9982,10 +9985,10 @@
         <v>149</v>
       </c>
       <c r="AH117" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI117" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10056,10 +10059,10 @@
         <v>149</v>
       </c>
       <c r="AH118" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI118" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10127,10 +10130,10 @@
         <v>149</v>
       </c>
       <c r="AH119" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI119" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10201,10 +10204,10 @@
         <v>150</v>
       </c>
       <c r="AH120" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI120" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10275,10 +10278,10 @@
         <v>149</v>
       </c>
       <c r="AH121" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI121" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10349,10 +10352,10 @@
         <v>149</v>
       </c>
       <c r="AH122" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI122" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10423,10 +10426,10 @@
         <v>149</v>
       </c>
       <c r="AH123" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI123" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10494,10 +10497,10 @@
         <v>149</v>
       </c>
       <c r="AH124" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI124" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10568,10 +10571,10 @@
         <v>150</v>
       </c>
       <c r="AH125" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI125" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10648,10 +10651,10 @@
         <v>150</v>
       </c>
       <c r="AH126" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI126" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10728,10 +10731,10 @@
         <v>150</v>
       </c>
       <c r="AH127" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI127" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10802,10 +10805,10 @@
         <v>153</v>
       </c>
       <c r="AH128" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI128" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10876,10 +10879,10 @@
         <v>153</v>
       </c>
       <c r="AH129" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI129" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -10956,10 +10959,10 @@
         <v>153</v>
       </c>
       <c r="AH130" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI130" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11030,10 +11033,10 @@
         <v>153</v>
       </c>
       <c r="AH131" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI131" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11104,10 +11107,10 @@
         <v>153</v>
       </c>
       <c r="AH132" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI132" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11178,10 +11181,10 @@
         <v>153</v>
       </c>
       <c r="AH133" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI133" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11252,10 +11255,10 @@
         <v>153</v>
       </c>
       <c r="AH134" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI134" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11332,10 +11335,10 @@
         <v>153</v>
       </c>
       <c r="AH135" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI135" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11406,10 +11409,10 @@
         <v>153</v>
       </c>
       <c r="AH136" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI136" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11480,10 +11483,10 @@
         <v>153</v>
       </c>
       <c r="AH137" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI137" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11554,10 +11557,10 @@
         <v>153</v>
       </c>
       <c r="AH138" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI138" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11634,10 +11637,10 @@
         <v>153</v>
       </c>
       <c r="AH139" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI139" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11708,10 +11711,10 @@
         <v>153</v>
       </c>
       <c r="AH140" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI140" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11782,10 +11785,10 @@
         <v>153</v>
       </c>
       <c r="AH141" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI141" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11856,10 +11859,10 @@
         <v>153</v>
       </c>
       <c r="AH142" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI142" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11930,10 +11933,10 @@
         <v>153</v>
       </c>
       <c r="AH143" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI143" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -12004,10 +12007,10 @@
         <v>153</v>
       </c>
       <c r="AH144" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI144" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12078,10 +12081,10 @@
         <v>153</v>
       </c>
       <c r="AH145" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI145" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12152,10 +12155,10 @@
         <v>153</v>
       </c>
       <c r="AH146" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI146" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12226,10 +12229,10 @@
         <v>153</v>
       </c>
       <c r="AH147" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI147" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12300,10 +12303,10 @@
         <v>153</v>
       </c>
       <c r="AH148" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI148" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12374,10 +12377,10 @@
         <v>153</v>
       </c>
       <c r="AH149" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI149" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12454,10 +12457,10 @@
         <v>153</v>
       </c>
       <c r="AH150" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI150" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12528,10 +12531,10 @@
         <v>153</v>
       </c>
       <c r="AH151" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI151" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12602,10 +12605,10 @@
         <v>153</v>
       </c>
       <c r="AH152" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI152" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12676,10 +12679,10 @@
         <v>153</v>
       </c>
       <c r="AH153" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI153" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12750,10 +12753,10 @@
         <v>154</v>
       </c>
       <c r="AH154" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI154" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12824,10 +12827,10 @@
         <v>154</v>
       </c>
       <c r="AH155" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI155" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12898,10 +12901,10 @@
         <v>154</v>
       </c>
       <c r="AH156" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI156" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -12972,10 +12975,10 @@
         <v>154</v>
       </c>
       <c r="AH157" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI157" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13046,10 +13049,10 @@
         <v>154</v>
       </c>
       <c r="AH158" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI158" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13120,10 +13123,10 @@
         <v>154</v>
       </c>
       <c r="AH159" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI159" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13194,10 +13197,10 @@
         <v>154</v>
       </c>
       <c r="AH160" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI160" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13268,10 +13271,10 @@
         <v>154</v>
       </c>
       <c r="AH161" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI161" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13342,10 +13345,10 @@
         <v>154</v>
       </c>
       <c r="AH162" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI162" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13416,10 +13419,10 @@
         <v>154</v>
       </c>
       <c r="AH163" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI163" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13490,10 +13493,10 @@
         <v>154</v>
       </c>
       <c r="AH164" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI164" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13564,10 +13567,10 @@
         <v>154</v>
       </c>
       <c r="AH165" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI165" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13638,10 +13641,10 @@
         <v>154</v>
       </c>
       <c r="AH166" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI166" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13712,10 +13715,10 @@
         <v>154</v>
       </c>
       <c r="AH167" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI167" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13786,10 +13789,10 @@
         <v>154</v>
       </c>
       <c r="AH168" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI168" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13860,10 +13863,10 @@
         <v>154</v>
       </c>
       <c r="AH169" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI169" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13934,10 +13937,10 @@
         <v>154</v>
       </c>
       <c r="AH170" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI170" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14008,10 +14011,10 @@
         <v>154</v>
       </c>
       <c r="AH171" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI171" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14082,10 +14085,10 @@
         <v>154</v>
       </c>
       <c r="AH172" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI172" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14159,10 +14162,10 @@
         <v>154</v>
       </c>
       <c r="AH173" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI173" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14236,10 +14239,10 @@
         <v>154</v>
       </c>
       <c r="AH174" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI174" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14313,10 +14316,10 @@
         <v>154</v>
       </c>
       <c r="AH175" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI175" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14390,10 +14393,10 @@
         <v>154</v>
       </c>
       <c r="AH176" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI176" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14467,10 +14470,10 @@
         <v>154</v>
       </c>
       <c r="AH177" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI177" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14544,10 +14547,10 @@
         <v>154</v>
       </c>
       <c r="AH178" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI178" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14621,10 +14624,10 @@
         <v>154</v>
       </c>
       <c r="AH179" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI179" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14698,10 +14701,10 @@
         <v>154</v>
       </c>
       <c r="AH180" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI180" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14775,10 +14778,10 @@
         <v>154</v>
       </c>
       <c r="AH181" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI181" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14852,10 +14855,10 @@
         <v>154</v>
       </c>
       <c r="AH182" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI182" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14929,10 +14932,10 @@
         <v>154</v>
       </c>
       <c r="AH183" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI183" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -15006,10 +15009,10 @@
         <v>154</v>
       </c>
       <c r="AH184" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI184" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15083,10 +15086,10 @@
         <v>154</v>
       </c>
       <c r="AH185" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI185" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15160,10 +15163,10 @@
         <v>154</v>
       </c>
       <c r="AH186" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI186" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15231,10 +15234,10 @@
         <v>154</v>
       </c>
       <c r="AH187" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI187" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15302,10 +15305,10 @@
         <v>154</v>
       </c>
       <c r="AH188" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI188" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15373,10 +15376,10 @@
         <v>154</v>
       </c>
       <c r="AH189" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI189" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15444,10 +15447,10 @@
         <v>154</v>
       </c>
       <c r="AH190" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI190" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15515,10 +15518,10 @@
         <v>154</v>
       </c>
       <c r="AH191" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI191" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15586,10 +15589,10 @@
         <v>154</v>
       </c>
       <c r="AH192" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI192" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15657,10 +15660,10 @@
         <v>54</v>
       </c>
       <c r="AH193" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI193" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15728,10 +15731,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI194" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15799,10 +15802,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI195" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15870,10 +15873,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI196" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15941,10 +15944,10 @@
         <v>155</v>
       </c>
       <c r="AH197" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI197" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -16012,10 +16015,10 @@
         <v>55</v>
       </c>
       <c r="AH198" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI198" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16083,10 +16086,10 @@
         <v>54</v>
       </c>
       <c r="AH199" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI199" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16154,10 +16157,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI200" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16225,10 +16228,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI201" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16296,10 +16299,10 @@
         <v>155</v>
       </c>
       <c r="AH202" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI202" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16367,10 +16370,10 @@
         <v>54</v>
       </c>
       <c r="AH203" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI203" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16438,10 +16441,10 @@
         <v>155</v>
       </c>
       <c r="AH204" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI204" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16509,10 +16512,10 @@
         <v>54</v>
       </c>
       <c r="AH205" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI205" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16580,10 +16583,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI206" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16651,10 +16654,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI207" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16722,10 +16725,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI208" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16793,10 +16796,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI209" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16864,10 +16867,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI210" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -16935,10 +16938,10 @@
         <v>155</v>
       </c>
       <c r="AH211" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI211" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -17006,10 +17009,10 @@
         <v>55</v>
       </c>
       <c r="AH212" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI212" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17080,10 +17083,10 @@
         <v>54</v>
       </c>
       <c r="AH213" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI213" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17154,10 +17157,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI214" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17228,10 +17231,10 @@
         <v>54</v>
       </c>
       <c r="AH215" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI215" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17302,10 +17305,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI216" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17373,10 +17376,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI217" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17444,10 +17447,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI218" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17518,10 +17521,10 @@
         <v>54</v>
       </c>
       <c r="AH219" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI219" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17589,10 +17592,10 @@
         <v>54</v>
       </c>
       <c r="AH220" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI220" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17660,13 +17663,13 @@
         <v>0</v>
       </c>
       <c r="AC221" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AH221" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI221" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17740,10 +17743,10 @@
         <v>144</v>
       </c>
       <c r="AH222" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI222" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="223" spans="1:35">
@@ -17820,10 +17823,10 @@
         <v>141</v>
       </c>
       <c r="AH223" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI223" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="224" spans="1:35">
@@ -17900,10 +17903,10 @@
         <v>147</v>
       </c>
       <c r="AH224" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI224" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="225" spans="1:35">
@@ -17980,10 +17983,10 @@
         <v>142</v>
       </c>
       <c r="AH225" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI225" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="226" spans="1:35">
@@ -18054,10 +18057,10 @@
         <v>143</v>
       </c>
       <c r="AH226" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AI226" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="227" spans="1:35">
@@ -18131,33 +18134,33 @@
         <v>149</v>
       </c>
       <c r="AH227" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI227" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="228" spans="1:35">
       <c r="A228">
-        <v>6548</v>
+        <v>6962</v>
       </c>
       <c r="B228" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C228" t="s">
         <v>50</v>
       </c>
       <c r="D228" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E228" t="s">
         <v>54</v>
       </c>
       <c r="F228" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G228">
-        <v>1867</v>
+        <v>1866</v>
       </c>
       <c r="H228">
         <v>0</v>
@@ -18166,14 +18169,11 @@
         <v>62</v>
       </c>
       <c r="J228" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N228" s="1">
         <v>46274</v>
       </c>
-      <c r="O228" t="s">
-        <v>131</v>
-      </c>
       <c r="P228">
         <v>8</v>
       </c>
@@ -18181,10 +18181,10 @@
         <v>2026</v>
       </c>
       <c r="R228">
-        <v>17988543</v>
+        <v>18186946</v>
       </c>
       <c r="S228" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="T228" t="s">
         <v>149</v>
@@ -18193,13 +18193,13 @@
         <v>166</v>
       </c>
       <c r="V228" s="1">
-        <v>46274.64801501157</v>
+        <v>46274.66470667824</v>
       </c>
       <c r="W228">
         <v>0</v>
       </c>
       <c r="X228" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="Y228" t="s">
         <v>247</v>
@@ -18208,21 +18208,21 @@
         <v>0</v>
       </c>
       <c r="AC228" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="AH228" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI228" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="229" spans="1:35">
       <c r="A229">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B229" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C229" t="s">
         <v>50</v>
@@ -18231,7 +18231,7 @@
         <v>51</v>
       </c>
       <c r="E229" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F229" t="s">
         <v>56</v>
@@ -18251,6 +18251,9 @@
       <c r="N229" s="1">
         <v>46274</v>
       </c>
+      <c r="O229" t="s">
+        <v>131</v>
+      </c>
       <c r="P229">
         <v>8</v>
       </c>
@@ -18258,10 +18261,10 @@
         <v>2026</v>
       </c>
       <c r="R229">
-        <v>17968379</v>
+        <v>17988543</v>
       </c>
       <c r="S229" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="T229" t="s">
         <v>149</v>
@@ -18270,33 +18273,36 @@
         <v>166</v>
       </c>
       <c r="V229" s="1">
-        <v>46274.36695243056</v>
+        <v>46274.64801501157</v>
       </c>
       <c r="W229">
         <v>0</v>
       </c>
       <c r="X229" t="s">
-        <v>168</v>
+        <v>167</v>
+      </c>
+      <c r="Y229" t="s">
+        <v>248</v>
       </c>
       <c r="AB229">
         <v>0</v>
       </c>
       <c r="AC229" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AH229" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AI229" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="230" spans="1:35">
       <c r="A230">
-        <v>5417</v>
+        <v>6627</v>
       </c>
       <c r="B230" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C230" t="s">
         <v>50</v>
@@ -18305,25 +18311,25 @@
         <v>51</v>
       </c>
       <c r="E230" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F230" t="s">
         <v>56</v>
       </c>
       <c r="G230">
-        <v>11303</v>
+        <v>1867</v>
       </c>
       <c r="H230">
         <v>0</v>
       </c>
       <c r="I230" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J230" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="N230" s="1">
-        <v>46279</v>
+        <v>46274</v>
       </c>
       <c r="P230">
         <v>8</v>
@@ -18332,54 +18338,51 @@
         <v>2026</v>
       </c>
       <c r="R230">
-        <v>17399454</v>
+        <v>17968379</v>
       </c>
       <c r="S230" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="T230" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="U230" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="V230" s="1">
-        <v>46274.42878043981</v>
+        <v>46274.36695243056</v>
       </c>
       <c r="W230">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="X230" t="s">
-        <v>173</v>
-      </c>
-      <c r="Y230" t="s">
-        <v>248</v>
+        <v>168</v>
       </c>
       <c r="AB230">
         <v>0</v>
       </c>
       <c r="AC230" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="AH230" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AI230" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="231" spans="1:35">
       <c r="A231">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B231" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C231" t="s">
         <v>50</v>
       </c>
       <c r="D231" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E231" t="s">
         <v>54</v>
@@ -18388,69 +18391,75 @@
         <v>56</v>
       </c>
       <c r="G231">
-        <v>5989</v>
+        <v>11303</v>
       </c>
       <c r="H231">
         <v>0</v>
       </c>
       <c r="I231" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J231" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="N231" s="1">
-        <v>46273</v>
+        <v>46279</v>
       </c>
       <c r="P231">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q231">
         <v>2026</v>
       </c>
       <c r="R231">
-        <v>17941177</v>
+        <v>17399454</v>
       </c>
       <c r="S231" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+      <c r="T231" t="s">
+        <v>163</v>
       </c>
       <c r="U231" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="V231" s="1">
-        <v>46274.41771849537</v>
+        <v>46274.42878043981</v>
       </c>
       <c r="W231">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="X231" t="s">
-        <v>176</v>
+        <v>173</v>
+      </c>
+      <c r="Y231" t="s">
+        <v>249</v>
       </c>
       <c r="AB231">
         <v>0</v>
       </c>
       <c r="AC231" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AH231" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AI231" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="232" spans="1:35">
       <c r="A232">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B232" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C232" t="s">
         <v>50</v>
       </c>
       <c r="D232" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E232" t="s">
         <v>54</v>
@@ -18480,7 +18489,7 @@
         <v>2026</v>
       </c>
       <c r="R232">
-        <v>17952385</v>
+        <v>17941177</v>
       </c>
       <c r="S232" t="s">
         <v>154</v>
@@ -18489,13 +18498,13 @@
         <v>164</v>
       </c>
       <c r="V232" s="1">
-        <v>46274.41775447917</v>
+        <v>46274.41771849537</v>
       </c>
       <c r="W232">
         <v>1</v>
       </c>
       <c r="X232" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="AB232">
         <v>0</v>
@@ -18504,24 +18513,24 @@
         <v>154</v>
       </c>
       <c r="AH232" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI232" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="233" spans="1:35">
       <c r="A233">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B233" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C233" t="s">
         <v>50</v>
       </c>
       <c r="D233" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E233" t="s">
         <v>54</v>
@@ -18551,7 +18560,7 @@
         <v>2026</v>
       </c>
       <c r="R233">
-        <v>17952569</v>
+        <v>17952385</v>
       </c>
       <c r="S233" t="s">
         <v>154</v>
@@ -18560,7 +18569,7 @@
         <v>164</v>
       </c>
       <c r="V233" s="1">
-        <v>46274.41777533565</v>
+        <v>46274.41775447917</v>
       </c>
       <c r="W233">
         <v>1</v>
@@ -18575,18 +18584,18 @@
         <v>154</v>
       </c>
       <c r="AH233" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI233" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="234" spans="1:35">
       <c r="A234">
-        <v>6945</v>
+        <v>6705</v>
       </c>
       <c r="B234" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C234" t="s">
         <v>50</v>
@@ -18598,7 +18607,7 @@
         <v>54</v>
       </c>
       <c r="F234" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G234">
         <v>5989</v>
@@ -18622,7 +18631,7 @@
         <v>2026</v>
       </c>
       <c r="R234">
-        <v>18164516</v>
+        <v>17952569</v>
       </c>
       <c r="S234" t="s">
         <v>154</v>
@@ -18631,13 +18640,13 @@
         <v>164</v>
       </c>
       <c r="V234" s="1">
-        <v>46274.41799166667</v>
+        <v>46274.41777533565</v>
       </c>
       <c r="W234">
         <v>1</v>
       </c>
       <c r="X234" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AB234">
         <v>0</v>
@@ -18646,24 +18655,24 @@
         <v>154</v>
       </c>
       <c r="AH234" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI234" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="235" spans="1:35">
       <c r="A235">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B235" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C235" t="s">
         <v>50</v>
       </c>
       <c r="D235" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E235" t="s">
         <v>54</v>
@@ -18693,7 +18702,7 @@
         <v>2026</v>
       </c>
       <c r="R235">
-        <v>18178157</v>
+        <v>18164516</v>
       </c>
       <c r="S235" t="s">
         <v>154</v>
@@ -18702,13 +18711,13 @@
         <v>164</v>
       </c>
       <c r="V235" s="1">
-        <v>46274.41800114583</v>
+        <v>46274.41799166667</v>
       </c>
       <c r="W235">
         <v>1</v>
       </c>
       <c r="X235" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AB235">
         <v>0</v>
@@ -18717,45 +18726,45 @@
         <v>154</v>
       </c>
       <c r="AH235" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI235" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="236" spans="1:35">
       <c r="A236">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B236" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C236" t="s">
         <v>50</v>
       </c>
       <c r="D236" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E236" t="s">
         <v>54</v>
       </c>
       <c r="F236" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G236">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H236">
         <v>0</v>
       </c>
       <c r="I236" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J236" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N236" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P236">
         <v>9</v>
@@ -18764,48 +18773,48 @@
         <v>2026</v>
       </c>
       <c r="R236">
-        <v>17941187</v>
+        <v>18178157</v>
       </c>
       <c r="S236" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="U236" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="V236" s="1">
-        <v>46274.41772148148</v>
+        <v>46274.41800114583</v>
       </c>
       <c r="W236">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X236" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="AB236">
         <v>0</v>
       </c>
       <c r="AC236" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="AH236" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI236" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="237" spans="1:35">
       <c r="A237">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B237" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C237" t="s">
         <v>50</v>
       </c>
       <c r="D237" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E237" t="s">
         <v>54</v>
@@ -18835,7 +18844,7 @@
         <v>2026</v>
       </c>
       <c r="R237">
-        <v>17952400</v>
+        <v>17941187</v>
       </c>
       <c r="S237" t="s">
         <v>54</v>
@@ -18844,13 +18853,13 @@
         <v>166</v>
       </c>
       <c r="V237" s="1">
-        <v>46274.41773631945</v>
+        <v>46274.41772148148</v>
       </c>
       <c r="W237">
         <v>0</v>
       </c>
       <c r="X237" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="AB237">
         <v>0</v>
@@ -18859,24 +18868,24 @@
         <v>54</v>
       </c>
       <c r="AH237" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI237" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="238" spans="1:35">
       <c r="A238">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B238" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C238" t="s">
         <v>50</v>
       </c>
       <c r="D238" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E238" t="s">
         <v>54</v>
@@ -18906,7 +18915,7 @@
         <v>2026</v>
       </c>
       <c r="R238">
-        <v>17952580</v>
+        <v>17952400</v>
       </c>
       <c r="S238" t="s">
         <v>54</v>
@@ -18915,7 +18924,7 @@
         <v>166</v>
       </c>
       <c r="V238" s="1">
-        <v>46274.41777481481</v>
+        <v>46274.41773631945</v>
       </c>
       <c r="W238">
         <v>0</v>
@@ -18930,18 +18939,18 @@
         <v>54</v>
       </c>
       <c r="AH238" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI238" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="239" spans="1:35">
       <c r="A239">
-        <v>6945</v>
+        <v>6705</v>
       </c>
       <c r="B239" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C239" t="s">
         <v>50</v>
@@ -18953,7 +18962,7 @@
         <v>54</v>
       </c>
       <c r="F239" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G239">
         <v>6215</v>
@@ -18977,7 +18986,7 @@
         <v>2026</v>
       </c>
       <c r="R239">
-        <v>18164523</v>
+        <v>17952580</v>
       </c>
       <c r="S239" t="s">
         <v>54</v>
@@ -18986,13 +18995,13 @@
         <v>166</v>
       </c>
       <c r="V239" s="1">
-        <v>46274.41799332176</v>
+        <v>46274.41777481481</v>
       </c>
       <c r="W239">
         <v>0</v>
       </c>
       <c r="X239" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AB239">
         <v>0</v>
@@ -19001,24 +19010,24 @@
         <v>54</v>
       </c>
       <c r="AH239" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AI239" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="240" spans="1:35">
       <c r="A240">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B240" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C240" t="s">
         <v>50</v>
       </c>
       <c r="D240" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E240" t="s">
         <v>54</v>
@@ -19048,34 +19057,105 @@
         <v>2026</v>
       </c>
       <c r="R240">
-        <v>18178163</v>
+        <v>18164523</v>
       </c>
       <c r="S240" t="s">
-        <v>155</v>
+        <v>54</v>
       </c>
       <c r="U240" t="s">
         <v>166</v>
       </c>
       <c r="V240" s="1">
+        <v>46274.41799332176</v>
+      </c>
+      <c r="W240">
+        <v>0</v>
+      </c>
+      <c r="X240" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB240">
+        <v>0</v>
+      </c>
+      <c r="AC240" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH240" t="s">
+        <v>256</v>
+      </c>
+      <c r="AI240" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="241" spans="1:35">
+      <c r="A241">
+        <v>6949</v>
+      </c>
+      <c r="B241" t="s">
+        <v>37</v>
+      </c>
+      <c r="C241" t="s">
+        <v>50</v>
+      </c>
+      <c r="D241" t="s">
+        <v>51</v>
+      </c>
+      <c r="E241" t="s">
+        <v>54</v>
+      </c>
+      <c r="F241" t="s">
+        <v>57</v>
+      </c>
+      <c r="G241">
+        <v>6215</v>
+      </c>
+      <c r="H241">
+        <v>0</v>
+      </c>
+      <c r="I241" t="s">
+        <v>65</v>
+      </c>
+      <c r="J241" t="s">
+        <v>121</v>
+      </c>
+      <c r="N241" s="1">
+        <v>46274</v>
+      </c>
+      <c r="P241">
+        <v>9</v>
+      </c>
+      <c r="Q241">
+        <v>2026</v>
+      </c>
+      <c r="R241">
+        <v>18178163</v>
+      </c>
+      <c r="S241" t="s">
+        <v>155</v>
+      </c>
+      <c r="U241" t="s">
+        <v>166</v>
+      </c>
+      <c r="V241" s="1">
         <v>46274.41800085648</v>
       </c>
-      <c r="W240">
-        <v>0</v>
-      </c>
-      <c r="X240" t="s">
+      <c r="W241">
+        <v>0</v>
+      </c>
+      <c r="X241" t="s">
         <v>169</v>
       </c>
-      <c r="AB240">
-        <v>0</v>
-      </c>
-      <c r="AC240" t="s">
+      <c r="AB241">
+        <v>0</v>
+      </c>
+      <c r="AC241" t="s">
         <v>155</v>
       </c>
-      <c r="AH240" t="s">
-        <v>255</v>
-      </c>
-      <c r="AI240" t="s">
-        <v>257</v>
+      <c r="AH241" t="s">
+        <v>256</v>
+      </c>
+      <c r="AI241" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-10 11:23
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3721" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3790" uniqueCount="272">
   <si>
     <t>CodCliente</t>
   </si>
@@ -810,6 +810,18 @@
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-09/09/2026 17:52:06.. - Data Comentário: 09/09/2026 17:47</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-09/09/2026 15:33:08.. - Data Comentário: 09/09/2026 15:28</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-08/09/2026 16:18:23.. - Data Comentário: 08/09/2026 16:13</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-09/09/2026 17:27:34.. - Data Comentário: 09/09/2026 17:22</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-09/09/2026 17:53:38.. - Data Comentário: 09/09/2026 17:48</t>
   </si>
   <si>
     <t>Karen Ribeiro</t>
@@ -1172,7 +1184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI261"/>
+  <dimension ref="A1:AI266"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1353,10 +1365,10 @@
         <v>134</v>
       </c>
       <c r="AH2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1430,10 +1442,10 @@
         <v>135</v>
       </c>
       <c r="AH3" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI3" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1507,10 +1519,10 @@
         <v>134</v>
       </c>
       <c r="AH4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1581,10 +1593,10 @@
         <v>134</v>
       </c>
       <c r="AH5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1655,10 +1667,10 @@
         <v>135</v>
       </c>
       <c r="AH6" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1729,10 +1741,10 @@
         <v>135</v>
       </c>
       <c r="AH7" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI7" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1803,10 +1815,10 @@
         <v>136</v>
       </c>
       <c r="AH8" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI8" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1877,10 +1889,10 @@
         <v>134</v>
       </c>
       <c r="AH9" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI9" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1951,10 +1963,10 @@
         <v>137</v>
       </c>
       <c r="AH10" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI10" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -2025,10 +2037,10 @@
         <v>137</v>
       </c>
       <c r="AH11" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI11" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2099,10 +2111,10 @@
         <v>138</v>
       </c>
       <c r="AH12" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI12" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2170,13 +2182,13 @@
         <v>0</v>
       </c>
       <c r="AC13" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="AH13" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI13" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2244,13 +2256,13 @@
         <v>0</v>
       </c>
       <c r="AC14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="AH14" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI14" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2318,10 +2330,10 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI15" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2383,10 +2395,10 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI16" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2454,10 +2466,10 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI17" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2531,10 +2543,10 @@
         <v>140</v>
       </c>
       <c r="AH18" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI18" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2608,10 +2620,10 @@
         <v>139</v>
       </c>
       <c r="AH19" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI19" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2685,10 +2697,10 @@
         <v>140</v>
       </c>
       <c r="AH20" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI20" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2762,10 +2774,10 @@
         <v>138</v>
       </c>
       <c r="AH21" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI21" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2836,10 +2848,10 @@
         <v>141</v>
       </c>
       <c r="AH22" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI22" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2910,10 +2922,10 @@
         <v>138</v>
       </c>
       <c r="AH23" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI23" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2984,10 +2996,10 @@
         <v>138</v>
       </c>
       <c r="AH24" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI24" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3058,10 +3070,10 @@
         <v>138</v>
       </c>
       <c r="AH25" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI25" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3132,10 +3144,10 @@
         <v>139</v>
       </c>
       <c r="AH26" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI26" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3206,10 +3218,10 @@
         <v>138</v>
       </c>
       <c r="AH27" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI27" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3280,10 +3292,10 @@
         <v>138</v>
       </c>
       <c r="AH28" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI28" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3354,10 +3366,10 @@
         <v>138</v>
       </c>
       <c r="AH29" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI29" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3428,10 +3440,10 @@
         <v>142</v>
       </c>
       <c r="AH30" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI30" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3508,10 +3520,10 @@
         <v>143</v>
       </c>
       <c r="AH31" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI31" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3582,10 +3594,10 @@
         <v>144</v>
       </c>
       <c r="AH32" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI32" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3662,10 +3674,10 @@
         <v>145</v>
       </c>
       <c r="AH33" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI33" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3739,10 +3751,10 @@
         <v>146</v>
       </c>
       <c r="AH34" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI34" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3816,13 +3828,13 @@
         <v>0</v>
       </c>
       <c r="AC35" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="AH35" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI35" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3899,10 +3911,10 @@
         <v>148</v>
       </c>
       <c r="AH36" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI36" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3979,10 +3991,10 @@
         <v>142</v>
       </c>
       <c r="AH37" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI37" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4056,10 +4068,10 @@
         <v>164</v>
       </c>
       <c r="AH38" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI38" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4136,10 +4148,10 @@
         <v>143</v>
       </c>
       <c r="AH39" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI39" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4216,10 +4228,10 @@
         <v>143</v>
       </c>
       <c r="AH40" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI40" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4296,10 +4308,10 @@
         <v>143</v>
       </c>
       <c r="AH41" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI41" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4376,10 +4388,10 @@
         <v>142</v>
       </c>
       <c r="AH42" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI42" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4456,10 +4468,10 @@
         <v>149</v>
       </c>
       <c r="AH43" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI43" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4536,10 +4548,10 @@
         <v>144</v>
       </c>
       <c r="AH44" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI44" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4616,10 +4628,10 @@
         <v>145</v>
       </c>
       <c r="AH45" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI45" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4687,10 +4699,10 @@
         <v>146</v>
       </c>
       <c r="AH46" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI46" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4761,10 +4773,10 @@
         <v>143</v>
       </c>
       <c r="AH47" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI47" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4835,10 +4847,10 @@
         <v>143</v>
       </c>
       <c r="AH48" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI48" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4909,10 +4921,10 @@
         <v>143</v>
       </c>
       <c r="AH49" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI49" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4983,10 +4995,10 @@
         <v>142</v>
       </c>
       <c r="AH50" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI50" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5057,10 +5069,10 @@
         <v>149</v>
       </c>
       <c r="AH51" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI51" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5137,10 +5149,10 @@
         <v>144</v>
       </c>
       <c r="AH52" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI52" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5211,10 +5223,10 @@
         <v>145</v>
       </c>
       <c r="AH53" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI53" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5291,10 +5303,10 @@
         <v>143</v>
       </c>
       <c r="AH54" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI54" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5371,10 +5383,10 @@
         <v>143</v>
       </c>
       <c r="AH55" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI55" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5451,10 +5463,10 @@
         <v>143</v>
       </c>
       <c r="AH56" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI56" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5531,10 +5543,10 @@
         <v>142</v>
       </c>
       <c r="AH57" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI57" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5608,10 +5620,10 @@
         <v>146</v>
       </c>
       <c r="AH58" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI58" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5685,13 +5697,13 @@
         <v>0</v>
       </c>
       <c r="AC59" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="AH59" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI59" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5768,10 +5780,10 @@
         <v>143</v>
       </c>
       <c r="AH60" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI60" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5848,10 +5860,10 @@
         <v>143</v>
       </c>
       <c r="AH61" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI61" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5928,10 +5940,10 @@
         <v>143</v>
       </c>
       <c r="AH62" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI62" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -6008,10 +6020,10 @@
         <v>142</v>
       </c>
       <c r="AH63" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI63" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6088,10 +6100,10 @@
         <v>149</v>
       </c>
       <c r="AH64" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI64" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6168,10 +6180,10 @@
         <v>144</v>
       </c>
       <c r="AH65" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI65" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6248,10 +6260,10 @@
         <v>145</v>
       </c>
       <c r="AH66" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI66" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6328,10 +6340,10 @@
         <v>143</v>
       </c>
       <c r="AH67" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI67" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6399,10 +6411,10 @@
         <v>146</v>
       </c>
       <c r="AH68" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI68" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6470,13 +6482,13 @@
         <v>0</v>
       </c>
       <c r="AC69" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="AH69" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI69" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6547,10 +6559,10 @@
         <v>143</v>
       </c>
       <c r="AH70" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI70" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6621,10 +6633,10 @@
         <v>143</v>
       </c>
       <c r="AH71" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI71" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6695,10 +6707,10 @@
         <v>143</v>
       </c>
       <c r="AH72" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI72" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6769,10 +6781,10 @@
         <v>142</v>
       </c>
       <c r="AH73" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI73" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6843,10 +6855,10 @@
         <v>149</v>
       </c>
       <c r="AH74" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI74" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6917,10 +6929,10 @@
         <v>144</v>
       </c>
       <c r="AH75" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI75" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6991,10 +7003,10 @@
         <v>145</v>
       </c>
       <c r="AH76" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI76" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7065,10 +7077,10 @@
         <v>145</v>
       </c>
       <c r="AH77" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI77" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7139,10 +7151,10 @@
         <v>145</v>
       </c>
       <c r="AH78" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI78" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7213,10 +7225,10 @@
         <v>145</v>
       </c>
       <c r="AH79" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI79" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7287,10 +7299,10 @@
         <v>151</v>
       </c>
       <c r="AH80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI80" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7361,10 +7373,10 @@
         <v>151</v>
       </c>
       <c r="AH81" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI81" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7435,10 +7447,10 @@
         <v>152</v>
       </c>
       <c r="AH82" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI82" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7509,10 +7521,10 @@
         <v>151</v>
       </c>
       <c r="AH83" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI83" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7583,10 +7595,10 @@
         <v>151</v>
       </c>
       <c r="AH84" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI84" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7660,10 +7672,10 @@
         <v>151</v>
       </c>
       <c r="AH85" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI85" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7734,10 +7746,10 @@
         <v>152</v>
       </c>
       <c r="AH86" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI86" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7808,10 +7820,10 @@
         <v>151</v>
       </c>
       <c r="AH87" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI87" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7882,10 +7894,10 @@
         <v>151</v>
       </c>
       <c r="AH88" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI88" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7956,10 +7968,10 @@
         <v>151</v>
       </c>
       <c r="AH89" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI89" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -8027,10 +8039,10 @@
         <v>151</v>
       </c>
       <c r="AH90" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI90" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8101,10 +8113,10 @@
         <v>152</v>
       </c>
       <c r="AH91" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI91" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8175,10 +8187,10 @@
         <v>151</v>
       </c>
       <c r="AH92" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI92" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8249,10 +8261,10 @@
         <v>151</v>
       </c>
       <c r="AH93" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI93" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8323,10 +8335,10 @@
         <v>151</v>
       </c>
       <c r="AH94" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI94" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8394,10 +8406,10 @@
         <v>151</v>
       </c>
       <c r="AH95" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI95" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8468,10 +8480,10 @@
         <v>152</v>
       </c>
       <c r="AH96" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI96" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8542,10 +8554,10 @@
         <v>151</v>
       </c>
       <c r="AH97" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI97" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8616,10 +8628,10 @@
         <v>151</v>
       </c>
       <c r="AH98" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI98" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8690,10 +8702,10 @@
         <v>152</v>
       </c>
       <c r="AH99" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI99" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8770,10 +8782,10 @@
         <v>151</v>
       </c>
       <c r="AH100" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI100" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8841,10 +8853,10 @@
         <v>151</v>
       </c>
       <c r="AH101" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI101" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8915,10 +8927,10 @@
         <v>151</v>
       </c>
       <c r="AH102" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI102" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8989,10 +9001,10 @@
         <v>151</v>
       </c>
       <c r="AH103" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI103" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9063,10 +9075,10 @@
         <v>151</v>
       </c>
       <c r="AH104" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI104" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9134,10 +9146,10 @@
         <v>151</v>
       </c>
       <c r="AH105" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI105" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9208,10 +9220,10 @@
         <v>152</v>
       </c>
       <c r="AH106" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI106" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9282,10 +9294,10 @@
         <v>151</v>
       </c>
       <c r="AH107" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI107" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9356,10 +9368,10 @@
         <v>151</v>
       </c>
       <c r="AH108" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI108" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9427,10 +9439,10 @@
         <v>151</v>
       </c>
       <c r="AH109" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI109" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9501,10 +9513,10 @@
         <v>152</v>
       </c>
       <c r="AH110" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI110" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9572,10 +9584,10 @@
         <v>153</v>
       </c>
       <c r="AH111" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI111" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9646,10 +9658,10 @@
         <v>152</v>
       </c>
       <c r="AH112" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI112" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9720,10 +9732,10 @@
         <v>150</v>
       </c>
       <c r="AH113" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI113" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9791,10 +9803,10 @@
         <v>153</v>
       </c>
       <c r="AH114" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI114" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9865,10 +9877,10 @@
         <v>152</v>
       </c>
       <c r="AH115" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI115" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9939,10 +9951,10 @@
         <v>151</v>
       </c>
       <c r="AH116" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI116" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -10013,10 +10025,10 @@
         <v>151</v>
       </c>
       <c r="AH117" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI117" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10087,10 +10099,10 @@
         <v>151</v>
       </c>
       <c r="AH118" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI118" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10158,10 +10170,10 @@
         <v>151</v>
       </c>
       <c r="AH119" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI119" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10232,10 +10244,10 @@
         <v>152</v>
       </c>
       <c r="AH120" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI120" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10306,10 +10318,10 @@
         <v>151</v>
       </c>
       <c r="AH121" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI121" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10380,10 +10392,10 @@
         <v>151</v>
       </c>
       <c r="AH122" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI122" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10454,10 +10466,10 @@
         <v>151</v>
       </c>
       <c r="AH123" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI123" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10525,10 +10537,10 @@
         <v>151</v>
       </c>
       <c r="AH124" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI124" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10599,10 +10611,10 @@
         <v>152</v>
       </c>
       <c r="AH125" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI125" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10679,10 +10691,10 @@
         <v>152</v>
       </c>
       <c r="AH126" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI126" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10759,10 +10771,10 @@
         <v>152</v>
       </c>
       <c r="AH127" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI127" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10833,10 +10845,10 @@
         <v>155</v>
       </c>
       <c r="AH128" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI128" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10907,10 +10919,10 @@
         <v>155</v>
       </c>
       <c r="AH129" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI129" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -10987,10 +10999,10 @@
         <v>155</v>
       </c>
       <c r="AH130" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI130" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11061,10 +11073,10 @@
         <v>155</v>
       </c>
       <c r="AH131" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI131" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11135,10 +11147,10 @@
         <v>155</v>
       </c>
       <c r="AH132" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI132" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11209,10 +11221,10 @@
         <v>155</v>
       </c>
       <c r="AH133" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI133" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11283,10 +11295,10 @@
         <v>155</v>
       </c>
       <c r="AH134" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI134" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11363,10 +11375,10 @@
         <v>155</v>
       </c>
       <c r="AH135" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI135" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11437,10 +11449,10 @@
         <v>155</v>
       </c>
       <c r="AH136" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI136" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11511,10 +11523,10 @@
         <v>155</v>
       </c>
       <c r="AH137" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI137" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11585,10 +11597,10 @@
         <v>155</v>
       </c>
       <c r="AH138" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI138" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11665,10 +11677,10 @@
         <v>155</v>
       </c>
       <c r="AH139" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI139" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11739,10 +11751,10 @@
         <v>155</v>
       </c>
       <c r="AH140" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI140" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11813,10 +11825,10 @@
         <v>155</v>
       </c>
       <c r="AH141" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI141" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11887,10 +11899,10 @@
         <v>155</v>
       </c>
       <c r="AH142" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI142" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11961,10 +11973,10 @@
         <v>155</v>
       </c>
       <c r="AH143" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI143" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -12035,10 +12047,10 @@
         <v>155</v>
       </c>
       <c r="AH144" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI144" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12109,10 +12121,10 @@
         <v>155</v>
       </c>
       <c r="AH145" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI145" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12183,10 +12195,10 @@
         <v>155</v>
       </c>
       <c r="AH146" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI146" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12257,10 +12269,10 @@
         <v>155</v>
       </c>
       <c r="AH147" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI147" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12331,10 +12343,10 @@
         <v>155</v>
       </c>
       <c r="AH148" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI148" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12405,10 +12417,10 @@
         <v>155</v>
       </c>
       <c r="AH149" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI149" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12485,10 +12497,10 @@
         <v>155</v>
       </c>
       <c r="AH150" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI150" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12559,10 +12571,10 @@
         <v>155</v>
       </c>
       <c r="AH151" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI151" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12633,10 +12645,10 @@
         <v>155</v>
       </c>
       <c r="AH152" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI152" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12707,10 +12719,10 @@
         <v>155</v>
       </c>
       <c r="AH153" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI153" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12781,10 +12793,10 @@
         <v>156</v>
       </c>
       <c r="AH154" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI154" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12855,10 +12867,10 @@
         <v>156</v>
       </c>
       <c r="AH155" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI155" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12929,10 +12941,10 @@
         <v>156</v>
       </c>
       <c r="AH156" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI156" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -13003,10 +13015,10 @@
         <v>156</v>
       </c>
       <c r="AH157" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI157" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13077,10 +13089,10 @@
         <v>156</v>
       </c>
       <c r="AH158" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI158" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13151,10 +13163,10 @@
         <v>156</v>
       </c>
       <c r="AH159" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI159" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13225,10 +13237,10 @@
         <v>156</v>
       </c>
       <c r="AH160" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI160" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13299,10 +13311,10 @@
         <v>156</v>
       </c>
       <c r="AH161" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI161" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13373,10 +13385,10 @@
         <v>156</v>
       </c>
       <c r="AH162" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI162" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13447,10 +13459,10 @@
         <v>156</v>
       </c>
       <c r="AH163" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI163" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13521,10 +13533,10 @@
         <v>156</v>
       </c>
       <c r="AH164" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI164" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13595,10 +13607,10 @@
         <v>156</v>
       </c>
       <c r="AH165" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI165" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13669,10 +13681,10 @@
         <v>156</v>
       </c>
       <c r="AH166" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI166" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13743,10 +13755,10 @@
         <v>156</v>
       </c>
       <c r="AH167" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI167" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13817,10 +13829,10 @@
         <v>156</v>
       </c>
       <c r="AH168" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI168" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13891,10 +13903,10 @@
         <v>156</v>
       </c>
       <c r="AH169" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI169" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13965,10 +13977,10 @@
         <v>156</v>
       </c>
       <c r="AH170" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI170" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14039,10 +14051,10 @@
         <v>156</v>
       </c>
       <c r="AH171" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI171" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14113,10 +14125,10 @@
         <v>156</v>
       </c>
       <c r="AH172" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI172" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14190,10 +14202,10 @@
         <v>156</v>
       </c>
       <c r="AH173" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI173" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14267,10 +14279,10 @@
         <v>156</v>
       </c>
       <c r="AH174" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI174" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14344,10 +14356,10 @@
         <v>156</v>
       </c>
       <c r="AH175" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI175" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14421,10 +14433,10 @@
         <v>156</v>
       </c>
       <c r="AH176" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI176" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14498,10 +14510,10 @@
         <v>156</v>
       </c>
       <c r="AH177" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI177" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14575,10 +14587,10 @@
         <v>156</v>
       </c>
       <c r="AH178" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI178" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14652,10 +14664,10 @@
         <v>156</v>
       </c>
       <c r="AH179" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI179" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14729,10 +14741,10 @@
         <v>156</v>
       </c>
       <c r="AH180" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI180" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14806,10 +14818,10 @@
         <v>156</v>
       </c>
       <c r="AH181" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI181" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14883,10 +14895,10 @@
         <v>156</v>
       </c>
       <c r="AH182" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI182" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14960,10 +14972,10 @@
         <v>156</v>
       </c>
       <c r="AH183" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI183" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -15037,10 +15049,10 @@
         <v>156</v>
       </c>
       <c r="AH184" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI184" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15114,10 +15126,10 @@
         <v>156</v>
       </c>
       <c r="AH185" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI185" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15191,10 +15203,10 @@
         <v>156</v>
       </c>
       <c r="AH186" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI186" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15262,10 +15274,10 @@
         <v>156</v>
       </c>
       <c r="AH187" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI187" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15333,10 +15345,10 @@
         <v>156</v>
       </c>
       <c r="AH188" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI188" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15404,10 +15416,10 @@
         <v>156</v>
       </c>
       <c r="AH189" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI189" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15475,10 +15487,10 @@
         <v>156</v>
       </c>
       <c r="AH190" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI190" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15546,10 +15558,10 @@
         <v>156</v>
       </c>
       <c r="AH191" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI191" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15617,10 +15629,10 @@
         <v>156</v>
       </c>
       <c r="AH192" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI192" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15688,10 +15700,10 @@
         <v>54</v>
       </c>
       <c r="AH193" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI193" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15759,10 +15771,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI194" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15830,10 +15842,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI195" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15901,10 +15913,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI196" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15972,10 +15984,10 @@
         <v>157</v>
       </c>
       <c r="AH197" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI197" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -16043,10 +16055,10 @@
         <v>55</v>
       </c>
       <c r="AH198" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI198" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16114,10 +16126,10 @@
         <v>54</v>
       </c>
       <c r="AH199" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI199" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16185,10 +16197,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI200" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16256,10 +16268,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI201" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16327,10 +16339,10 @@
         <v>157</v>
       </c>
       <c r="AH202" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI202" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16398,10 +16410,10 @@
         <v>54</v>
       </c>
       <c r="AH203" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI203" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16469,10 +16481,10 @@
         <v>157</v>
       </c>
       <c r="AH204" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI204" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16540,10 +16552,10 @@
         <v>54</v>
       </c>
       <c r="AH205" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI205" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16611,10 +16623,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI206" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16682,10 +16694,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI207" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16753,10 +16765,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI208" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16824,10 +16836,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI209" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16895,10 +16907,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI210" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -16966,10 +16978,10 @@
         <v>157</v>
       </c>
       <c r="AH211" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI211" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -17037,10 +17049,10 @@
         <v>55</v>
       </c>
       <c r="AH212" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI212" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17111,10 +17123,10 @@
         <v>54</v>
       </c>
       <c r="AH213" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI213" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17185,10 +17197,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI214" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17259,10 +17271,10 @@
         <v>54</v>
       </c>
       <c r="AH215" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI215" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17333,10 +17345,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI216" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17404,10 +17416,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI217" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17475,10 +17487,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI218" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17543,10 +17555,10 @@
         <v>0</v>
       </c>
       <c r="AH219" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI219" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17608,10 +17620,10 @@
         <v>0</v>
       </c>
       <c r="AH220" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI220" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17679,13 +17691,13 @@
         <v>0</v>
       </c>
       <c r="AC221" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="AH221" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI221" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17759,10 +17771,10 @@
         <v>146</v>
       </c>
       <c r="AH222" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI222" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="223" spans="1:35">
@@ -17839,10 +17851,10 @@
         <v>143</v>
       </c>
       <c r="AH223" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI223" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="224" spans="1:35">
@@ -17919,10 +17931,10 @@
         <v>149</v>
       </c>
       <c r="AH224" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI224" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="225" spans="1:35">
@@ -17999,10 +18011,10 @@
         <v>144</v>
       </c>
       <c r="AH225" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI225" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="226" spans="1:35">
@@ -18073,10 +18085,10 @@
         <v>145</v>
       </c>
       <c r="AH226" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI226" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="227" spans="1:35">
@@ -18153,10 +18165,10 @@
         <v>143</v>
       </c>
       <c r="AH227" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI227" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="228" spans="1:35">
@@ -18233,10 +18245,10 @@
         <v>143</v>
       </c>
       <c r="AH228" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI228" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="229" spans="1:35">
@@ -18310,10 +18322,10 @@
         <v>151</v>
       </c>
       <c r="AH229" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI229" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="230" spans="1:35">
@@ -18387,10 +18399,10 @@
         <v>154</v>
       </c>
       <c r="AH230" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI230" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="231" spans="1:35">
@@ -18464,10 +18476,10 @@
         <v>154</v>
       </c>
       <c r="AH231" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI231" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="232" spans="1:35">
@@ -18544,10 +18556,10 @@
         <v>150</v>
       </c>
       <c r="AH232" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI232" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="233" spans="1:35">
@@ -18618,10 +18630,10 @@
         <v>151</v>
       </c>
       <c r="AH233" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI233" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="234" spans="1:35">
@@ -18692,10 +18704,10 @@
         <v>154</v>
       </c>
       <c r="AH234" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI234" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="235" spans="1:35">
@@ -18766,10 +18778,10 @@
         <v>154</v>
       </c>
       <c r="AH235" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI235" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="236" spans="1:35">
@@ -18840,10 +18852,10 @@
         <v>155</v>
       </c>
       <c r="AH236" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI236" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="237" spans="1:35">
@@ -18920,10 +18932,10 @@
         <v>155</v>
       </c>
       <c r="AH237" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI237" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="238" spans="1:35">
@@ -19000,10 +19012,10 @@
         <v>155</v>
       </c>
       <c r="AH238" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI238" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="239" spans="1:35">
@@ -19077,10 +19089,10 @@
         <v>155</v>
       </c>
       <c r="AH239" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI239" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="240" spans="1:35">
@@ -19154,10 +19166,10 @@
         <v>155</v>
       </c>
       <c r="AH240" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI240" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="241" spans="1:35">
@@ -19228,10 +19240,10 @@
         <v>156</v>
       </c>
       <c r="AH241" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI241" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="242" spans="1:35">
@@ -19302,10 +19314,10 @@
         <v>156</v>
       </c>
       <c r="AH242" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI242" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="243" spans="1:35">
@@ -19376,24 +19388,24 @@
         <v>156</v>
       </c>
       <c r="AH243" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AI243" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="244" spans="1:35">
       <c r="A244">
-        <v>6703</v>
+        <v>6548</v>
       </c>
       <c r="B244" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C244" t="s">
         <v>50</v>
       </c>
       <c r="D244" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E244" t="s">
         <v>54</v>
@@ -19402,7 +19414,7 @@
         <v>56</v>
       </c>
       <c r="G244">
-        <v>5989</v>
+        <v>951</v>
       </c>
       <c r="H244">
         <v>0</v>
@@ -19411,34 +19423,37 @@
         <v>64</v>
       </c>
       <c r="J244" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N244" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P244">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q244">
         <v>2026</v>
       </c>
       <c r="R244">
-        <v>17941177</v>
+        <v>17222405</v>
       </c>
       <c r="S244" t="s">
         <v>156</v>
       </c>
       <c r="U244" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V244" s="1">
-        <v>46274.41771849537</v>
+        <v>46275.45011145833</v>
       </c>
       <c r="W244">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X244" t="s">
-        <v>178</v>
+        <v>169</v>
+      </c>
+      <c r="Y244" t="s">
+        <v>259</v>
       </c>
       <c r="AB244">
         <v>0</v>
@@ -19447,33 +19462,33 @@
         <v>156</v>
       </c>
       <c r="AH244" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AI244" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="245" spans="1:35">
       <c r="A245">
-        <v>6704</v>
+        <v>6628</v>
       </c>
       <c r="B245" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C245" t="s">
         <v>50</v>
       </c>
       <c r="D245" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E245" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F245" t="s">
         <v>56</v>
       </c>
       <c r="G245">
-        <v>5989</v>
+        <v>951</v>
       </c>
       <c r="H245">
         <v>0</v>
@@ -19482,34 +19497,34 @@
         <v>64</v>
       </c>
       <c r="J245" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N245" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P245">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q245">
         <v>2026</v>
       </c>
       <c r="R245">
-        <v>17952385</v>
+        <v>16959950</v>
       </c>
       <c r="S245" t="s">
         <v>156</v>
       </c>
       <c r="U245" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V245" s="1">
-        <v>46274.41775447917</v>
+        <v>46275.44901016204</v>
       </c>
       <c r="W245">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X245" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="AB245">
         <v>0</v>
@@ -19518,33 +19533,33 @@
         <v>156</v>
       </c>
       <c r="AH245" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AI245" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="246" spans="1:35">
       <c r="A246">
-        <v>6705</v>
+        <v>6949</v>
       </c>
       <c r="B246" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C246" t="s">
         <v>50</v>
       </c>
       <c r="D246" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E246" t="s">
         <v>54</v>
       </c>
       <c r="F246" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G246">
-        <v>5989</v>
+        <v>951</v>
       </c>
       <c r="H246">
         <v>0</v>
@@ -19553,34 +19568,37 @@
         <v>64</v>
       </c>
       <c r="J246" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N246" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P246">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q246">
         <v>2026</v>
       </c>
       <c r="R246">
-        <v>17952569</v>
+        <v>18178138</v>
       </c>
       <c r="S246" t="s">
         <v>156</v>
       </c>
       <c r="U246" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V246" s="1">
-        <v>46274.41777533565</v>
+        <v>46275.44975668981</v>
       </c>
       <c r="W246">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X246" t="s">
-        <v>174</v>
+        <v>171</v>
+      </c>
+      <c r="Y246" t="s">
+        <v>260</v>
       </c>
       <c r="AB246">
         <v>0</v>
@@ -19589,24 +19607,24 @@
         <v>156</v>
       </c>
       <c r="AH246" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AI246" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="247" spans="1:35">
       <c r="A247">
-        <v>6945</v>
+        <v>6962</v>
       </c>
       <c r="B247" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C247" t="s">
         <v>50</v>
       </c>
       <c r="D247" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E247" t="s">
         <v>54</v>
@@ -19615,7 +19633,7 @@
         <v>57</v>
       </c>
       <c r="G247">
-        <v>5989</v>
+        <v>951</v>
       </c>
       <c r="H247">
         <v>0</v>
@@ -19624,34 +19642,37 @@
         <v>64</v>
       </c>
       <c r="J247" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N247" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P247">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q247">
         <v>2026</v>
       </c>
       <c r="R247">
-        <v>18164516</v>
+        <v>18188724</v>
       </c>
       <c r="S247" t="s">
         <v>156</v>
       </c>
       <c r="U247" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V247" s="1">
-        <v>46274.41799166667</v>
+        <v>46275.44933692129</v>
       </c>
       <c r="W247">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X247" t="s">
-        <v>172</v>
+        <v>173</v>
+      </c>
+      <c r="Y247" t="s">
+        <v>261</v>
       </c>
       <c r="AB247">
         <v>0</v>
@@ -19660,24 +19681,24 @@
         <v>156</v>
       </c>
       <c r="AH247" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AI247" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="248" spans="1:35">
       <c r="A248">
-        <v>6949</v>
+        <v>6963</v>
       </c>
       <c r="B248" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C248" t="s">
         <v>50</v>
       </c>
       <c r="D248" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E248" t="s">
         <v>54</v>
@@ -19686,7 +19707,7 @@
         <v>57</v>
       </c>
       <c r="G248">
-        <v>5989</v>
+        <v>951</v>
       </c>
       <c r="H248">
         <v>0</v>
@@ -19695,34 +19716,37 @@
         <v>64</v>
       </c>
       <c r="J248" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N248" s="1">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P248">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q248">
         <v>2026</v>
       </c>
       <c r="R248">
-        <v>18178157</v>
+        <v>18188630</v>
       </c>
       <c r="S248" t="s">
         <v>156</v>
       </c>
       <c r="U248" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V248" s="1">
-        <v>46274.41800114583</v>
+        <v>46275.44933814815</v>
       </c>
       <c r="W248">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X248" t="s">
-        <v>171</v>
+        <v>173</v>
+      </c>
+      <c r="Y248" t="s">
+        <v>262</v>
       </c>
       <c r="AB248">
         <v>0</v>
@@ -19731,10 +19755,10 @@
         <v>156</v>
       </c>
       <c r="AH248" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AI248" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="249" spans="1:35">
@@ -19757,19 +19781,19 @@
         <v>56</v>
       </c>
       <c r="G249">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H249">
         <v>0</v>
       </c>
       <c r="I249" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J249" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N249" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P249">
         <v>9</v>
@@ -19778,19 +19802,19 @@
         <v>2026</v>
       </c>
       <c r="R249">
-        <v>17941187</v>
+        <v>17941177</v>
       </c>
       <c r="S249" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="U249" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V249" s="1">
-        <v>46274.41772148148</v>
+        <v>46274.41771849537</v>
       </c>
       <c r="W249">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X249" t="s">
         <v>178</v>
@@ -19799,13 +19823,13 @@
         <v>0</v>
       </c>
       <c r="AC249" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="AH249" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI249" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="250" spans="1:35">
@@ -19828,19 +19852,19 @@
         <v>56</v>
       </c>
       <c r="G250">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H250">
         <v>0</v>
       </c>
       <c r="I250" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J250" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N250" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P250">
         <v>9</v>
@@ -19849,19 +19873,19 @@
         <v>2026</v>
       </c>
       <c r="R250">
-        <v>17952400</v>
+        <v>17952385</v>
       </c>
       <c r="S250" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="U250" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V250" s="1">
-        <v>46274.41773631945</v>
+        <v>46274.41775447917</v>
       </c>
       <c r="W250">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X250" t="s">
         <v>174</v>
@@ -19870,13 +19894,13 @@
         <v>0</v>
       </c>
       <c r="AC250" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="AH250" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI250" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="251" spans="1:35">
@@ -19899,19 +19923,19 @@
         <v>56</v>
       </c>
       <c r="G251">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H251">
         <v>0</v>
       </c>
       <c r="I251" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J251" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N251" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P251">
         <v>9</v>
@@ -19920,19 +19944,19 @@
         <v>2026</v>
       </c>
       <c r="R251">
-        <v>17952580</v>
+        <v>17952569</v>
       </c>
       <c r="S251" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="U251" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V251" s="1">
-        <v>46274.41777481481</v>
+        <v>46274.41777533565</v>
       </c>
       <c r="W251">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X251" t="s">
         <v>174</v>
@@ -19941,13 +19965,13 @@
         <v>0</v>
       </c>
       <c r="AC251" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="AH251" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI251" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="252" spans="1:35">
@@ -19970,19 +19994,19 @@
         <v>57</v>
       </c>
       <c r="G252">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H252">
         <v>0</v>
       </c>
       <c r="I252" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J252" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N252" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P252">
         <v>9</v>
@@ -19991,19 +20015,19 @@
         <v>2026</v>
       </c>
       <c r="R252">
-        <v>18164523</v>
+        <v>18164516</v>
       </c>
       <c r="S252" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="U252" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V252" s="1">
-        <v>46274.41799332176</v>
+        <v>46274.41799166667</v>
       </c>
       <c r="W252">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X252" t="s">
         <v>172</v>
@@ -20012,13 +20036,13 @@
         <v>0</v>
       </c>
       <c r="AC252" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
       <c r="AH252" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI252" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="253" spans="1:35">
@@ -20041,19 +20065,19 @@
         <v>57</v>
       </c>
       <c r="G253">
-        <v>6215</v>
+        <v>5989</v>
       </c>
       <c r="H253">
         <v>0</v>
       </c>
       <c r="I253" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J253" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N253" s="1">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="P253">
         <v>9</v>
@@ -20062,19 +20086,19 @@
         <v>2026</v>
       </c>
       <c r="R253">
-        <v>18178163</v>
+        <v>18178157</v>
       </c>
       <c r="S253" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="U253" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V253" s="1">
-        <v>46274.41800085648</v>
+        <v>46274.41800114583</v>
       </c>
       <c r="W253">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X253" t="s">
         <v>171</v>
@@ -20083,27 +20107,27 @@
         <v>0</v>
       </c>
       <c r="AC253" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AH253" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="AI253" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="254" spans="1:35">
       <c r="A254">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B254" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C254" t="s">
         <v>50</v>
       </c>
       <c r="D254" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E254" t="s">
         <v>54</v>
@@ -20112,7 +20136,7 @@
         <v>56</v>
       </c>
       <c r="G254">
-        <v>11746</v>
+        <v>6215</v>
       </c>
       <c r="H254">
         <v>0</v>
@@ -20121,19 +20145,19 @@
         <v>65</v>
       </c>
       <c r="J254" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="N254" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P254">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q254">
         <v>2026</v>
       </c>
       <c r="R254">
-        <v>17994311</v>
+        <v>17941187</v>
       </c>
       <c r="S254" t="s">
         <v>54</v>
@@ -20142,39 +20166,39 @@
         <v>168</v>
       </c>
       <c r="V254" s="1">
-        <v>46275.31737530093</v>
+        <v>46274.41772148148</v>
       </c>
       <c r="W254">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X254" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AB254">
         <v>0</v>
       </c>
       <c r="AC254" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="AH254" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AI254" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="255" spans="1:35">
       <c r="A255">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B255" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C255" t="s">
         <v>50</v>
       </c>
       <c r="D255" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E255" t="s">
         <v>54</v>
@@ -20183,7 +20207,7 @@
         <v>56</v>
       </c>
       <c r="G255">
-        <v>11746</v>
+        <v>6215</v>
       </c>
       <c r="H255">
         <v>0</v>
@@ -20192,19 +20216,19 @@
         <v>65</v>
       </c>
       <c r="J255" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="N255" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P255">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q255">
         <v>2026</v>
       </c>
       <c r="R255">
-        <v>17994675</v>
+        <v>17952400</v>
       </c>
       <c r="S255" t="s">
         <v>54</v>
@@ -20213,39 +20237,39 @@
         <v>168</v>
       </c>
       <c r="V255" s="1">
-        <v>46275.31747032407</v>
+        <v>46274.41773631945</v>
       </c>
       <c r="W255">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X255" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="AB255">
         <v>0</v>
       </c>
       <c r="AC255" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="AH255" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AI255" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="256" spans="1:35">
       <c r="A256">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B256" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C256" t="s">
         <v>50</v>
       </c>
       <c r="D256" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E256" t="s">
         <v>54</v>
@@ -20254,7 +20278,7 @@
         <v>56</v>
       </c>
       <c r="G256">
-        <v>11746</v>
+        <v>6215</v>
       </c>
       <c r="H256">
         <v>0</v>
@@ -20263,19 +20287,19 @@
         <v>65</v>
       </c>
       <c r="J256" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="N256" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P256">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q256">
         <v>2026</v>
       </c>
       <c r="R256">
-        <v>17994809</v>
+        <v>17952580</v>
       </c>
       <c r="S256" t="s">
         <v>54</v>
@@ -20284,48 +20308,48 @@
         <v>168</v>
       </c>
       <c r="V256" s="1">
-        <v>46275.31747981482</v>
+        <v>46274.41777481481</v>
       </c>
       <c r="W256">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X256" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="AB256">
         <v>0</v>
       </c>
       <c r="AC256" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="AH256" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AI256" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="257" spans="1:35">
       <c r="A257">
-        <v>6548</v>
+        <v>6945</v>
       </c>
       <c r="B257" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C257" t="s">
         <v>50</v>
       </c>
       <c r="D257" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E257" t="s">
         <v>54</v>
       </c>
       <c r="F257" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G257">
-        <v>11746</v>
+        <v>6215</v>
       </c>
       <c r="H257">
         <v>0</v>
@@ -20334,19 +20358,19 @@
         <v>65</v>
       </c>
       <c r="J257" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="N257" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P257">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q257">
         <v>2026</v>
       </c>
       <c r="R257">
-        <v>18006051</v>
+        <v>18164523</v>
       </c>
       <c r="S257" t="s">
         <v>54</v>
@@ -20355,48 +20379,48 @@
         <v>168</v>
       </c>
       <c r="V257" s="1">
-        <v>46275.31748724537</v>
+        <v>46274.41799332176</v>
       </c>
       <c r="W257">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X257" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB257">
         <v>0</v>
       </c>
       <c r="AC257" t="s">
-        <v>157</v>
+        <v>54</v>
       </c>
       <c r="AH257" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AI257" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="258" spans="1:35">
       <c r="A258">
-        <v>6628</v>
+        <v>6949</v>
       </c>
       <c r="B258" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C258" t="s">
         <v>50</v>
       </c>
       <c r="D258" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E258" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F258" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G258">
-        <v>11746</v>
+        <v>6215</v>
       </c>
       <c r="H258">
         <v>0</v>
@@ -20405,34 +20429,34 @@
         <v>65</v>
       </c>
       <c r="J258" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="N258" s="1">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="P258">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q258">
         <v>2026</v>
       </c>
       <c r="R258">
-        <v>18003256</v>
+        <v>18178163</v>
       </c>
       <c r="S258" t="s">
-        <v>55</v>
+        <v>157</v>
       </c>
       <c r="U258" t="s">
         <v>168</v>
       </c>
       <c r="V258" s="1">
-        <v>46275.31749535879</v>
+        <v>46274.41800085648</v>
       </c>
       <c r="W258">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X258" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AB258">
         <v>0</v>
@@ -20441,24 +20465,24 @@
         <v>157</v>
       </c>
       <c r="AH258" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AI258" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="259" spans="1:35">
       <c r="A259">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B259" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C259" t="s">
         <v>50</v>
       </c>
       <c r="D259" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E259" t="s">
         <v>54</v>
@@ -20488,7 +20512,7 @@
         <v>2026</v>
       </c>
       <c r="R259">
-        <v>18004017</v>
+        <v>17994311</v>
       </c>
       <c r="S259" t="s">
         <v>54</v>
@@ -20497,13 +20521,13 @@
         <v>168</v>
       </c>
       <c r="V259" s="1">
-        <v>46275.31750491898</v>
+        <v>46275.31737530093</v>
       </c>
       <c r="W259">
         <v>0</v>
       </c>
       <c r="X259" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="AB259">
         <v>0</v>
@@ -20512,24 +20536,24 @@
         <v>157</v>
       </c>
       <c r="AH259" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI259" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="260" spans="1:35">
       <c r="A260">
-        <v>6704</v>
+        <v>6404</v>
       </c>
       <c r="B260" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C260" t="s">
         <v>50</v>
       </c>
       <c r="D260" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E260" t="s">
         <v>54</v>
@@ -20559,7 +20583,7 @@
         <v>2026</v>
       </c>
       <c r="R260">
-        <v>17995164</v>
+        <v>17994675</v>
       </c>
       <c r="S260" t="s">
         <v>54</v>
@@ -20568,13 +20592,13 @@
         <v>168</v>
       </c>
       <c r="V260" s="1">
-        <v>46275.31750555555</v>
+        <v>46275.31747032407</v>
       </c>
       <c r="W260">
         <v>0</v>
       </c>
       <c r="X260" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="AB260">
         <v>0</v>
@@ -20583,24 +20607,24 @@
         <v>157</v>
       </c>
       <c r="AH260" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI260" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="261" spans="1:35">
       <c r="A261">
-        <v>6705</v>
+        <v>6486</v>
       </c>
       <c r="B261" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C261" t="s">
         <v>50</v>
       </c>
       <c r="D261" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E261" t="s">
         <v>54</v>
@@ -20630,7 +20654,7 @@
         <v>2026</v>
       </c>
       <c r="R261">
-        <v>18004028</v>
+        <v>17994809</v>
       </c>
       <c r="S261" t="s">
         <v>54</v>
@@ -20639,13 +20663,13 @@
         <v>168</v>
       </c>
       <c r="V261" s="1">
-        <v>46275.31750599537</v>
+        <v>46275.31747981482</v>
       </c>
       <c r="W261">
         <v>0</v>
       </c>
       <c r="X261" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AB261">
         <v>0</v>
@@ -20654,10 +20678,365 @@
         <v>157</v>
       </c>
       <c r="AH261" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AI261" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="262" spans="1:35">
+      <c r="A262">
+        <v>6548</v>
+      </c>
+      <c r="B262" t="s">
+        <v>35</v>
+      </c>
+      <c r="C262" t="s">
+        <v>50</v>
+      </c>
+      <c r="D262" t="s">
+        <v>51</v>
+      </c>
+      <c r="E262" t="s">
+        <v>54</v>
+      </c>
+      <c r="F262" t="s">
+        <v>56</v>
+      </c>
+      <c r="G262">
+        <v>11746</v>
+      </c>
+      <c r="H262">
+        <v>0</v>
+      </c>
+      <c r="I262" t="s">
+        <v>65</v>
+      </c>
+      <c r="J262" t="s">
+        <v>126</v>
+      </c>
+      <c r="N262" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P262">
+        <v>8</v>
+      </c>
+      <c r="Q262">
+        <v>2026</v>
+      </c>
+      <c r="R262">
+        <v>18006051</v>
+      </c>
+      <c r="S262" t="s">
+        <v>54</v>
+      </c>
+      <c r="U262" t="s">
+        <v>168</v>
+      </c>
+      <c r="V262" s="1">
+        <v>46275.31748724537</v>
+      </c>
+      <c r="W262">
+        <v>0</v>
+      </c>
+      <c r="X262" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB262">
+        <v>0</v>
+      </c>
+      <c r="AC262" t="s">
+        <v>157</v>
+      </c>
+      <c r="AH262" t="s">
         <v>267</v>
+      </c>
+      <c r="AI262" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="263" spans="1:35">
+      <c r="A263">
+        <v>6628</v>
+      </c>
+      <c r="B263" t="s">
+        <v>38</v>
+      </c>
+      <c r="C263" t="s">
+        <v>50</v>
+      </c>
+      <c r="D263" t="s">
+        <v>52</v>
+      </c>
+      <c r="E263" t="s">
+        <v>55</v>
+      </c>
+      <c r="F263" t="s">
+        <v>56</v>
+      </c>
+      <c r="G263">
+        <v>11746</v>
+      </c>
+      <c r="H263">
+        <v>0</v>
+      </c>
+      <c r="I263" t="s">
+        <v>65</v>
+      </c>
+      <c r="J263" t="s">
+        <v>126</v>
+      </c>
+      <c r="N263" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P263">
+        <v>8</v>
+      </c>
+      <c r="Q263">
+        <v>2026</v>
+      </c>
+      <c r="R263">
+        <v>18003256</v>
+      </c>
+      <c r="S263" t="s">
+        <v>55</v>
+      </c>
+      <c r="U263" t="s">
+        <v>168</v>
+      </c>
+      <c r="V263" s="1">
+        <v>46275.31749535879</v>
+      </c>
+      <c r="W263">
+        <v>0</v>
+      </c>
+      <c r="X263" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB263">
+        <v>0</v>
+      </c>
+      <c r="AC263" t="s">
+        <v>157</v>
+      </c>
+      <c r="AH263" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI263" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="264" spans="1:35">
+      <c r="A264">
+        <v>6703</v>
+      </c>
+      <c r="B264" t="s">
+        <v>46</v>
+      </c>
+      <c r="C264" t="s">
+        <v>50</v>
+      </c>
+      <c r="D264" t="s">
+        <v>53</v>
+      </c>
+      <c r="E264" t="s">
+        <v>54</v>
+      </c>
+      <c r="F264" t="s">
+        <v>56</v>
+      </c>
+      <c r="G264">
+        <v>11746</v>
+      </c>
+      <c r="H264">
+        <v>0</v>
+      </c>
+      <c r="I264" t="s">
+        <v>65</v>
+      </c>
+      <c r="J264" t="s">
+        <v>126</v>
+      </c>
+      <c r="N264" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P264">
+        <v>8</v>
+      </c>
+      <c r="Q264">
+        <v>2026</v>
+      </c>
+      <c r="R264">
+        <v>18004017</v>
+      </c>
+      <c r="S264" t="s">
+        <v>54</v>
+      </c>
+      <c r="U264" t="s">
+        <v>168</v>
+      </c>
+      <c r="V264" s="1">
+        <v>46275.31750491898</v>
+      </c>
+      <c r="W264">
+        <v>0</v>
+      </c>
+      <c r="X264" t="s">
+        <v>178</v>
+      </c>
+      <c r="AB264">
+        <v>0</v>
+      </c>
+      <c r="AC264" t="s">
+        <v>157</v>
+      </c>
+      <c r="AH264" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI264" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="265" spans="1:35">
+      <c r="A265">
+        <v>6704</v>
+      </c>
+      <c r="B265" t="s">
+        <v>42</v>
+      </c>
+      <c r="C265" t="s">
+        <v>50</v>
+      </c>
+      <c r="D265" t="s">
+        <v>51</v>
+      </c>
+      <c r="E265" t="s">
+        <v>54</v>
+      </c>
+      <c r="F265" t="s">
+        <v>56</v>
+      </c>
+      <c r="G265">
+        <v>11746</v>
+      </c>
+      <c r="H265">
+        <v>0</v>
+      </c>
+      <c r="I265" t="s">
+        <v>65</v>
+      </c>
+      <c r="J265" t="s">
+        <v>126</v>
+      </c>
+      <c r="N265" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P265">
+        <v>8</v>
+      </c>
+      <c r="Q265">
+        <v>2026</v>
+      </c>
+      <c r="R265">
+        <v>17995164</v>
+      </c>
+      <c r="S265" t="s">
+        <v>54</v>
+      </c>
+      <c r="U265" t="s">
+        <v>168</v>
+      </c>
+      <c r="V265" s="1">
+        <v>46275.31750555555</v>
+      </c>
+      <c r="W265">
+        <v>0</v>
+      </c>
+      <c r="X265" t="s">
+        <v>174</v>
+      </c>
+      <c r="AB265">
+        <v>0</v>
+      </c>
+      <c r="AC265" t="s">
+        <v>157</v>
+      </c>
+      <c r="AH265" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI265" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="266" spans="1:35">
+      <c r="A266">
+        <v>6705</v>
+      </c>
+      <c r="B266" t="s">
+        <v>48</v>
+      </c>
+      <c r="C266" t="s">
+        <v>50</v>
+      </c>
+      <c r="D266" t="s">
+        <v>52</v>
+      </c>
+      <c r="E266" t="s">
+        <v>54</v>
+      </c>
+      <c r="F266" t="s">
+        <v>56</v>
+      </c>
+      <c r="G266">
+        <v>11746</v>
+      </c>
+      <c r="H266">
+        <v>0</v>
+      </c>
+      <c r="I266" t="s">
+        <v>65</v>
+      </c>
+      <c r="J266" t="s">
+        <v>126</v>
+      </c>
+      <c r="N266" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P266">
+        <v>8</v>
+      </c>
+      <c r="Q266">
+        <v>2026</v>
+      </c>
+      <c r="R266">
+        <v>18004028</v>
+      </c>
+      <c r="S266" t="s">
+        <v>54</v>
+      </c>
+      <c r="U266" t="s">
+        <v>168</v>
+      </c>
+      <c r="V266" s="1">
+        <v>46275.31750599537</v>
+      </c>
+      <c r="W266">
+        <v>0</v>
+      </c>
+      <c r="X266" t="s">
+        <v>174</v>
+      </c>
+      <c r="AB266">
+        <v>0</v>
+      </c>
+      <c r="AC266" t="s">
+        <v>157</v>
+      </c>
+      <c r="AH266" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI266" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>